<commit_message>
test: fixed test config
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_access/test_casedb_case_access.xlsx
+++ b/test/casedb/integration/case_access/test_casedb_case_access.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_access\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEB63340-ABA8-4F02-AA39-53A97332F0B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9036432-E00B-4718-AC78-4145C9D0306C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="913" firstSheet="2" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="4" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Organization" sheetId="17" r:id="rId1"/>
@@ -1412,9 +1412,6 @@
     <t>roles</t>
   </si>
   <si>
-    <t>018bcd02-eb19-fb14-c520-64cbb78d9135</t>
-  </si>
-  <si>
     <t>root1_1@org1.org</t>
   </si>
   <si>
@@ -2256,6 +2253,9 @@
   </si>
   <si>
     <t>dm.is_active</t>
+  </si>
+  <si>
+    <t>019542cc-8225-8f5d-fa30-d9c3f2629703</t>
   </si>
 </sst>
 </file>
@@ -2776,13 +2776,13 @@
         <v>57</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>485</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>486</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -2790,10 +2790,10 @@
         <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C2" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -2801,10 +2801,10 @@
         <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -2812,10 +2812,10 @@
         <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C4" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -2823,10 +2823,10 @@
         <v>52</v>
       </c>
       <c r="B5" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C5" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -2834,10 +2834,10 @@
         <v>55</v>
       </c>
       <c r="B6" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C6" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
   </sheetData>
@@ -2921,7 +2921,7 @@
         <v>83</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>84</v>
@@ -3228,7 +3228,7 @@
         <v>58</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>59</v>
@@ -3237,13 +3237,13 @@
         <v>316</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>317</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -5165,7 +5165,7 @@
         <v>60</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>61</v>
@@ -5174,13 +5174,13 @@
         <v>139</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>140</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -6244,13 +6244,13 @@
         <v>41</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>3</v>
@@ -6427,145 +6427,145 @@
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>588</v>
+      </c>
+      <c r="B1" t="s">
+        <v>723</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>591</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>718</v>
+      </c>
+      <c r="F1" t="s">
         <v>589</v>
       </c>
-      <c r="B1" t="s">
-        <v>724</v>
-      </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="G1" s="19" t="s">
+        <v>599</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>675</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>676</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="R1" t="s">
+        <v>590</v>
+      </c>
+      <c r="S1" t="s">
         <v>592</v>
       </c>
-      <c r="E1" s="6" t="s">
-        <v>719</v>
-      </c>
-      <c r="F1" t="s">
-        <v>590</v>
-      </c>
-      <c r="G1" s="19" t="s">
-        <v>600</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>667</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>671</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>668</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>676</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="M1" s="6" t="s">
-        <v>602</v>
-      </c>
-      <c r="N1" s="6" t="s">
-        <v>670</v>
-      </c>
-      <c r="O1" s="6" t="s">
+      <c r="T1" s="6" t="s">
+        <v>660</v>
+      </c>
+      <c r="U1" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="V1" t="s">
+        <v>593</v>
+      </c>
+      <c r="W1" t="s">
+        <v>594</v>
+      </c>
+      <c r="X1" s="6" t="s">
+        <v>678</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>595</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>596</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>597</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>598</v>
+      </c>
+      <c r="AC1" s="6" t="s">
         <v>677</v>
       </c>
-      <c r="P1" s="6" t="s">
-        <v>603</v>
-      </c>
-      <c r="Q1" s="6" t="s">
-        <v>604</v>
-      </c>
-      <c r="R1" t="s">
-        <v>591</v>
-      </c>
-      <c r="S1" t="s">
-        <v>593</v>
-      </c>
-      <c r="T1" s="6" t="s">
-        <v>661</v>
-      </c>
-      <c r="U1" s="6" t="s">
-        <v>666</v>
-      </c>
-      <c r="V1" t="s">
-        <v>594</v>
-      </c>
-      <c r="W1" t="s">
-        <v>595</v>
-      </c>
-      <c r="X1" s="6" t="s">
+      <c r="AD1" s="6" t="s">
+        <v>681</v>
+      </c>
+      <c r="AE1" s="6" t="s">
+        <v>682</v>
+      </c>
+      <c r="AF1" s="6" t="s">
+        <v>687</v>
+      </c>
+      <c r="AG1" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>662</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>708</v>
+      </c>
+      <c r="AJ1" s="6" t="s">
         <v>679</v>
       </c>
-      <c r="Y1" t="s">
-        <v>596</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>597</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>598</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>599</v>
-      </c>
-      <c r="AC1" s="6" t="s">
-        <v>678</v>
-      </c>
-      <c r="AD1" s="6" t="s">
-        <v>682</v>
-      </c>
-      <c r="AE1" s="6" t="s">
+      <c r="AK1" s="6" t="s">
         <v>683</v>
       </c>
-      <c r="AF1" s="6" t="s">
-        <v>688</v>
-      </c>
-      <c r="AG1" s="6" t="s">
+      <c r="AL1" s="6" t="s">
+        <v>684</v>
+      </c>
+      <c r="AM1" s="6" t="s">
         <v>689</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AN1" s="6" t="s">
+        <v>690</v>
+      </c>
+      <c r="AO1" t="s">
         <v>663</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AP1" t="s">
         <v>709</v>
       </c>
-      <c r="AJ1" s="6" t="s">
+      <c r="AQ1" s="6" t="s">
         <v>680</v>
       </c>
-      <c r="AK1" s="6" t="s">
-        <v>684</v>
-      </c>
-      <c r="AL1" s="6" t="s">
+      <c r="AR1" s="6" t="s">
         <v>685</v>
       </c>
-      <c r="AM1" s="6" t="s">
-        <v>690</v>
-      </c>
-      <c r="AN1" s="6" t="s">
+      <c r="AS1" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="AT1" s="6" t="s">
         <v>691</v>
       </c>
-      <c r="AO1" t="s">
-        <v>664</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>710</v>
-      </c>
-      <c r="AQ1" s="6" t="s">
-        <v>681</v>
-      </c>
-      <c r="AR1" s="6" t="s">
-        <v>686</v>
-      </c>
-      <c r="AS1" s="6" t="s">
-        <v>687</v>
-      </c>
-      <c r="AT1" s="6" t="s">
+      <c r="AU1" s="6" t="s">
         <v>692</v>
-      </c>
-      <c r="AU1" s="6" t="s">
-        <v>693</v>
       </c>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.3">
@@ -6576,17 +6576,17 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D2" t="s">
-        <v>443</v>
+        <v>724</v>
       </c>
       <c r="E2" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($D2,User!$A:$A,0))</f>
         <v>root1_1</v>
       </c>
       <c r="F2" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="G2" s="19" t="b">
         <f t="shared" ref="G2:G33" si="0">IF($F2="CREATE",$I2,IF($F2="CREATE_CASES",OR($I2,AND($K2,$L2,$O2,$P2,$AE2,AG2,$AL2,$AN2,$AS2,$AU2)),"TBD"))</f>
@@ -6633,7 +6633,7 @@
         <v>0</v>
       </c>
       <c r="R2" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="S2" t="s">
         <v>119</v>
@@ -6660,7 +6660,7 @@
         <v>142</v>
       </c>
       <c r="AB2" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC2" s="6" t="str">
         <f>IF($AA2="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA2,CaseTypeCol!$A:$A,0)))</f>
@@ -6731,17 +6731,17 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="E3" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($D3,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
       <c r="F3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="G3" s="19" t="b">
         <f t="shared" si="0"/>
@@ -6788,7 +6788,7 @@
         <v>0</v>
       </c>
       <c r="R3" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="S3" t="s">
         <v>119</v>
@@ -6815,7 +6815,7 @@
         <v>142</v>
       </c>
       <c r="AB3" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC3" s="6" t="str">
         <f>IF($AA3="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA3,CaseTypeCol!$A:$A,0)))</f>
@@ -6886,17 +6886,17 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E4" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($D4,User!$A:$A,0))</f>
         <v>refdata_admin1_1</v>
       </c>
       <c r="F4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="G4" s="19" t="b">
         <f t="shared" si="0"/>
@@ -6943,7 +6943,7 @@
         <v>0</v>
       </c>
       <c r="R4" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="S4" t="s">
         <v>119</v>
@@ -6970,7 +6970,7 @@
         <v>142</v>
       </c>
       <c r="AB4" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC4" s="6" t="str">
         <f>IF($AA4="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA4,CaseTypeCol!$A:$A,0)))</f>
@@ -7041,7 +7041,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D5" t="s">
         <v>44</v>
@@ -7051,7 +7051,7 @@
         <v>org_admin1_1</v>
       </c>
       <c r="F5" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="G5" s="19" t="b">
         <f t="shared" si="0"/>
@@ -7098,7 +7098,7 @@
         <v>0</v>
       </c>
       <c r="R5" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="S5" t="s">
         <v>119</v>
@@ -7125,7 +7125,7 @@
         <v>142</v>
       </c>
       <c r="AB5" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC5" s="6" t="str">
         <f>IF($AA5="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA5,CaseTypeCol!$A:$A,0)))</f>
@@ -7196,7 +7196,7 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="D6" t="s">
         <v>10</v>
@@ -7206,7 +7206,7 @@
         <v>org_user1_1</v>
       </c>
       <c r="F6" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="G6" s="19" t="b">
         <f t="shared" si="0"/>
@@ -7253,7 +7253,7 @@
         <v>1</v>
       </c>
       <c r="R6" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="S6" t="s">
         <v>119</v>
@@ -7280,7 +7280,7 @@
         <v>142</v>
       </c>
       <c r="AB6" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC6" s="6" t="str">
         <f>IF($AA6="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA6,CaseTypeCol!$A:$A,0)))</f>
@@ -7351,17 +7351,17 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="D7" t="s">
-        <v>443</v>
+        <v>724</v>
       </c>
       <c r="E7" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($D7,User!$A:$A,0))</f>
         <v>root1_1</v>
       </c>
       <c r="F7" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G7" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -7408,7 +7408,7 @@
         <v>0</v>
       </c>
       <c r="R7" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="S7" t="s">
         <v>119</v>
@@ -7435,7 +7435,7 @@
         <v>142</v>
       </c>
       <c r="AB7" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC7" s="6" t="str">
         <f>IF($AA7="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA7,CaseTypeCol!$A:$A,0)))</f>
@@ -7506,17 +7506,17 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="D8" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="E8" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($D8,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
       <c r="F8" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G8" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -7563,7 +7563,7 @@
         <v>0</v>
       </c>
       <c r="R8" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="S8" t="s">
         <v>119</v>
@@ -7590,7 +7590,7 @@
         <v>142</v>
       </c>
       <c r="AB8" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC8" s="6" t="str">
         <f>IF($AA8="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA8,CaseTypeCol!$A:$A,0)))</f>
@@ -7661,7 +7661,7 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D9" t="s">
         <v>44</v>
@@ -7671,7 +7671,7 @@
         <v>org_admin1_1</v>
       </c>
       <c r="F9" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G9" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -7718,7 +7718,7 @@
         <v>0</v>
       </c>
       <c r="R9" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="S9" t="s">
         <v>119</v>
@@ -7745,7 +7745,7 @@
         <v>142</v>
       </c>
       <c r="AB9" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC9" s="6" t="str">
         <f>IF($AA9="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA9,CaseTypeCol!$A:$A,0)))</f>
@@ -7816,7 +7816,7 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D10" t="s">
         <v>47</v>
@@ -7826,7 +7826,7 @@
         <v>org_admin2_1</v>
       </c>
       <c r="F10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G10" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -7873,7 +7873,7 @@
         <v>0</v>
       </c>
       <c r="R10" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="S10" t="s">
         <v>119</v>
@@ -7900,7 +7900,7 @@
         <v>142</v>
       </c>
       <c r="AB10" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC10" s="6" t="str">
         <f>IF($AA10="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA10,CaseTypeCol!$A:$A,0)))</f>
@@ -7971,7 +7971,7 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D11" t="s">
         <v>50</v>
@@ -7981,7 +7981,7 @@
         <v>org_admin3_1</v>
       </c>
       <c r="F11" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G11" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8028,7 +8028,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="S11" t="s">
         <v>119</v>
@@ -8055,7 +8055,7 @@
         <v>142</v>
       </c>
       <c r="AB11" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC11" s="6" t="str">
         <f>IF($AA11="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA11,CaseTypeCol!$A:$A,0)))</f>
@@ -8126,7 +8126,7 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D12" t="s">
         <v>53</v>
@@ -8136,7 +8136,7 @@
         <v>org_admin4_1</v>
       </c>
       <c r="F12" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G12" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8183,7 +8183,7 @@
         <v>0</v>
       </c>
       <c r="R12" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="S12" t="s">
         <v>119</v>
@@ -8210,7 +8210,7 @@
         <v>142</v>
       </c>
       <c r="AB12" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC12" s="6" t="str">
         <f>IF($AA12="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA12,CaseTypeCol!$A:$A,0)))</f>
@@ -8281,7 +8281,7 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D13" t="s">
         <v>56</v>
@@ -8291,7 +8291,7 @@
         <v>org_admin5_1</v>
       </c>
       <c r="F13" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G13" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8338,7 +8338,7 @@
         <v>0</v>
       </c>
       <c r="R13" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="S13" t="s">
         <v>119</v>
@@ -8365,7 +8365,7 @@
         <v>142</v>
       </c>
       <c r="AB13" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC13" s="6" t="str">
         <f>IF($AA13="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA13,CaseTypeCol!$A:$A,0)))</f>
@@ -8436,7 +8436,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D14" t="s">
         <v>10</v>
@@ -8446,7 +8446,7 @@
         <v>org_user1_1</v>
       </c>
       <c r="F14" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G14" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8493,7 +8493,7 @@
         <v>1</v>
       </c>
       <c r="R14" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="S14" t="s">
         <v>119</v>
@@ -8520,7 +8520,7 @@
         <v>142</v>
       </c>
       <c r="AB14" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC14" s="6" t="str">
         <f>IF($AA14="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA14,CaseTypeCol!$A:$A,0)))</f>
@@ -8591,7 +8591,7 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
@@ -8601,7 +8601,7 @@
         <v>org_user1_2</v>
       </c>
       <c r="F15" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G15" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8648,7 +8648,7 @@
         <v>0</v>
       </c>
       <c r="R15" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="S15" t="s">
         <v>119</v>
@@ -8675,7 +8675,7 @@
         <v>142</v>
       </c>
       <c r="AB15" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC15" s="6" t="str">
         <f>IF($AA15="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA15,CaseTypeCol!$A:$A,0)))</f>
@@ -8746,7 +8746,7 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D16" t="s">
         <v>13</v>
@@ -8756,7 +8756,7 @@
         <v>org_user1_3</v>
       </c>
       <c r="F16" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G16" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8803,7 +8803,7 @@
         <v>0</v>
       </c>
       <c r="R16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="S16" t="s">
         <v>119</v>
@@ -8830,7 +8830,7 @@
         <v>142</v>
       </c>
       <c r="AB16" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC16" s="6" t="str">
         <f>IF($AA16="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA16,CaseTypeCol!$A:$A,0)))</f>
@@ -8901,7 +8901,7 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D17" t="s">
         <v>14</v>
@@ -8911,7 +8911,7 @@
         <v>org_user1_4</v>
       </c>
       <c r="F17" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G17" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8958,7 +8958,7 @@
         <v>0</v>
       </c>
       <c r="R17" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="S17" t="s">
         <v>119</v>
@@ -8985,7 +8985,7 @@
         <v>142</v>
       </c>
       <c r="AB17" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC17" s="6" t="str">
         <f>IF($AA17="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA17,CaseTypeCol!$A:$A,0)))</f>
@@ -9056,7 +9056,7 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D18" t="s">
         <v>16</v>
@@ -9066,7 +9066,7 @@
         <v>org_user2_1</v>
       </c>
       <c r="F18" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G18" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -9113,7 +9113,7 @@
         <v>0</v>
       </c>
       <c r="R18" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="S18" t="s">
         <v>119</v>
@@ -9140,7 +9140,7 @@
         <v>142</v>
       </c>
       <c r="AB18" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC18" s="6" t="str">
         <f>IF($AA18="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA18,CaseTypeCol!$A:$A,0)))</f>
@@ -9211,7 +9211,7 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D19" t="s">
         <v>18</v>
@@ -9221,7 +9221,7 @@
         <v>org_user2_2</v>
       </c>
       <c r="F19" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G19" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -9268,7 +9268,7 @@
         <v>0</v>
       </c>
       <c r="R19" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="S19" t="s">
         <v>119</v>
@@ -9295,7 +9295,7 @@
         <v>142</v>
       </c>
       <c r="AB19" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC19" s="6" t="str">
         <f>IF($AA19="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA19,CaseTypeCol!$A:$A,0)))</f>
@@ -9366,7 +9366,7 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D20" t="s">
         <v>19</v>
@@ -9376,7 +9376,7 @@
         <v>org_user2_3</v>
       </c>
       <c r="F20" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G20" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -9423,7 +9423,7 @@
         <v>0</v>
       </c>
       <c r="R20" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="S20" t="s">
         <v>119</v>
@@ -9450,7 +9450,7 @@
         <v>142</v>
       </c>
       <c r="AB20" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC20" s="6" t="str">
         <f>IF($AA20="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA20,CaseTypeCol!$A:$A,0)))</f>
@@ -9521,7 +9521,7 @@
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D21" t="s">
         <v>20</v>
@@ -9531,7 +9531,7 @@
         <v>org_user2_4</v>
       </c>
       <c r="F21" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G21" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -9578,7 +9578,7 @@
         <v>0</v>
       </c>
       <c r="R21" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="S21" t="s">
         <v>119</v>
@@ -9605,7 +9605,7 @@
         <v>142</v>
       </c>
       <c r="AB21" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC21" s="6" t="str">
         <f>IF($AA21="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA21,CaseTypeCol!$A:$A,0)))</f>
@@ -9676,7 +9676,7 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D22" t="s">
         <v>22</v>
@@ -9686,7 +9686,7 @@
         <v>org_user3_1</v>
       </c>
       <c r="F22" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G22" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -9733,7 +9733,7 @@
         <v>0</v>
       </c>
       <c r="R22" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="S22" t="s">
         <v>119</v>
@@ -9760,7 +9760,7 @@
         <v>142</v>
       </c>
       <c r="AB22" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC22" s="6" t="str">
         <f>IF($AA22="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA22,CaseTypeCol!$A:$A,0)))</f>
@@ -9831,7 +9831,7 @@
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D23" t="s">
         <v>24</v>
@@ -9841,7 +9841,7 @@
         <v>org_user3_2</v>
       </c>
       <c r="F23" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G23" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -9888,7 +9888,7 @@
         <v>0</v>
       </c>
       <c r="R23" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="S23" t="s">
         <v>119</v>
@@ -9915,7 +9915,7 @@
         <v>142</v>
       </c>
       <c r="AB23" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC23" s="6" t="str">
         <f>IF($AA23="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA23,CaseTypeCol!$A:$A,0)))</f>
@@ -9986,7 +9986,7 @@
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D24" t="s">
         <v>25</v>
@@ -9996,7 +9996,7 @@
         <v>org_user3_3</v>
       </c>
       <c r="F24" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G24" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10043,7 +10043,7 @@
         <v>0</v>
       </c>
       <c r="R24" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="S24" t="s">
         <v>119</v>
@@ -10070,7 +10070,7 @@
         <v>142</v>
       </c>
       <c r="AB24" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC24" s="6" t="str">
         <f>IF($AA24="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA24,CaseTypeCol!$A:$A,0)))</f>
@@ -10141,7 +10141,7 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D25" t="s">
         <v>26</v>
@@ -10151,7 +10151,7 @@
         <v>org_user3_4</v>
       </c>
       <c r="F25" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G25" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10198,7 +10198,7 @@
         <v>0</v>
       </c>
       <c r="R25" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="S25" t="s">
         <v>119</v>
@@ -10225,7 +10225,7 @@
         <v>142</v>
       </c>
       <c r="AB25" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC25" s="6" t="str">
         <f>IF($AA25="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA25,CaseTypeCol!$A:$A,0)))</f>
@@ -10296,7 +10296,7 @@
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -10306,7 +10306,7 @@
         <v>org_user4_1</v>
       </c>
       <c r="F26" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G26" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10353,7 +10353,7 @@
         <v>0</v>
       </c>
       <c r="R26" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="S26" t="s">
         <v>119</v>
@@ -10380,7 +10380,7 @@
         <v>142</v>
       </c>
       <c r="AB26" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC26" s="6" t="str">
         <f>IF($AA26="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA26,CaseTypeCol!$A:$A,0)))</f>
@@ -10451,7 +10451,7 @@
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D27" t="s">
         <v>30</v>
@@ -10461,7 +10461,7 @@
         <v>org_user4_2</v>
       </c>
       <c r="F27" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G27" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10508,7 +10508,7 @@
         <v>0</v>
       </c>
       <c r="R27" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="S27" t="s">
         <v>119</v>
@@ -10535,7 +10535,7 @@
         <v>142</v>
       </c>
       <c r="AB27" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC27" s="6" t="str">
         <f>IF($AA27="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA27,CaseTypeCol!$A:$A,0)))</f>
@@ -10606,7 +10606,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D28" t="s">
         <v>31</v>
@@ -10616,7 +10616,7 @@
         <v>org_user4_3</v>
       </c>
       <c r="F28" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G28" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10663,7 +10663,7 @@
         <v>0</v>
       </c>
       <c r="R28" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="S28" t="s">
         <v>119</v>
@@ -10690,7 +10690,7 @@
         <v>142</v>
       </c>
       <c r="AB28" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC28" s="6" t="str">
         <f>IF($AA28="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA28,CaseTypeCol!$A:$A,0)))</f>
@@ -10761,7 +10761,7 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D29" t="s">
         <v>32</v>
@@ -10771,7 +10771,7 @@
         <v>org_user4_4</v>
       </c>
       <c r="F29" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G29" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10818,7 +10818,7 @@
         <v>0</v>
       </c>
       <c r="R29" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="S29" t="s">
         <v>119</v>
@@ -10845,7 +10845,7 @@
         <v>142</v>
       </c>
       <c r="AB29" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC29" s="6" t="str">
         <f>IF($AA29="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA29,CaseTypeCol!$A:$A,0)))</f>
@@ -10916,7 +10916,7 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D30" t="s">
         <v>34</v>
@@ -10926,7 +10926,7 @@
         <v>org_user5_1</v>
       </c>
       <c r="F30" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G30" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10973,7 +10973,7 @@
         <v>0</v>
       </c>
       <c r="R30" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="S30" t="s">
         <v>119</v>
@@ -11000,7 +11000,7 @@
         <v>142</v>
       </c>
       <c r="AB30" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC30" s="6" t="str">
         <f>IF($AA30="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA30,CaseTypeCol!$A:$A,0)))</f>
@@ -11071,7 +11071,7 @@
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D31" t="s">
         <v>36</v>
@@ -11081,7 +11081,7 @@
         <v>org_user5_2</v>
       </c>
       <c r="F31" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G31" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -11128,7 +11128,7 @@
         <v>0</v>
       </c>
       <c r="R31" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="S31" t="s">
         <v>119</v>
@@ -11155,7 +11155,7 @@
         <v>142</v>
       </c>
       <c r="AB31" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC31" s="6" t="str">
         <f>IF($AA31="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA31,CaseTypeCol!$A:$A,0)))</f>
@@ -11226,7 +11226,7 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D32" t="s">
         <v>37</v>
@@ -11236,7 +11236,7 @@
         <v>org_user5_3</v>
       </c>
       <c r="F32" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G32" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -11283,7 +11283,7 @@
         <v>0</v>
       </c>
       <c r="R32" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="S32" t="s">
         <v>119</v>
@@ -11310,7 +11310,7 @@
         <v>142</v>
       </c>
       <c r="AB32" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC32" s="6" t="str">
         <f>IF($AA32="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA32,CaseTypeCol!$A:$A,0)))</f>
@@ -11381,7 +11381,7 @@
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D33" t="s">
         <v>38</v>
@@ -11391,7 +11391,7 @@
         <v>org_user5_4</v>
       </c>
       <c r="F33" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G33" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -11438,7 +11438,7 @@
         <v>0</v>
       </c>
       <c r="R33" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="S33" t="s">
         <v>119</v>
@@ -11465,7 +11465,7 @@
         <v>142</v>
       </c>
       <c r="AB33" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AC33" s="6" t="str">
         <f>IF($AA33="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA33,CaseTypeCol!$A:$A,0)))</f>
@@ -11577,19 +11577,19 @@
         <v>2</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>4</v>
@@ -11598,16 +11598,16 @@
         <v>5</v>
       </c>
       <c r="J1" s="7" t="s">
+        <v>559</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>561</v>
+      </c>
+      <c r="L1" s="7" t="s">
         <v>560</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="M1" s="8" t="s">
         <v>562</v>
-      </c>
-      <c r="L1" s="7" t="s">
-        <v>561</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>563</v>
       </c>
       <c r="N1" s="7" t="s">
         <v>6</v>
@@ -11625,16 +11625,16 @@
         <v>41</v>
       </c>
       <c r="S1" s="8" t="s">
+        <v>563</v>
+      </c>
+      <c r="T1" s="4" t="s">
         <v>564</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="U1" s="8" t="s">
         <v>565</v>
       </c>
-      <c r="U1" s="8" t="s">
-        <v>566</v>
-      </c>
       <c r="V1" s="8" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
@@ -12431,13 +12431,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>3</v>
@@ -12449,16 +12449,16 @@
         <v>5</v>
       </c>
       <c r="I1" s="7" t="s">
+        <v>559</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>561</v>
+      </c>
+      <c r="K1" s="7" t="s">
         <v>560</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="L1" s="8" t="s">
         <v>562</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>561</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>563</v>
       </c>
       <c r="M1" s="7" t="s">
         <v>6</v>
@@ -12473,25 +12473,25 @@
         <v>9</v>
       </c>
       <c r="Q1" s="8" t="s">
+        <v>569</v>
+      </c>
+      <c r="R1" s="8" t="s">
         <v>570</v>
       </c>
-      <c r="R1" s="8" t="s">
-        <v>571</v>
-      </c>
       <c r="S1" s="4" t="s">
+        <v>564</v>
+      </c>
+      <c r="T1" s="8" t="s">
         <v>565</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="U1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="V1" s="8" t="s">
         <v>566</v>
       </c>
-      <c r="U1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="V1" s="8" t="s">
-        <v>567</v>
-      </c>
       <c r="W1" s="15" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
@@ -13342,7 +13342,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C2" s="6" t="str">
         <f>"dc"&amp;RIGHT($B2,LEN($B2)-15)</f>
@@ -13354,7 +13354,7 @@
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C3" s="6" t="str">
         <f t="shared" ref="C3:C12" si="0">"dc"&amp;RIGHT($B3,LEN($B3)-15)</f>
@@ -13366,7 +13366,7 @@
         <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C4" s="6" t="str">
         <f t="shared" si="0"/>
@@ -13378,7 +13378,7 @@
         <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C5" s="6" t="str">
         <f t="shared" si="0"/>
@@ -13390,7 +13390,7 @@
         <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C6" s="6" t="str">
         <f t="shared" si="0"/>
@@ -13402,7 +13402,7 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="C7" s="6" t="str">
         <f t="shared" si="0"/>
@@ -13414,7 +13414,7 @@
         <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C8" s="6" t="str">
         <f t="shared" si="0"/>
@@ -13426,7 +13426,7 @@
         <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C9" s="6" t="str">
         <f t="shared" si="0"/>
@@ -13438,7 +13438,7 @@
         <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C10" s="6" t="str">
         <f t="shared" si="0"/>
@@ -13450,7 +13450,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C11" s="6" t="str">
         <f t="shared" si="0"/>
@@ -13462,7 +13462,7 @@
         <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C12" s="6" t="str">
         <f t="shared" si="0"/>
@@ -13504,13 +13504,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="D1" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -13528,27 +13528,27 @@
         <v>7</v>
       </c>
       <c r="K1" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="M1" s="6" t="s">
+        <v>569</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>570</v>
       </c>
-      <c r="N1" s="3" t="s">
-        <v>571</v>
-      </c>
       <c r="O1" s="7" t="s">
         <v>1</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
@@ -13640,13 +13640,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="D1" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -13664,21 +13664,21 @@
         <v>7</v>
       </c>
       <c r="K1" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="M1" t="s">
         <v>41</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
@@ -13770,30 +13770,30 @@
         <v>41</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="H1" s="5" t="s">
+        <v>672</v>
+      </c>
+      <c r="I1" s="5" t="s">
         <v>673</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
+        <v>719</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>674</v>
       </c>
-      <c r="J1" s="5" t="s">
-        <v>720</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>675</v>
-      </c>
       <c r="L1" s="17" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>724</v>
+      </c>
+      <c r="B2" t="s">
         <v>443</v>
-      </c>
-      <c r="B2" t="s">
-        <v>444</v>
       </c>
       <c r="C2" t="str">
         <f>LEFT(B2,FIND("@",B2)-1)</f>
@@ -13803,7 +13803,7 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="F2" t="s">
         <v>43</v>
@@ -13835,10 +13835,10 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>444</v>
+      </c>
+      <c r="B3" t="s">
         <v>445</v>
-      </c>
-      <c r="B3" t="s">
-        <v>446</v>
       </c>
       <c r="C3" t="str">
         <f t="shared" ref="C3:C29" si="0">LEFT(B3,FIND("@",B3)-1)</f>
@@ -13848,7 +13848,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="F3" t="s">
         <v>43</v>
@@ -13880,10 +13880,10 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="C4" t="str">
         <f t="shared" si="0"/>
@@ -13893,7 +13893,7 @@
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="F4" t="s">
         <v>43</v>
@@ -13928,7 +13928,7 @@
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="0"/>
@@ -13938,7 +13938,7 @@
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F5" t="s">
         <v>43</v>
@@ -13973,7 +13973,7 @@
         <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C6" t="str">
         <f t="shared" si="0"/>
@@ -13983,7 +13983,7 @@
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F6" t="s">
         <v>46</v>
@@ -14018,7 +14018,7 @@
         <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="0"/>
@@ -14028,7 +14028,7 @@
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F7" t="s">
         <v>49</v>
@@ -14063,7 +14063,7 @@
         <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="0"/>
@@ -14073,7 +14073,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F8" t="s">
         <v>52</v>
@@ -14108,7 +14108,7 @@
         <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C9" t="str">
         <f t="shared" si="0"/>
@@ -14118,7 +14118,7 @@
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F9" t="s">
         <v>55</v>
@@ -14153,7 +14153,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C10" t="str">
         <f t="shared" si="0"/>
@@ -14163,7 +14163,7 @@
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F10" t="s">
         <v>43</v>
@@ -14198,7 +14198,7 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C11" t="str">
         <f t="shared" si="0"/>
@@ -14208,7 +14208,7 @@
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F11" t="s">
         <v>43</v>
@@ -14243,7 +14243,7 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C12" t="str">
         <f t="shared" si="0"/>
@@ -14253,7 +14253,7 @@
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F12" t="s">
         <v>43</v>
@@ -14288,7 +14288,7 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C13" t="str">
         <f t="shared" si="0"/>
@@ -14298,7 +14298,7 @@
         <v>1</v>
       </c>
       <c r="E13" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F13" t="s">
         <v>43</v>
@@ -14333,7 +14333,7 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C14" t="str">
         <f t="shared" si="0"/>
@@ -14343,7 +14343,7 @@
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F14" t="s">
         <v>46</v>
@@ -14378,7 +14378,7 @@
         <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C15" t="str">
         <f t="shared" si="0"/>
@@ -14388,7 +14388,7 @@
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F15" t="s">
         <v>46</v>
@@ -14423,7 +14423,7 @@
         <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C16" t="str">
         <f t="shared" si="0"/>
@@ -14433,7 +14433,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F16" t="s">
         <v>46</v>
@@ -14468,7 +14468,7 @@
         <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C17" t="str">
         <f t="shared" si="0"/>
@@ -14478,7 +14478,7 @@
         <v>1</v>
       </c>
       <c r="E17" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F17" t="s">
         <v>46</v>
@@ -14513,7 +14513,7 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C18" t="str">
         <f t="shared" si="0"/>
@@ -14523,7 +14523,7 @@
         <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F18" t="s">
         <v>49</v>
@@ -14558,7 +14558,7 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C19" t="str">
         <f t="shared" si="0"/>
@@ -14568,7 +14568,7 @@
         <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F19" t="s">
         <v>49</v>
@@ -14603,7 +14603,7 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C20" t="str">
         <f t="shared" si="0"/>
@@ -14613,7 +14613,7 @@
         <v>1</v>
       </c>
       <c r="E20" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F20" t="s">
         <v>49</v>
@@ -14648,7 +14648,7 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C21" t="str">
         <f t="shared" si="0"/>
@@ -14658,7 +14658,7 @@
         <v>1</v>
       </c>
       <c r="E21" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F21" t="s">
         <v>49</v>
@@ -14693,7 +14693,7 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C22" t="str">
         <f t="shared" si="0"/>
@@ -14703,7 +14703,7 @@
         <v>1</v>
       </c>
       <c r="E22" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F22" t="s">
         <v>52</v>
@@ -14738,7 +14738,7 @@
         <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C23" t="str">
         <f t="shared" si="0"/>
@@ -14748,7 +14748,7 @@
         <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F23" t="s">
         <v>52</v>
@@ -14783,7 +14783,7 @@
         <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C24" t="str">
         <f t="shared" si="0"/>
@@ -14793,7 +14793,7 @@
         <v>1</v>
       </c>
       <c r="E24" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F24" t="s">
         <v>52</v>
@@ -14828,7 +14828,7 @@
         <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C25" t="str">
         <f t="shared" si="0"/>
@@ -14838,7 +14838,7 @@
         <v>1</v>
       </c>
       <c r="E25" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F25" t="s">
         <v>52</v>
@@ -14873,7 +14873,7 @@
         <v>34</v>
       </c>
       <c r="B26" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C26" t="str">
         <f t="shared" si="0"/>
@@ -14883,7 +14883,7 @@
         <v>1</v>
       </c>
       <c r="E26" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F26" t="s">
         <v>55</v>
@@ -14918,7 +14918,7 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C27" t="str">
         <f t="shared" si="0"/>
@@ -14928,7 +14928,7 @@
         <v>1</v>
       </c>
       <c r="E27" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F27" t="s">
         <v>55</v>
@@ -14963,7 +14963,7 @@
         <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C28" t="str">
         <f t="shared" si="0"/>
@@ -14973,7 +14973,7 @@
         <v>1</v>
       </c>
       <c r="E28" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F28" t="s">
         <v>55</v>
@@ -15008,7 +15008,7 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C29" t="str">
         <f t="shared" si="0"/>
@@ -15018,7 +15018,7 @@
         <v>1</v>
       </c>
       <c r="E29" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F29" t="s">
         <v>55</v>
@@ -15081,52 +15081,52 @@
         <v>441</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>493</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>494</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>442</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>41</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C2" s="6" t="str">
         <f>LEFT($B2,LEN($B2)-9)</f>
         <v>app_admin1_1</v>
       </c>
       <c r="D2" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E2" s="2">
         <v>45743.390918726589</v>
       </c>
       <c r="F2" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="G2" t="s">
-        <v>443</v>
+        <v>724</v>
       </c>
       <c r="H2" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G2,User!$A:$A,0))</f>
@@ -15142,26 +15142,26 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="C3" s="6" t="str">
         <f t="shared" ref="C3:C28" si="0">LEFT($B3,LEN($B3)-9)</f>
         <v>refdata_admin1_1</v>
       </c>
       <c r="D3" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="E3" s="2">
         <v>45743.390918741461</v>
       </c>
       <c r="F3" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H3" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G3,User!$A:$A,0))</f>
@@ -15177,26 +15177,26 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C4" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_admin1_1</v>
       </c>
       <c r="D4" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="E4" s="2">
         <v>45743.390918746562</v>
       </c>
       <c r="F4" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G4" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H4" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G4,User!$A:$A,0))</f>
@@ -15212,26 +15212,26 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B5" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C5" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_admin2_1</v>
       </c>
       <c r="D5" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="E5" s="2">
         <v>45743.390918763551</v>
       </c>
       <c r="F5" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G5" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H5" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G5,User!$A:$A,0))</f>
@@ -15247,26 +15247,26 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B6" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C6" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_admin3_1</v>
       </c>
       <c r="D6" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="E6" s="2">
         <v>45743.390918772537</v>
       </c>
       <c r="F6" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G6" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H6" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G6,User!$A:$A,0))</f>
@@ -15282,26 +15282,26 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B7" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C7" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_admin4_1</v>
       </c>
       <c r="D7" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="E7" s="2">
         <v>45743.390918781181</v>
       </c>
       <c r="F7" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G7" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H7" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G7,User!$A:$A,0))</f>
@@ -15317,26 +15317,26 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B8" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C8" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_admin5_1</v>
       </c>
       <c r="D8" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="E8" s="2">
         <v>45743.3909187889</v>
       </c>
       <c r="F8" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G8" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H8" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G8,User!$A:$A,0))</f>
@@ -15352,26 +15352,26 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B9" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C9" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user1_1</v>
       </c>
       <c r="D9" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="E9" s="2">
         <v>45743.390918796598</v>
       </c>
       <c r="F9" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G9" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H9" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G9,User!$A:$A,0))</f>
@@ -15387,26 +15387,26 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B10" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C10" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user1_2</v>
       </c>
       <c r="D10" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="E10" s="2">
         <v>45743.390918801953</v>
       </c>
       <c r="F10" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G10" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H10" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G10,User!$A:$A,0))</f>
@@ -15422,26 +15422,26 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B11" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C11" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user1_3</v>
       </c>
       <c r="D11" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="E11" s="2">
         <v>45743.390918807163</v>
       </c>
       <c r="F11" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G11" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H11" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G11,User!$A:$A,0))</f>
@@ -15457,26 +15457,26 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B12" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C12" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user1_4</v>
       </c>
       <c r="D12" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="E12" s="2">
         <v>45743.3909188123</v>
       </c>
       <c r="F12" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G12" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H12" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G12,User!$A:$A,0))</f>
@@ -15492,26 +15492,26 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B13" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C13" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user2_1</v>
       </c>
       <c r="D13" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="E13" s="2">
         <v>45743.390918817633</v>
       </c>
       <c r="F13" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G13" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H13" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G13,User!$A:$A,0))</f>
@@ -15527,26 +15527,26 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B14" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C14" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user2_2</v>
       </c>
       <c r="D14" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="E14" s="2">
         <v>45743.390918822908</v>
       </c>
       <c r="F14" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G14" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H14" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G14,User!$A:$A,0))</f>
@@ -15562,26 +15562,26 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B15" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C15" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user2_3</v>
       </c>
       <c r="D15" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E15" s="2">
         <v>45743.390918828743</v>
       </c>
       <c r="F15" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G15" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H15" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G15,User!$A:$A,0))</f>
@@ -15597,26 +15597,26 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B16" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C16" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user2_4</v>
       </c>
       <c r="D16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E16" s="2">
         <v>45743.390918834302</v>
       </c>
       <c r="F16" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G16" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H16" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G16,User!$A:$A,0))</f>
@@ -15632,26 +15632,26 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B17" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C17" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user3_1</v>
       </c>
       <c r="D17" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="E17" s="2">
         <v>45743.390918839839</v>
       </c>
       <c r="F17" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G17" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H17" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G17,User!$A:$A,0))</f>
@@ -15667,26 +15667,26 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B18" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C18" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user3_2</v>
       </c>
       <c r="D18" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="E18" s="2">
         <v>45743.390918845187</v>
       </c>
       <c r="F18" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G18" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H18" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G18,User!$A:$A,0))</f>
@@ -15702,26 +15702,26 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B19" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C19" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user3_3</v>
       </c>
       <c r="D19" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="E19" s="2">
         <v>45743.390918851088</v>
       </c>
       <c r="F19" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G19" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H19" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G19,User!$A:$A,0))</f>
@@ -15737,26 +15737,26 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B20" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C20" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user3_4</v>
       </c>
       <c r="D20" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="E20" s="2">
         <v>45743.39091885696</v>
       </c>
       <c r="F20" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G20" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H20" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G20,User!$A:$A,0))</f>
@@ -15772,26 +15772,26 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B21" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C21" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user4_1</v>
       </c>
       <c r="D21" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="E21" s="2">
         <v>45743.390918862962</v>
       </c>
       <c r="F21" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G21" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H21" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G21,User!$A:$A,0))</f>
@@ -15807,26 +15807,26 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B22" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C22" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user4_2</v>
       </c>
       <c r="D22" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="E22" s="2">
         <v>45743.390918868739</v>
       </c>
       <c r="F22" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G22" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H22" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G22,User!$A:$A,0))</f>
@@ -15842,26 +15842,26 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B23" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C23" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user4_3</v>
       </c>
       <c r="D23" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="E23" s="2">
         <v>45743.390918874728</v>
       </c>
       <c r="F23" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G23" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H23" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G23,User!$A:$A,0))</f>
@@ -15877,26 +15877,26 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B24" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C24" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user4_4</v>
       </c>
       <c r="D24" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="E24" s="2">
         <v>45743.390918881109</v>
       </c>
       <c r="F24" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G24" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H24" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G24,User!$A:$A,0))</f>
@@ -15912,26 +15912,26 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B25" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C25" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user5_1</v>
       </c>
       <c r="D25" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="E25" s="2">
         <v>45743.390918887373</v>
       </c>
       <c r="F25" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G25" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H25" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G25,User!$A:$A,0))</f>
@@ -15947,26 +15947,26 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B26" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C26" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user5_2</v>
       </c>
       <c r="D26" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E26" s="2">
         <v>45743.39091889358</v>
       </c>
       <c r="F26" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G26" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H26" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G26,User!$A:$A,0))</f>
@@ -15982,26 +15982,26 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B27" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C27" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user5_3</v>
       </c>
       <c r="D27" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="E27" s="2">
         <v>45743.390918900091</v>
       </c>
       <c r="F27" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G27" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H27" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G27,User!$A:$A,0))</f>
@@ -16017,26 +16017,26 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B28" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C28" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user5_4</v>
       </c>
       <c r="D28" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="E28" s="2">
         <v>45743.390918906553</v>
       </c>
       <c r="F28" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G28" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H28" s="6" t="str">
         <f>INDEX(User!$C:$C,MATCH($G28,User!$A:$A,0))</f>
@@ -16103,10 +16103,10 @@
         <v>424</v>
       </c>
       <c r="B2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D2" t="s">
         <v>438</v>
@@ -16124,10 +16124,10 @@
         <v>428</v>
       </c>
       <c r="B3" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D3" t="s">
         <v>439</v>
@@ -16145,10 +16145,10 @@
         <v>432</v>
       </c>
       <c r="B4" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="D4" t="s">
         <v>440</v>
@@ -16247,7 +16247,7 @@
         <v>424</v>
       </c>
       <c r="E2" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -16256,7 +16256,7 @@
         <v>425</v>
       </c>
       <c r="H2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="O2" s="13" t="str">
         <f>"col"&amp;$E2&amp;"("&amp;$H2&amp;")"</f>
@@ -16274,7 +16274,7 @@
         <v>424</v>
       </c>
       <c r="E3" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="F3">
         <v>2</v>
@@ -16283,7 +16283,7 @@
         <v>426</v>
       </c>
       <c r="H3" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="O3" s="13" t="str">
         <f t="shared" ref="O3:O10" si="0">"col"&amp;$E3&amp;"("&amp;$H3&amp;")"</f>
@@ -16301,7 +16301,7 @@
         <v>424</v>
       </c>
       <c r="E4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="F4">
         <v>3</v>
@@ -16310,7 +16310,7 @@
         <v>427</v>
       </c>
       <c r="H4" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="O4" s="13" t="str">
         <f t="shared" si="0"/>
@@ -16328,7 +16328,7 @@
         <v>428</v>
       </c>
       <c r="E5" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -16337,7 +16337,7 @@
         <v>429</v>
       </c>
       <c r="H5" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="O5" s="13" t="str">
         <f t="shared" si="0"/>
@@ -16355,7 +16355,7 @@
         <v>428</v>
       </c>
       <c r="E6" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="F6">
         <v>2</v>
@@ -16364,7 +16364,7 @@
         <v>430</v>
       </c>
       <c r="H6" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="O6" s="13" t="str">
         <f t="shared" si="0"/>
@@ -16382,7 +16382,7 @@
         <v>428</v>
       </c>
       <c r="E7" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="F7">
         <v>3</v>
@@ -16391,7 +16391,7 @@
         <v>431</v>
       </c>
       <c r="H7" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="O7" s="13" t="str">
         <f t="shared" si="0"/>
@@ -16409,7 +16409,7 @@
         <v>432</v>
       </c>
       <c r="E8" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -16418,7 +16418,7 @@
         <v>433</v>
       </c>
       <c r="H8" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="O8" s="13" t="str">
         <f t="shared" si="0"/>
@@ -16436,7 +16436,7 @@
         <v>432</v>
       </c>
       <c r="E9" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="F9">
         <v>2</v>
@@ -16445,7 +16445,7 @@
         <v>434</v>
       </c>
       <c r="H9" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="O9" s="13" t="str">
         <f t="shared" si="0"/>
@@ -16463,7 +16463,7 @@
         <v>432</v>
       </c>
       <c r="E10" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="F10">
         <v>3</v>
@@ -16472,7 +16472,7 @@
         <v>435</v>
       </c>
       <c r="H10" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="O10" s="13" t="str">
         <f t="shared" si="0"/>
@@ -16503,7 +16503,7 @@
         <v>57</v>
       </c>
       <c r="C1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -16511,7 +16511,7 @@
         <v>121</v>
       </c>
       <c r="B2" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -16519,7 +16519,7 @@
         <v>125</v>
       </c>
       <c r="B3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -16527,7 +16527,7 @@
         <v>129</v>
       </c>
       <c r="B4" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -16535,7 +16535,7 @@
         <v>133</v>
       </c>
       <c r="B5" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -16543,7 +16543,7 @@
         <v>137</v>
       </c>
       <c r="B6" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
   </sheetData>
@@ -16570,7 +16570,7 @@
         <v>57</v>
       </c>
       <c r="C1" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -16578,10 +16578,10 @@
         <v>122</v>
       </c>
       <c r="B2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="C2" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -16589,10 +16589,10 @@
         <v>126</v>
       </c>
       <c r="B3" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C3" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -16600,10 +16600,10 @@
         <v>130</v>
       </c>
       <c r="B4" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C4" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -16611,10 +16611,10 @@
         <v>134</v>
       </c>
       <c r="B5" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="C5" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -16622,10 +16622,10 @@
         <v>138</v>
       </c>
       <c r="B6" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C6" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
   </sheetData>
@@ -16663,7 +16663,7 @@
         <v>115</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>116</v>
@@ -16672,7 +16672,7 @@
         <v>117</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>118</v>

</xml_diff>

<commit_message>
refactor: User.roles as string; WIP omopdb/seqdb/casedb refactored but ETL still to be run and tested further test: general.unit.shortest_input_path added
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_access/test_casedb_case_access.xlsx
+++ b/test/casedb/integration/case_access/test_casedb_case_access.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_access\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C9948B-3BC4-47F4-B53C-6DB869600E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A61D31B2-B840-4A5B-BB17-403CEBADC04A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2508" yWindow="2508" windowWidth="30960" windowHeight="12120" tabRatio="913" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3552" yWindow="3552" windowWidth="30960" windowHeight="12120" tabRatio="913" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Organization" sheetId="17" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2143" uniqueCount="786">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2143" uniqueCount="790">
   <si>
     <t>id</t>
   </si>
@@ -1739,9 +1739,6 @@
     <t>dm.organization</t>
   </si>
   <si>
-    <t>["ROOT"]</t>
-  </si>
-  <si>
     <t>["APP_ADMIN"]</t>
   </si>
   <si>
@@ -2439,6 +2436,21 @@
   </si>
   <si>
     <t>key</t>
+  </si>
+  <si>
+    <t>["CASEDB_ROOT"]</t>
+  </si>
+  <si>
+    <t>["CASEDB_APP_ADMIN"]</t>
+  </si>
+  <si>
+    <t>["CASEDB_REFDATA_ADMIN"]</t>
+  </si>
+  <si>
+    <t>["CASEDB_ORG_ADMIN"]</t>
+  </si>
+  <si>
+    <t>["CASEDB_ORG_USER"]</t>
   </si>
 </sst>
 </file>
@@ -3104,7 +3116,7 @@
         <v>83</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>84</v>
@@ -3411,7 +3423,7 @@
         <v>58</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>59</v>
@@ -3420,13 +3432,13 @@
         <v>316</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>317</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -5347,7 +5359,7 @@
         <v>60</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>61</v>
@@ -5356,13 +5368,13 @@
         <v>139</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>140</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -6609,145 +6621,145 @@
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>587</v>
+      </c>
+      <c r="B1" t="s">
+        <v>722</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>590</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>717</v>
+      </c>
+      <c r="F1" t="s">
         <v>588</v>
       </c>
-      <c r="B1" t="s">
-        <v>723</v>
-      </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="G1" s="19" t="s">
+        <v>598</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>675</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="R1" t="s">
+        <v>589</v>
+      </c>
+      <c r="S1" t="s">
         <v>591</v>
       </c>
-      <c r="E1" s="6" t="s">
-        <v>718</v>
-      </c>
-      <c r="F1" t="s">
-        <v>589</v>
-      </c>
-      <c r="G1" s="19" t="s">
-        <v>599</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>666</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>670</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>667</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>675</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>600</v>
-      </c>
-      <c r="M1" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="N1" s="6" t="s">
-        <v>669</v>
-      </c>
-      <c r="O1" s="6" t="s">
+      <c r="T1" s="6" t="s">
+        <v>659</v>
+      </c>
+      <c r="U1" s="6" t="s">
+        <v>664</v>
+      </c>
+      <c r="V1" t="s">
+        <v>592</v>
+      </c>
+      <c r="W1" t="s">
+        <v>593</v>
+      </c>
+      <c r="X1" s="6" t="s">
+        <v>677</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>594</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>595</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>596</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>597</v>
+      </c>
+      <c r="AC1" s="6" t="s">
         <v>676</v>
       </c>
-      <c r="P1" s="6" t="s">
-        <v>602</v>
-      </c>
-      <c r="Q1" s="6" t="s">
-        <v>603</v>
-      </c>
-      <c r="R1" t="s">
-        <v>590</v>
-      </c>
-      <c r="S1" t="s">
-        <v>592</v>
-      </c>
-      <c r="T1" s="6" t="s">
-        <v>660</v>
-      </c>
-      <c r="U1" s="6" t="s">
-        <v>665</v>
-      </c>
-      <c r="V1" t="s">
-        <v>593</v>
-      </c>
-      <c r="W1" t="s">
-        <v>594</v>
-      </c>
-      <c r="X1" s="6" t="s">
+      <c r="AD1" s="6" t="s">
+        <v>680</v>
+      </c>
+      <c r="AE1" s="6" t="s">
+        <v>681</v>
+      </c>
+      <c r="AF1" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="AG1" s="6" t="s">
+        <v>687</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>661</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>707</v>
+      </c>
+      <c r="AJ1" s="6" t="s">
         <v>678</v>
       </c>
-      <c r="Y1" t="s">
-        <v>595</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>596</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>597</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>598</v>
-      </c>
-      <c r="AC1" s="6" t="s">
-        <v>677</v>
-      </c>
-      <c r="AD1" s="6" t="s">
-        <v>681</v>
-      </c>
-      <c r="AE1" s="6" t="s">
+      <c r="AK1" s="6" t="s">
         <v>682</v>
       </c>
-      <c r="AF1" s="6" t="s">
-        <v>687</v>
-      </c>
-      <c r="AG1" s="6" t="s">
+      <c r="AL1" s="6" t="s">
+        <v>683</v>
+      </c>
+      <c r="AM1" s="6" t="s">
         <v>688</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AN1" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="AO1" t="s">
         <v>662</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AP1" t="s">
         <v>708</v>
       </c>
-      <c r="AJ1" s="6" t="s">
+      <c r="AQ1" s="6" t="s">
         <v>679</v>
       </c>
-      <c r="AK1" s="6" t="s">
-        <v>683</v>
-      </c>
-      <c r="AL1" s="6" t="s">
+      <c r="AR1" s="6" t="s">
         <v>684</v>
       </c>
-      <c r="AM1" s="6" t="s">
-        <v>689</v>
-      </c>
-      <c r="AN1" s="6" t="s">
+      <c r="AS1" s="6" t="s">
+        <v>685</v>
+      </c>
+      <c r="AT1" s="6" t="s">
         <v>690</v>
       </c>
-      <c r="AO1" t="s">
-        <v>663</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>709</v>
-      </c>
-      <c r="AQ1" s="6" t="s">
-        <v>680</v>
-      </c>
-      <c r="AR1" s="6" t="s">
-        <v>685</v>
-      </c>
-      <c r="AS1" s="6" t="s">
-        <v>686</v>
-      </c>
-      <c r="AT1" s="6" t="s">
+      <c r="AU1" s="6" t="s">
         <v>691</v>
-      </c>
-      <c r="AU1" s="6" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.3">
@@ -6758,17 +6770,17 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D2" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="E2" s="6" t="str">
         <f>INDEX(User!$D:$D,MATCH($D2,User!$A:$A,0))</f>
         <v>root1_1</v>
       </c>
       <c r="F2" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="G2" s="19" t="b">
         <f t="shared" ref="G2:G65" si="0">IF($F2="CREATE",$I2,IF($F2="CREATE_CASES",OR($I2,AND($K2,$L2,$O2,$P2,$AE2,AG2,$AL2,$AN2,$AS2,$AU2)),"TBD"))</f>
@@ -6815,7 +6827,7 @@
         <v>0</v>
       </c>
       <c r="R2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="S2" t="s">
         <v>119</v>
@@ -6842,7 +6854,7 @@
         <v>142</v>
       </c>
       <c r="AB2" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC2" s="6" t="str">
         <f>IF($AA2="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA2,CaseTypeCol!$A:$A,0)))</f>
@@ -6913,7 +6925,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D3" t="s">
         <v>444</v>
@@ -6923,7 +6935,7 @@
         <v>app_admin1_1</v>
       </c>
       <c r="F3" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="G3" s="19" t="b">
         <f t="shared" si="0"/>
@@ -6970,7 +6982,7 @@
         <v>0</v>
       </c>
       <c r="R3" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="S3" t="s">
         <v>119</v>
@@ -6997,7 +7009,7 @@
         <v>142</v>
       </c>
       <c r="AB3" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC3" s="6" t="str">
         <f>IF($AA3="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA3,CaseTypeCol!$A:$A,0)))</f>
@@ -7068,7 +7080,7 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D4" t="s">
         <v>446</v>
@@ -7078,7 +7090,7 @@
         <v>refdata_admin1_1</v>
       </c>
       <c r="F4" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="G4" s="19" t="b">
         <f t="shared" si="0"/>
@@ -7125,7 +7137,7 @@
         <v>0</v>
       </c>
       <c r="R4" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="S4" t="s">
         <v>119</v>
@@ -7152,7 +7164,7 @@
         <v>142</v>
       </c>
       <c r="AB4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC4" s="6" t="str">
         <f>IF($AA4="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA4,CaseTypeCol!$A:$A,0)))</f>
@@ -7223,7 +7235,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D5" t="s">
         <v>44</v>
@@ -7233,7 +7245,7 @@
         <v>org_admin1_1</v>
       </c>
       <c r="F5" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="G5" s="19" t="b">
         <f t="shared" si="0"/>
@@ -7280,7 +7292,7 @@
         <v>0</v>
       </c>
       <c r="R5" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="S5" t="s">
         <v>119</v>
@@ -7307,7 +7319,7 @@
         <v>142</v>
       </c>
       <c r="AB5" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC5" s="6" t="str">
         <f>IF($AA5="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA5,CaseTypeCol!$A:$A,0)))</f>
@@ -7378,7 +7390,7 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D6" t="s">
         <v>10</v>
@@ -7388,7 +7400,7 @@
         <v>org_user1_1</v>
       </c>
       <c r="F6" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="G6" s="19" t="b">
         <f t="shared" si="0"/>
@@ -7435,7 +7447,7 @@
         <v>1</v>
       </c>
       <c r="R6" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="S6" t="s">
         <v>119</v>
@@ -7462,7 +7474,7 @@
         <v>142</v>
       </c>
       <c r="AB6" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC6" s="6" t="str">
         <f>IF($AA6="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA6,CaseTypeCol!$A:$A,0)))</f>
@@ -7533,17 +7545,17 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="D7" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="E7" s="6" t="str">
         <f>INDEX(User!$D:$D,MATCH($D7,User!$A:$A,0))</f>
         <v>root1_1</v>
       </c>
       <c r="F7" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G7" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -7590,7 +7602,7 @@
         <v>0</v>
       </c>
       <c r="R7" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="S7" t="s">
         <v>119</v>
@@ -7617,7 +7629,7 @@
         <v>142</v>
       </c>
       <c r="AB7" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC7" s="6" t="str">
         <f>IF($AA7="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA7,CaseTypeCol!$A:$A,0)))</f>
@@ -7688,7 +7700,7 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="D8" t="s">
         <v>444</v>
@@ -7698,7 +7710,7 @@
         <v>app_admin1_1</v>
       </c>
       <c r="F8" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G8" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -7745,7 +7757,7 @@
         <v>0</v>
       </c>
       <c r="R8" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="S8" t="s">
         <v>119</v>
@@ -7772,7 +7784,7 @@
         <v>142</v>
       </c>
       <c r="AB8" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC8" s="6" t="str">
         <f>IF($AA8="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA8,CaseTypeCol!$A:$A,0)))</f>
@@ -7843,7 +7855,7 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D9" t="s">
         <v>44</v>
@@ -7853,7 +7865,7 @@
         <v>org_admin1_1</v>
       </c>
       <c r="F9" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G9" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -7900,7 +7912,7 @@
         <v>0</v>
       </c>
       <c r="R9" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="S9" t="s">
         <v>119</v>
@@ -7927,7 +7939,7 @@
         <v>142</v>
       </c>
       <c r="AB9" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC9" s="6" t="str">
         <f>IF($AA9="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA9,CaseTypeCol!$A:$A,0)))</f>
@@ -7998,7 +8010,7 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D10" t="s">
         <v>47</v>
@@ -8008,7 +8020,7 @@
         <v>org_admin2_1</v>
       </c>
       <c r="F10" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G10" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8055,7 +8067,7 @@
         <v>0</v>
       </c>
       <c r="R10" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="S10" t="s">
         <v>119</v>
@@ -8082,7 +8094,7 @@
         <v>142</v>
       </c>
       <c r="AB10" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC10" s="6" t="str">
         <f>IF($AA10="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA10,CaseTypeCol!$A:$A,0)))</f>
@@ -8153,7 +8165,7 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D11" t="s">
         <v>50</v>
@@ -8163,7 +8175,7 @@
         <v>org_admin3_1</v>
       </c>
       <c r="F11" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G11" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8210,7 +8222,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="S11" t="s">
         <v>119</v>
@@ -8237,7 +8249,7 @@
         <v>142</v>
       </c>
       <c r="AB11" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC11" s="6" t="str">
         <f>IF($AA11="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA11,CaseTypeCol!$A:$A,0)))</f>
@@ -8308,7 +8320,7 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D12" t="s">
         <v>53</v>
@@ -8318,7 +8330,7 @@
         <v>org_admin4_1</v>
       </c>
       <c r="F12" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G12" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8365,7 +8377,7 @@
         <v>0</v>
       </c>
       <c r="R12" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="S12" t="s">
         <v>119</v>
@@ -8392,7 +8404,7 @@
         <v>142</v>
       </c>
       <c r="AB12" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC12" s="6" t="str">
         <f>IF($AA12="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA12,CaseTypeCol!$A:$A,0)))</f>
@@ -8463,7 +8475,7 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D13" t="s">
         <v>56</v>
@@ -8473,7 +8485,7 @@
         <v>org_admin5_1</v>
       </c>
       <c r="F13" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G13" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8520,7 +8532,7 @@
         <v>0</v>
       </c>
       <c r="R13" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="S13" t="s">
         <v>119</v>
@@ -8547,7 +8559,7 @@
         <v>142</v>
       </c>
       <c r="AB13" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC13" s="6" t="str">
         <f>IF($AA13="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA13,CaseTypeCol!$A:$A,0)))</f>
@@ -8618,7 +8630,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D14" t="s">
         <v>10</v>
@@ -8628,7 +8640,7 @@
         <v>org_user1_1</v>
       </c>
       <c r="F14" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G14" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8675,7 +8687,7 @@
         <v>1</v>
       </c>
       <c r="R14" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="S14" t="s">
         <v>119</v>
@@ -8702,7 +8714,7 @@
         <v>142</v>
       </c>
       <c r="AB14" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC14" s="6" t="str">
         <f>IF($AA14="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA14,CaseTypeCol!$A:$A,0)))</f>
@@ -8773,7 +8785,7 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
@@ -8783,7 +8795,7 @@
         <v>org_user1_2</v>
       </c>
       <c r="F15" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G15" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8830,7 +8842,7 @@
         <v>0</v>
       </c>
       <c r="R15" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="S15" t="s">
         <v>119</v>
@@ -8857,7 +8869,7 @@
         <v>142</v>
       </c>
       <c r="AB15" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC15" s="6" t="str">
         <f>IF($AA15="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA15,CaseTypeCol!$A:$A,0)))</f>
@@ -8928,7 +8940,7 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D16" t="s">
         <v>13</v>
@@ -8938,7 +8950,7 @@
         <v>org_user1_3</v>
       </c>
       <c r="F16" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G16" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -8985,7 +8997,7 @@
         <v>0</v>
       </c>
       <c r="R16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="S16" t="s">
         <v>119</v>
@@ -9012,7 +9024,7 @@
         <v>142</v>
       </c>
       <c r="AB16" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC16" s="6" t="str">
         <f>IF($AA16="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA16,CaseTypeCol!$A:$A,0)))</f>
@@ -9083,7 +9095,7 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D17" t="s">
         <v>14</v>
@@ -9093,7 +9105,7 @@
         <v>org_user1_4</v>
       </c>
       <c r="F17" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G17" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -9140,7 +9152,7 @@
         <v>0</v>
       </c>
       <c r="R17" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="S17" t="s">
         <v>119</v>
@@ -9167,7 +9179,7 @@
         <v>142</v>
       </c>
       <c r="AB17" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC17" s="6" t="str">
         <f>IF($AA17="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA17,CaseTypeCol!$A:$A,0)))</f>
@@ -9238,7 +9250,7 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D18" t="s">
         <v>16</v>
@@ -9248,7 +9260,7 @@
         <v>org_user2_1</v>
       </c>
       <c r="F18" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G18" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -9295,7 +9307,7 @@
         <v>0</v>
       </c>
       <c r="R18" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="S18" t="s">
         <v>119</v>
@@ -9322,7 +9334,7 @@
         <v>142</v>
       </c>
       <c r="AB18" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC18" s="6" t="str">
         <f>IF($AA18="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA18,CaseTypeCol!$A:$A,0)))</f>
@@ -9393,7 +9405,7 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D19" t="s">
         <v>18</v>
@@ -9403,7 +9415,7 @@
         <v>org_user2_2</v>
       </c>
       <c r="F19" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G19" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -9450,7 +9462,7 @@
         <v>0</v>
       </c>
       <c r="R19" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="S19" t="s">
         <v>119</v>
@@ -9477,7 +9489,7 @@
         <v>142</v>
       </c>
       <c r="AB19" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC19" s="6" t="str">
         <f>IF($AA19="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA19,CaseTypeCol!$A:$A,0)))</f>
@@ -9548,7 +9560,7 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D20" t="s">
         <v>19</v>
@@ -9558,7 +9570,7 @@
         <v>org_user2_3</v>
       </c>
       <c r="F20" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G20" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -9605,7 +9617,7 @@
         <v>0</v>
       </c>
       <c r="R20" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="S20" t="s">
         <v>119</v>
@@ -9632,7 +9644,7 @@
         <v>142</v>
       </c>
       <c r="AB20" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC20" s="6" t="str">
         <f>IF($AA20="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA20,CaseTypeCol!$A:$A,0)))</f>
@@ -9703,7 +9715,7 @@
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D21" t="s">
         <v>20</v>
@@ -9713,7 +9725,7 @@
         <v>org_user2_4</v>
       </c>
       <c r="F21" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G21" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -9760,7 +9772,7 @@
         <v>0</v>
       </c>
       <c r="R21" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="S21" t="s">
         <v>119</v>
@@ -9787,7 +9799,7 @@
         <v>142</v>
       </c>
       <c r="AB21" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC21" s="6" t="str">
         <f>IF($AA21="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA21,CaseTypeCol!$A:$A,0)))</f>
@@ -9858,7 +9870,7 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D22" t="s">
         <v>22</v>
@@ -9868,7 +9880,7 @@
         <v>org_user3_1</v>
       </c>
       <c r="F22" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G22" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -9915,7 +9927,7 @@
         <v>0</v>
       </c>
       <c r="R22" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="S22" t="s">
         <v>119</v>
@@ -9942,7 +9954,7 @@
         <v>142</v>
       </c>
       <c r="AB22" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC22" s="6" t="str">
         <f>IF($AA22="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA22,CaseTypeCol!$A:$A,0)))</f>
@@ -10013,7 +10025,7 @@
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D23" t="s">
         <v>24</v>
@@ -10023,7 +10035,7 @@
         <v>org_user3_2</v>
       </c>
       <c r="F23" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G23" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10070,7 +10082,7 @@
         <v>0</v>
       </c>
       <c r="R23" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="S23" t="s">
         <v>119</v>
@@ -10097,7 +10109,7 @@
         <v>142</v>
       </c>
       <c r="AB23" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC23" s="6" t="str">
         <f>IF($AA23="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA23,CaseTypeCol!$A:$A,0)))</f>
@@ -10168,7 +10180,7 @@
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D24" t="s">
         <v>25</v>
@@ -10178,7 +10190,7 @@
         <v>org_user3_3</v>
       </c>
       <c r="F24" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G24" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10225,7 +10237,7 @@
         <v>0</v>
       </c>
       <c r="R24" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="S24" t="s">
         <v>119</v>
@@ -10252,7 +10264,7 @@
         <v>142</v>
       </c>
       <c r="AB24" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC24" s="6" t="str">
         <f>IF($AA24="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA24,CaseTypeCol!$A:$A,0)))</f>
@@ -10323,7 +10335,7 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D25" t="s">
         <v>26</v>
@@ -10333,7 +10345,7 @@
         <v>org_user3_4</v>
       </c>
       <c r="F25" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G25" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10380,7 +10392,7 @@
         <v>0</v>
       </c>
       <c r="R25" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="S25" t="s">
         <v>119</v>
@@ -10407,7 +10419,7 @@
         <v>142</v>
       </c>
       <c r="AB25" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC25" s="6" t="str">
         <f>IF($AA25="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA25,CaseTypeCol!$A:$A,0)))</f>
@@ -10478,7 +10490,7 @@
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -10488,7 +10500,7 @@
         <v>org_user4_1</v>
       </c>
       <c r="F26" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G26" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10535,7 +10547,7 @@
         <v>0</v>
       </c>
       <c r="R26" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="S26" t="s">
         <v>119</v>
@@ -10562,7 +10574,7 @@
         <v>142</v>
       </c>
       <c r="AB26" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC26" s="6" t="str">
         <f>IF($AA26="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA26,CaseTypeCol!$A:$A,0)))</f>
@@ -10633,7 +10645,7 @@
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D27" t="s">
         <v>30</v>
@@ -10643,7 +10655,7 @@
         <v>org_user4_2</v>
       </c>
       <c r="F27" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G27" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10690,7 +10702,7 @@
         <v>0</v>
       </c>
       <c r="R27" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="S27" t="s">
         <v>119</v>
@@ -10717,7 +10729,7 @@
         <v>142</v>
       </c>
       <c r="AB27" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC27" s="6" t="str">
         <f>IF($AA27="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA27,CaseTypeCol!$A:$A,0)))</f>
@@ -10788,7 +10800,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D28" t="s">
         <v>31</v>
@@ -10798,7 +10810,7 @@
         <v>org_user4_3</v>
       </c>
       <c r="F28" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G28" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -10845,7 +10857,7 @@
         <v>0</v>
       </c>
       <c r="R28" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="S28" t="s">
         <v>119</v>
@@ -10872,7 +10884,7 @@
         <v>142</v>
       </c>
       <c r="AB28" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC28" s="6" t="str">
         <f>IF($AA28="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA28,CaseTypeCol!$A:$A,0)))</f>
@@ -10943,7 +10955,7 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D29" t="s">
         <v>32</v>
@@ -10953,7 +10965,7 @@
         <v>org_user4_4</v>
       </c>
       <c r="F29" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G29" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -11000,7 +11012,7 @@
         <v>0</v>
       </c>
       <c r="R29" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="S29" t="s">
         <v>119</v>
@@ -11027,7 +11039,7 @@
         <v>142</v>
       </c>
       <c r="AB29" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC29" s="6" t="str">
         <f>IF($AA29="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA29,CaseTypeCol!$A:$A,0)))</f>
@@ -11098,7 +11110,7 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D30" t="s">
         <v>34</v>
@@ -11108,7 +11120,7 @@
         <v>org_user5_1</v>
       </c>
       <c r="F30" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G30" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -11155,7 +11167,7 @@
         <v>0</v>
       </c>
       <c r="R30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="S30" t="s">
         <v>119</v>
@@ -11182,7 +11194,7 @@
         <v>142</v>
       </c>
       <c r="AB30" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC30" s="6" t="str">
         <f>IF($AA30="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA30,CaseTypeCol!$A:$A,0)))</f>
@@ -11253,7 +11265,7 @@
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D31" t="s">
         <v>36</v>
@@ -11263,7 +11275,7 @@
         <v>org_user5_2</v>
       </c>
       <c r="F31" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G31" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -11310,7 +11322,7 @@
         <v>0</v>
       </c>
       <c r="R31" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="S31" t="s">
         <v>119</v>
@@ -11337,7 +11349,7 @@
         <v>142</v>
       </c>
       <c r="AB31" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC31" s="6" t="str">
         <f>IF($AA31="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA31,CaseTypeCol!$A:$A,0)))</f>
@@ -11408,7 +11420,7 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D32" t="s">
         <v>37</v>
@@ -11418,7 +11430,7 @@
         <v>org_user5_3</v>
       </c>
       <c r="F32" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G32" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -11465,7 +11477,7 @@
         <v>0</v>
       </c>
       <c r="R32" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="S32" t="s">
         <v>119</v>
@@ -11492,7 +11504,7 @@
         <v>142</v>
       </c>
       <c r="AB32" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC32" s="6" t="str">
         <f>IF($AA32="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA32,CaseTypeCol!$A:$A,0)))</f>
@@ -11563,7 +11575,7 @@
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D33" t="s">
         <v>38</v>
@@ -11573,7 +11585,7 @@
         <v>org_user5_4</v>
       </c>
       <c r="F33" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G33" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -11620,7 +11632,7 @@
         <v>0</v>
       </c>
       <c r="R33" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="S33" t="s">
         <v>119</v>
@@ -11647,7 +11659,7 @@
         <v>142</v>
       </c>
       <c r="AB33" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC33" s="6" t="str">
         <f>IF($AA33="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA33,CaseTypeCol!$A:$A,0)))</f>
@@ -11718,7 +11730,7 @@
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="D34" t="s">
         <v>10</v>
@@ -11728,7 +11740,7 @@
         <v>org_user1_1</v>
       </c>
       <c r="F34" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G34" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -11775,7 +11787,7 @@
         <v>1</v>
       </c>
       <c r="R34" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S34" t="s">
         <v>119</v>
@@ -11802,7 +11814,7 @@
         <v>142</v>
       </c>
       <c r="AB34" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC34" s="6" t="str">
         <f>IF($AA34="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA34,CaseTypeCol!$A:$A,0)))</f>
@@ -11828,7 +11840,7 @@
         <v>142</v>
       </c>
       <c r="AI34" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="AJ34" s="6" t="str">
         <f>IF($AH34="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH34,CaseTypeCol!$A:$A,0)))</f>
@@ -11854,7 +11866,7 @@
         <v>142</v>
       </c>
       <c r="AP34" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="AQ34" s="6" t="str">
         <f>IF($AO34="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO34,CaseTypeCol!$A:$A,0)))</f>
@@ -11885,7 +11897,7 @@
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="D35" t="s">
         <v>12</v>
@@ -11895,7 +11907,7 @@
         <v>org_user1_2</v>
       </c>
       <c r="F35" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G35" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -11942,7 +11954,7 @@
         <v>0</v>
       </c>
       <c r="R35" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S35" t="s">
         <v>119</v>
@@ -11969,7 +11981,7 @@
         <v>142</v>
       </c>
       <c r="AB35" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC35" s="6" t="str">
         <f>IF($AA35="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA35,CaseTypeCol!$A:$A,0)))</f>
@@ -11992,7 +12004,7 @@
         <v>0</v>
       </c>
       <c r="AI35" s="11" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="AJ35" s="6" t="str">
         <f>IF($AH35="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH35,CaseTypeCol!$A:$A,0)))</f>
@@ -12043,7 +12055,7 @@
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D36" t="s">
         <v>13</v>
@@ -12053,7 +12065,7 @@
         <v>org_user1_3</v>
       </c>
       <c r="F36" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G36" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -12100,7 +12112,7 @@
         <v>0</v>
       </c>
       <c r="R36" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S36" t="s">
         <v>119</v>
@@ -12127,7 +12139,7 @@
         <v>142</v>
       </c>
       <c r="AB36" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC36" s="6" t="str">
         <f>IF($AA36="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA36,CaseTypeCol!$A:$A,0)))</f>
@@ -12150,7 +12162,7 @@
         <v>0</v>
       </c>
       <c r="AI36" s="11" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="AJ36" s="6" t="str">
         <f>IF($AH36="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH36,CaseTypeCol!$A:$A,0)))</f>
@@ -12201,7 +12213,7 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="D37" t="s">
         <v>14</v>
@@ -12211,7 +12223,7 @@
         <v>org_user1_4</v>
       </c>
       <c r="F37" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G37" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -12258,7 +12270,7 @@
         <v>0</v>
       </c>
       <c r="R37" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S37" t="s">
         <v>119</v>
@@ -12285,7 +12297,7 @@
         <v>142</v>
       </c>
       <c r="AB37" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC37" s="6" t="str">
         <f>IF($AA37="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA37,CaseTypeCol!$A:$A,0)))</f>
@@ -12308,7 +12320,7 @@
         <v>0</v>
       </c>
       <c r="AI37" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="AJ37" s="6" t="str">
         <f>IF($AH37="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH37,CaseTypeCol!$A:$A,0)))</f>
@@ -12359,7 +12371,7 @@
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="D38" t="s">
         <v>16</v>
@@ -12369,7 +12381,7 @@
         <v>org_user2_1</v>
       </c>
       <c r="F38" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G38" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -12416,7 +12428,7 @@
         <v>0</v>
       </c>
       <c r="R38" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S38" t="s">
         <v>119</v>
@@ -12443,7 +12455,7 @@
         <v>142</v>
       </c>
       <c r="AB38" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC38" s="6" t="str">
         <f>IF($AA38="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA38,CaseTypeCol!$A:$A,0)))</f>
@@ -12466,7 +12478,7 @@
         <v>0</v>
       </c>
       <c r="AI38" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AJ38" s="6" t="str">
         <f>IF($AH38="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH38,CaseTypeCol!$A:$A,0)))</f>
@@ -12517,7 +12529,7 @@
         <v>1</v>
       </c>
       <c r="C39" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="D39" t="s">
         <v>18</v>
@@ -12527,7 +12539,7 @@
         <v>org_user2_2</v>
       </c>
       <c r="F39" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G39" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -12574,7 +12586,7 @@
         <v>0</v>
       </c>
       <c r="R39" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S39" t="s">
         <v>119</v>
@@ -12601,7 +12613,7 @@
         <v>142</v>
       </c>
       <c r="AB39" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC39" s="6" t="str">
         <f>IF($AA39="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA39,CaseTypeCol!$A:$A,0)))</f>
@@ -12624,7 +12636,7 @@
         <v>0</v>
       </c>
       <c r="AI39" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="AJ39" s="6" t="str">
         <f>IF($AH39="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH39,CaseTypeCol!$A:$A,0)))</f>
@@ -12675,7 +12687,7 @@
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="D40" t="s">
         <v>19</v>
@@ -12685,7 +12697,7 @@
         <v>org_user2_3</v>
       </c>
       <c r="F40" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G40" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -12732,7 +12744,7 @@
         <v>0</v>
       </c>
       <c r="R40" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S40" t="s">
         <v>119</v>
@@ -12759,7 +12771,7 @@
         <v>142</v>
       </c>
       <c r="AB40" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC40" s="6" t="str">
         <f>IF($AA40="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA40,CaseTypeCol!$A:$A,0)))</f>
@@ -12782,7 +12794,7 @@
         <v>0</v>
       </c>
       <c r="AI40" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="AJ40" s="6" t="str">
         <f>IF($AH40="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH40,CaseTypeCol!$A:$A,0)))</f>
@@ -12833,7 +12845,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="D41" t="s">
         <v>20</v>
@@ -12843,7 +12855,7 @@
         <v>org_user2_4</v>
       </c>
       <c r="F41" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G41" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -12890,7 +12902,7 @@
         <v>0</v>
       </c>
       <c r="R41" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S41" t="s">
         <v>119</v>
@@ -12917,7 +12929,7 @@
         <v>142</v>
       </c>
       <c r="AB41" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC41" s="6" t="str">
         <f>IF($AA41="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA41,CaseTypeCol!$A:$A,0)))</f>
@@ -12940,7 +12952,7 @@
         <v>0</v>
       </c>
       <c r="AI41" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="AJ41" s="6" t="str">
         <f>IF($AH41="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH41,CaseTypeCol!$A:$A,0)))</f>
@@ -12991,7 +13003,7 @@
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="D42" t="s">
         <v>22</v>
@@ -13001,7 +13013,7 @@
         <v>org_user3_1</v>
       </c>
       <c r="F42" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G42" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -13048,7 +13060,7 @@
         <v>0</v>
       </c>
       <c r="R42" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S42" t="s">
         <v>119</v>
@@ -13075,7 +13087,7 @@
         <v>142</v>
       </c>
       <c r="AB42" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC42" s="6" t="str">
         <f>IF($AA42="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA42,CaseTypeCol!$A:$A,0)))</f>
@@ -13098,7 +13110,7 @@
         <v>0</v>
       </c>
       <c r="AI42" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="AJ42" s="6" t="str">
         <f>IF($AH42="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH42,CaseTypeCol!$A:$A,0)))</f>
@@ -13149,7 +13161,7 @@
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="D43" t="s">
         <v>24</v>
@@ -13159,7 +13171,7 @@
         <v>org_user3_2</v>
       </c>
       <c r="F43" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G43" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -13206,7 +13218,7 @@
         <v>0</v>
       </c>
       <c r="R43" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S43" t="s">
         <v>119</v>
@@ -13233,7 +13245,7 @@
         <v>142</v>
       </c>
       <c r="AB43" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC43" s="6" t="str">
         <f>IF($AA43="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA43,CaseTypeCol!$A:$A,0)))</f>
@@ -13256,7 +13268,7 @@
         <v>0</v>
       </c>
       <c r="AI43" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ43" s="6" t="str">
         <f>IF($AH43="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH43,CaseTypeCol!$A:$A,0)))</f>
@@ -13307,7 +13319,7 @@
         <v>1</v>
       </c>
       <c r="C44" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="D44" t="s">
         <v>25</v>
@@ -13317,7 +13329,7 @@
         <v>org_user3_3</v>
       </c>
       <c r="F44" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G44" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -13364,7 +13376,7 @@
         <v>0</v>
       </c>
       <c r="R44" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S44" t="s">
         <v>119</v>
@@ -13391,7 +13403,7 @@
         <v>142</v>
       </c>
       <c r="AB44" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC44" s="6" t="str">
         <f>IF($AA44="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA44,CaseTypeCol!$A:$A,0)))</f>
@@ -13462,7 +13474,7 @@
         <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="D45" t="s">
         <v>26</v>
@@ -13472,7 +13484,7 @@
         <v>org_user3_4</v>
       </c>
       <c r="F45" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G45" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -13519,7 +13531,7 @@
         <v>0</v>
       </c>
       <c r="R45" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S45" t="s">
         <v>119</v>
@@ -13546,7 +13558,7 @@
         <v>142</v>
       </c>
       <c r="AB45" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC45" s="6" t="str">
         <f>IF($AA45="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA45,CaseTypeCol!$A:$A,0)))</f>
@@ -13617,7 +13629,7 @@
         <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="D46" t="s">
         <v>28</v>
@@ -13627,7 +13639,7 @@
         <v>org_user4_1</v>
       </c>
       <c r="F46" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G46" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -13674,7 +13686,7 @@
         <v>0</v>
       </c>
       <c r="R46" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="S46" t="s">
         <v>119</v>
@@ -13701,7 +13713,7 @@
         <v>142</v>
       </c>
       <c r="AB46" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC46" s="6" t="str">
         <f>IF($AA46="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA46,CaseTypeCol!$A:$A,0)))</f>
@@ -13744,7 +13756,7 @@
         <v>1</v>
       </c>
       <c r="AP46" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="AQ46" s="6" t="str">
         <f>IF($AO46="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO46,CaseTypeCol!$A:$A,0)))</f>
@@ -13775,7 +13787,7 @@
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="D47" t="s">
         <v>30</v>
@@ -13785,7 +13797,7 @@
         <v>org_user4_2</v>
       </c>
       <c r="F47" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G47" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -13832,7 +13844,7 @@
         <v>0</v>
       </c>
       <c r="R47" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="S47" t="s">
         <v>119</v>
@@ -13859,7 +13871,7 @@
         <v>142</v>
       </c>
       <c r="AB47" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC47" s="6" t="str">
         <f>IF($AA47="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA47,CaseTypeCol!$A:$A,0)))</f>
@@ -13902,7 +13914,7 @@
         <v>1</v>
       </c>
       <c r="AP47" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="AQ47" s="6" t="str">
         <f>IF($AO47="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO47,CaseTypeCol!$A:$A,0)))</f>
@@ -13933,7 +13945,7 @@
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="D48" t="s">
         <v>31</v>
@@ -13943,7 +13955,7 @@
         <v>org_user4_3</v>
       </c>
       <c r="F48" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G48" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -13990,7 +14002,7 @@
         <v>0</v>
       </c>
       <c r="R48" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="S48" t="s">
         <v>119</v>
@@ -14017,7 +14029,7 @@
         <v>142</v>
       </c>
       <c r="AB48" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC48" s="6" t="str">
         <f>IF($AA48="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA48,CaseTypeCol!$A:$A,0)))</f>
@@ -14060,7 +14072,7 @@
         <v>1</v>
       </c>
       <c r="AP48" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="AQ48" s="6" t="str">
         <f>IF($AO48="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO48,CaseTypeCol!$A:$A,0)))</f>
@@ -14091,7 +14103,7 @@
         <v>1</v>
       </c>
       <c r="C49" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="D49" t="s">
         <v>32</v>
@@ -14101,7 +14113,7 @@
         <v>org_user4_4</v>
       </c>
       <c r="F49" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G49" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -14148,7 +14160,7 @@
         <v>0</v>
       </c>
       <c r="R49" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="S49" t="s">
         <v>119</v>
@@ -14175,7 +14187,7 @@
         <v>142</v>
       </c>
       <c r="AB49" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC49" s="6" t="str">
         <f>IF($AA49="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA49,CaseTypeCol!$A:$A,0)))</f>
@@ -14218,7 +14230,7 @@
         <v>1</v>
       </c>
       <c r="AP49" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="AQ49" s="6" t="str">
         <f>IF($AO49="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO49,CaseTypeCol!$A:$A,0)))</f>
@@ -14249,7 +14261,7 @@
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="D50" t="s">
         <v>34</v>
@@ -14259,7 +14271,7 @@
         <v>org_user5_1</v>
       </c>
       <c r="F50" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G50" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -14306,7 +14318,7 @@
         <v>0</v>
       </c>
       <c r="R50" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="S50" t="s">
         <v>119</v>
@@ -14333,7 +14345,7 @@
         <v>142</v>
       </c>
       <c r="AB50" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC50" s="6" t="str">
         <f>IF($AA50="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA50,CaseTypeCol!$A:$A,0)))</f>
@@ -14376,7 +14388,7 @@
         <v>1</v>
       </c>
       <c r="AP50" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="AQ50" s="6" t="str">
         <f>IF($AO50="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO50,CaseTypeCol!$A:$A,0)))</f>
@@ -14407,7 +14419,7 @@
         <v>1</v>
       </c>
       <c r="C51" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="D51" t="s">
         <v>36</v>
@@ -14417,7 +14429,7 @@
         <v>org_user5_2</v>
       </c>
       <c r="F51" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G51" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -14464,7 +14476,7 @@
         <v>0</v>
       </c>
       <c r="R51" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="S51" t="s">
         <v>119</v>
@@ -14491,7 +14503,7 @@
         <v>142</v>
       </c>
       <c r="AB51" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC51" s="6" t="str">
         <f>IF($AA51="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA51,CaseTypeCol!$A:$A,0)))</f>
@@ -14534,7 +14546,7 @@
         <v>1</v>
       </c>
       <c r="AP51" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="AQ51" s="6" t="str">
         <f>IF($AO51="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO51,CaseTypeCol!$A:$A,0)))</f>
@@ -14565,7 +14577,7 @@
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="D52" t="s">
         <v>37</v>
@@ -14575,7 +14587,7 @@
         <v>org_user5_3</v>
       </c>
       <c r="F52" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G52" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -14622,7 +14634,7 @@
         <v>0</v>
       </c>
       <c r="R52" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="S52" t="s">
         <v>119</v>
@@ -14649,7 +14661,7 @@
         <v>142</v>
       </c>
       <c r="AB52" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC52" s="6" t="str">
         <f>IF($AA52="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA52,CaseTypeCol!$A:$A,0)))</f>
@@ -14692,7 +14704,7 @@
         <v>1</v>
       </c>
       <c r="AP52" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="AQ52" s="6" t="str">
         <f>IF($AO52="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO52,CaseTypeCol!$A:$A,0)))</f>
@@ -14723,7 +14735,7 @@
         <v>1</v>
       </c>
       <c r="C53" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="D53" t="s">
         <v>38</v>
@@ -14733,7 +14745,7 @@
         <v>org_user5_4</v>
       </c>
       <c r="F53" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G53" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -14780,7 +14792,7 @@
         <v>0</v>
       </c>
       <c r="R53" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="S53" t="s">
         <v>119</v>
@@ -14807,7 +14819,7 @@
         <v>142</v>
       </c>
       <c r="AB53" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC53" s="6" t="str">
         <f>IF($AA53="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA53,CaseTypeCol!$A:$A,0)))</f>
@@ -14850,7 +14862,7 @@
         <v>1</v>
       </c>
       <c r="AP53" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="AQ53" s="6" t="str">
         <f>IF($AO53="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO53,CaseTypeCol!$A:$A,0)))</f>
@@ -14881,7 +14893,7 @@
         <v>1</v>
       </c>
       <c r="C54" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="D54" t="s">
         <v>10</v>
@@ -14891,7 +14903,7 @@
         <v>org_user1_1</v>
       </c>
       <c r="F54" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G54" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -14938,7 +14950,7 @@
         <v>0</v>
       </c>
       <c r="R54" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="S54" t="s">
         <v>123</v>
@@ -14965,7 +14977,7 @@
         <v>142</v>
       </c>
       <c r="AB54" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC54" s="6" t="str">
         <f>IF($AA54="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA54,CaseTypeCol!$A:$A,0)))</f>
@@ -14991,7 +15003,7 @@
         <v>142</v>
       </c>
       <c r="AI54" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="AJ54" s="6" t="str">
         <f>IF($AH54="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH54,CaseTypeCol!$A:$A,0)))</f>
@@ -15017,7 +15029,7 @@
         <v>142</v>
       </c>
       <c r="AP54" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="AQ54" s="6" t="str">
         <f>IF($AO54="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO54,CaseTypeCol!$A:$A,0)))</f>
@@ -15048,7 +15060,7 @@
         <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="D55" t="s">
         <v>10</v>
@@ -15058,7 +15070,7 @@
         <v>org_user1_1</v>
       </c>
       <c r="F55" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G55" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -15105,7 +15117,7 @@
         <v>0</v>
       </c>
       <c r="R55" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="S55" t="s">
         <v>127</v>
@@ -15132,7 +15144,7 @@
         <v>145</v>
       </c>
       <c r="AB55" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC55" s="6" t="str">
         <f>IF($AA55="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA55,CaseTypeCol!$A:$A,0)))</f>
@@ -15158,7 +15170,7 @@
         <v>145</v>
       </c>
       <c r="AI55" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="AJ55" s="6" t="str">
         <f>IF($AH55="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH55,CaseTypeCol!$A:$A,0)))</f>
@@ -15184,7 +15196,7 @@
         <v>145</v>
       </c>
       <c r="AP55" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="AQ55" s="6" t="str">
         <f>IF($AO55="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO55,CaseTypeCol!$A:$A,0)))</f>
@@ -15215,7 +15227,7 @@
         <v>1</v>
       </c>
       <c r="C56" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="D56" t="s">
         <v>10</v>
@@ -15225,7 +15237,7 @@
         <v>org_user1_1</v>
       </c>
       <c r="F56" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G56" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -15272,7 +15284,7 @@
         <v>0</v>
       </c>
       <c r="R56" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="S56" t="s">
         <v>131</v>
@@ -15299,7 +15311,7 @@
         <v>148</v>
       </c>
       <c r="AB56" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC56" s="6" t="str">
         <f>IF($AA56="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA56,CaseTypeCol!$A:$A,0)))</f>
@@ -15325,7 +15337,7 @@
         <v>148</v>
       </c>
       <c r="AI56" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="AJ56" s="6" t="str">
         <f>IF($AH56="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH56,CaseTypeCol!$A:$A,0)))</f>
@@ -15351,7 +15363,7 @@
         <v>148</v>
       </c>
       <c r="AP56" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="AQ56" s="6" t="str">
         <f>IF($AO56="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO56,CaseTypeCol!$A:$A,0)))</f>
@@ -15382,7 +15394,7 @@
         <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D57" t="s">
         <v>12</v>
@@ -15392,7 +15404,7 @@
         <v>org_user1_2</v>
       </c>
       <c r="F57" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G57" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -15439,7 +15451,7 @@
         <v>0</v>
       </c>
       <c r="R57" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="S57" t="s">
         <v>123</v>
@@ -15466,7 +15478,7 @@
         <v>142</v>
       </c>
       <c r="AB57" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC57" s="6" t="str">
         <f>IF($AA57="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA57,CaseTypeCol!$A:$A,0)))</f>
@@ -15512,7 +15524,7 @@
         <v>145</v>
       </c>
       <c r="AP57" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="AQ57" s="6" t="str">
         <f>IF($AO57="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO57,CaseTypeCol!$A:$A,0)))</f>
@@ -15543,7 +15555,7 @@
         <v>1</v>
       </c>
       <c r="C58" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="D58" t="s">
         <v>12</v>
@@ -15553,7 +15565,7 @@
         <v>org_user1_2</v>
       </c>
       <c r="F58" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G58" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -15600,7 +15612,7 @@
         <v>0</v>
       </c>
       <c r="R58" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="S58" t="s">
         <v>123</v>
@@ -15627,7 +15639,7 @@
         <v>142</v>
       </c>
       <c r="AB58" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC58" s="6" t="str">
         <f>IF($AA58="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA58,CaseTypeCol!$A:$A,0)))</f>
@@ -15673,7 +15685,7 @@
         <v>145</v>
       </c>
       <c r="AP58" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="AQ58" s="6" t="str">
         <f>IF($AO58="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO58,CaseTypeCol!$A:$A,0)))</f>
@@ -15704,7 +15716,7 @@
         <v>1</v>
       </c>
       <c r="C59" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="D59" t="s">
         <v>13</v>
@@ -15714,7 +15726,7 @@
         <v>org_user1_3</v>
       </c>
       <c r="F59" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G59" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -15761,7 +15773,7 @@
         <v>0</v>
       </c>
       <c r="R59" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="S59" t="s">
         <v>119</v>
@@ -15788,7 +15800,7 @@
         <v>142</v>
       </c>
       <c r="AB59" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC59" s="6" t="str">
         <f>IF($AA59="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA59,CaseTypeCol!$A:$A,0)))</f>
@@ -15834,7 +15846,7 @@
         <v>151</v>
       </c>
       <c r="AP59" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="AQ59" s="6" t="str">
         <f>IF($AO59="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO59,CaseTypeCol!$A:$A,0)))</f>
@@ -15865,7 +15877,7 @@
         <v>1</v>
       </c>
       <c r="C60" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D60" t="s">
         <v>22</v>
@@ -15875,7 +15887,7 @@
         <v>org_user3_1</v>
       </c>
       <c r="F60" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G60" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -15922,7 +15934,7 @@
         <v>0</v>
       </c>
       <c r="R60" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S60" t="s">
         <v>119</v>
@@ -15949,7 +15961,7 @@
         <v>142</v>
       </c>
       <c r="AB60" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC60" s="6" t="str">
         <f>IF($AA60="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA60,CaseTypeCol!$A:$A,0)))</f>
@@ -15972,7 +15984,7 @@
         <v>0</v>
       </c>
       <c r="AI60" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ60" s="6" t="str">
         <f>IF($AH60="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH60,CaseTypeCol!$A:$A,0)))</f>
@@ -16023,7 +16035,7 @@
         <v>1</v>
       </c>
       <c r="C61" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="D61" t="s">
         <v>24</v>
@@ -16033,7 +16045,7 @@
         <v>org_user3_2</v>
       </c>
       <c r="F61" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G61" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -16080,7 +16092,7 @@
         <v>0</v>
       </c>
       <c r="R61" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S61" t="s">
         <v>119</v>
@@ -16107,7 +16119,7 @@
         <v>142</v>
       </c>
       <c r="AB61" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC61" s="6" t="str">
         <f>IF($AA61="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA61,CaseTypeCol!$A:$A,0)))</f>
@@ -16130,7 +16142,7 @@
         <v>0</v>
       </c>
       <c r="AI61" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ61" s="6" t="str">
         <f>IF($AH61="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH61,CaseTypeCol!$A:$A,0)))</f>
@@ -16181,7 +16193,7 @@
         <v>1</v>
       </c>
       <c r="C62" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="D62" t="s">
         <v>25</v>
@@ -16191,7 +16203,7 @@
         <v>org_user3_3</v>
       </c>
       <c r="F62" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G62" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -16238,7 +16250,7 @@
         <v>0</v>
       </c>
       <c r="R62" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S62" t="s">
         <v>119</v>
@@ -16265,7 +16277,7 @@
         <v>142</v>
       </c>
       <c r="AB62" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC62" s="6" t="str">
         <f>IF($AA62="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA62,CaseTypeCol!$A:$A,0)))</f>
@@ -16288,7 +16300,7 @@
         <v>0</v>
       </c>
       <c r="AI62" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ62" s="6" t="str">
         <f>IF($AH62="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH62,CaseTypeCol!$A:$A,0)))</f>
@@ -16339,7 +16351,7 @@
         <v>1</v>
       </c>
       <c r="C63" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="D63" t="s">
         <v>26</v>
@@ -16349,7 +16361,7 @@
         <v>org_user3_4</v>
       </c>
       <c r="F63" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G63" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -16396,7 +16408,7 @@
         <v>0</v>
       </c>
       <c r="R63" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S63" t="s">
         <v>119</v>
@@ -16423,7 +16435,7 @@
         <v>142</v>
       </c>
       <c r="AB63" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC63" s="6" t="str">
         <f>IF($AA63="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA63,CaseTypeCol!$A:$A,0)))</f>
@@ -16446,7 +16458,7 @@
         <v>0</v>
       </c>
       <c r="AI63" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ63" s="6" t="str">
         <f>IF($AH63="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH63,CaseTypeCol!$A:$A,0)))</f>
@@ -16497,7 +16509,7 @@
         <v>1</v>
       </c>
       <c r="C64" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="D64" t="s">
         <v>28</v>
@@ -16507,7 +16519,7 @@
         <v>org_user4_1</v>
       </c>
       <c r="F64" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G64" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -16554,7 +16566,7 @@
         <v>0</v>
       </c>
       <c r="R64" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="S64" t="s">
         <v>119</v>
@@ -16581,7 +16593,7 @@
         <v>142</v>
       </c>
       <c r="AB64" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC64" s="6" t="str">
         <f>IF($AA64="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA64,CaseTypeCol!$A:$A,0)))</f>
@@ -16604,7 +16616,7 @@
         <v>0</v>
       </c>
       <c r="AI64" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ64" s="6" t="str">
         <f>IF($AH64="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH64,CaseTypeCol!$A:$A,0)))</f>
@@ -16627,7 +16639,7 @@
         <v>1</v>
       </c>
       <c r="AP64" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="AQ64" s="6" t="str">
         <f>IF($AO64="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO64,CaseTypeCol!$A:$A,0)))</f>
@@ -16658,7 +16670,7 @@
         <v>1</v>
       </c>
       <c r="C65" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="D65" t="s">
         <v>30</v>
@@ -16668,7 +16680,7 @@
         <v>org_user4_2</v>
       </c>
       <c r="F65" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G65" s="19" t="b">
         <f t="shared" ca="1" si="0"/>
@@ -16715,7 +16727,7 @@
         <v>0</v>
       </c>
       <c r="R65" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="S65" t="s">
         <v>119</v>
@@ -16742,7 +16754,7 @@
         <v>142</v>
       </c>
       <c r="AB65" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC65" s="6" t="str">
         <f>IF($AA65="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA65,CaseTypeCol!$A:$A,0)))</f>
@@ -16765,7 +16777,7 @@
         <v>0</v>
       </c>
       <c r="AI65" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ65" s="6" t="str">
         <f>IF($AH65="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH65,CaseTypeCol!$A:$A,0)))</f>
@@ -16788,7 +16800,7 @@
         <v>1</v>
       </c>
       <c r="AP65" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="AQ65" s="6" t="str">
         <f>IF($AO65="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO65,CaseTypeCol!$A:$A,0)))</f>
@@ -16819,7 +16831,7 @@
         <v>1</v>
       </c>
       <c r="C66" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="D66" t="s">
         <v>31</v>
@@ -16829,7 +16841,7 @@
         <v>org_user4_3</v>
       </c>
       <c r="F66" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G66" s="19" t="b">
         <f t="shared" ref="G66:G75" ca="1" si="1">IF($F66="CREATE",$I66,IF($F66="CREATE_CASES",OR($I66,AND($K66,$L66,$O66,$P66,$AE66,AG66,$AL66,$AN66,$AS66,$AU66)),"TBD"))</f>
@@ -16876,7 +16888,7 @@
         <v>0</v>
       </c>
       <c r="R66" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="S66" t="s">
         <v>119</v>
@@ -16903,7 +16915,7 @@
         <v>142</v>
       </c>
       <c r="AB66" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC66" s="6" t="str">
         <f>IF($AA66="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA66,CaseTypeCol!$A:$A,0)))</f>
@@ -16926,7 +16938,7 @@
         <v>0</v>
       </c>
       <c r="AI66" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ66" s="6" t="str">
         <f>IF($AH66="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH66,CaseTypeCol!$A:$A,0)))</f>
@@ -16949,7 +16961,7 @@
         <v>1</v>
       </c>
       <c r="AP66" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="AQ66" s="6" t="str">
         <f>IF($AO66="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO66,CaseTypeCol!$A:$A,0)))</f>
@@ -16980,7 +16992,7 @@
         <v>1</v>
       </c>
       <c r="C67" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="D67" t="s">
         <v>32</v>
@@ -16990,7 +17002,7 @@
         <v>org_user4_4</v>
       </c>
       <c r="F67" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G67" s="19" t="b">
         <f t="shared" ca="1" si="1"/>
@@ -17037,7 +17049,7 @@
         <v>0</v>
       </c>
       <c r="R67" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="S67" t="s">
         <v>119</v>
@@ -17064,7 +17076,7 @@
         <v>142</v>
       </c>
       <c r="AB67" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC67" s="6" t="str">
         <f>IF($AA67="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA67,CaseTypeCol!$A:$A,0)))</f>
@@ -17087,7 +17099,7 @@
         <v>0</v>
       </c>
       <c r="AI67" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ67" s="6" t="str">
         <f>IF($AH67="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH67,CaseTypeCol!$A:$A,0)))</f>
@@ -17110,7 +17122,7 @@
         <v>1</v>
       </c>
       <c r="AP67" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="AQ67" s="6" t="str">
         <f>IF($AO67="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO67,CaseTypeCol!$A:$A,0)))</f>
@@ -17141,7 +17153,7 @@
         <v>1</v>
       </c>
       <c r="C68" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="D68" t="s">
         <v>34</v>
@@ -17151,7 +17163,7 @@
         <v>org_user5_1</v>
       </c>
       <c r="F68" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G68" s="19" t="b">
         <f t="shared" ca="1" si="1"/>
@@ -17198,7 +17210,7 @@
         <v>0</v>
       </c>
       <c r="R68" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="S68" t="s">
         <v>119</v>
@@ -17225,7 +17237,7 @@
         <v>142</v>
       </c>
       <c r="AB68" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC68" s="6" t="str">
         <f>IF($AA68="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA68,CaseTypeCol!$A:$A,0)))</f>
@@ -17248,7 +17260,7 @@
         <v>0</v>
       </c>
       <c r="AI68" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ68" s="6" t="str">
         <f>IF($AH68="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH68,CaseTypeCol!$A:$A,0)))</f>
@@ -17271,7 +17283,7 @@
         <v>1</v>
       </c>
       <c r="AP68" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="AQ68" s="6" t="str">
         <f>IF($AO68="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO68,CaseTypeCol!$A:$A,0)))</f>
@@ -17302,7 +17314,7 @@
         <v>1</v>
       </c>
       <c r="C69" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="D69" t="s">
         <v>36</v>
@@ -17312,7 +17324,7 @@
         <v>org_user5_2</v>
       </c>
       <c r="F69" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G69" s="19" t="b">
         <f t="shared" ca="1" si="1"/>
@@ -17359,7 +17371,7 @@
         <v>0</v>
       </c>
       <c r="R69" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="S69" t="s">
         <v>119</v>
@@ -17386,7 +17398,7 @@
         <v>142</v>
       </c>
       <c r="AB69" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC69" s="6" t="str">
         <f>IF($AA69="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA69,CaseTypeCol!$A:$A,0)))</f>
@@ -17409,7 +17421,7 @@
         <v>0</v>
       </c>
       <c r="AI69" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ69" s="6" t="str">
         <f>IF($AH69="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH69,CaseTypeCol!$A:$A,0)))</f>
@@ -17432,7 +17444,7 @@
         <v>1</v>
       </c>
       <c r="AP69" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="AQ69" s="6" t="str">
         <f>IF($AO69="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO69,CaseTypeCol!$A:$A,0)))</f>
@@ -17463,7 +17475,7 @@
         <v>1</v>
       </c>
       <c r="C70" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="D70" t="s">
         <v>37</v>
@@ -17473,7 +17485,7 @@
         <v>org_user5_3</v>
       </c>
       <c r="F70" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G70" s="19" t="b">
         <f t="shared" ca="1" si="1"/>
@@ -17520,7 +17532,7 @@
         <v>0</v>
       </c>
       <c r="R70" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="S70" t="s">
         <v>119</v>
@@ -17547,7 +17559,7 @@
         <v>142</v>
       </c>
       <c r="AB70" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC70" s="6" t="str">
         <f>IF($AA70="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA70,CaseTypeCol!$A:$A,0)))</f>
@@ -17570,7 +17582,7 @@
         <v>0</v>
       </c>
       <c r="AI70" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ70" s="6" t="str">
         <f>IF($AH70="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH70,CaseTypeCol!$A:$A,0)))</f>
@@ -17593,7 +17605,7 @@
         <v>1</v>
       </c>
       <c r="AP70" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="AQ70" s="6" t="str">
         <f>IF($AO70="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO70,CaseTypeCol!$A:$A,0)))</f>
@@ -17624,7 +17636,7 @@
         <v>1</v>
       </c>
       <c r="C71" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="D71" t="s">
         <v>38</v>
@@ -17634,7 +17646,7 @@
         <v>org_user5_4</v>
       </c>
       <c r="F71" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G71" s="19" t="b">
         <f t="shared" ca="1" si="1"/>
@@ -17681,7 +17693,7 @@
         <v>0</v>
       </c>
       <c r="R71" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="S71" t="s">
         <v>119</v>
@@ -17708,7 +17720,7 @@
         <v>142</v>
       </c>
       <c r="AB71" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC71" s="6" t="str">
         <f>IF($AA71="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA71,CaseTypeCol!$A:$A,0)))</f>
@@ -17731,7 +17743,7 @@
         <v>0</v>
       </c>
       <c r="AI71" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ71" s="6" t="str">
         <f>IF($AH71="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH71,CaseTypeCol!$A:$A,0)))</f>
@@ -17754,7 +17766,7 @@
         <v>1</v>
       </c>
       <c r="AP71" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="AQ71" s="6" t="str">
         <f>IF($AO71="","",INDEX(CaseTypeCol!$G:$G,MATCH($AO71,CaseTypeCol!$A:$A,0)))</f>
@@ -17785,7 +17797,7 @@
         <v>1</v>
       </c>
       <c r="C72" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="D72" t="s">
         <v>16</v>
@@ -17795,7 +17807,7 @@
         <v>org_user2_1</v>
       </c>
       <c r="F72" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G72" s="19" t="b">
         <f t="shared" ca="1" si="1"/>
@@ -17842,7 +17854,7 @@
         <v>0</v>
       </c>
       <c r="R72" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S72" t="s">
         <v>119</v>
@@ -17869,7 +17881,7 @@
         <v>142</v>
       </c>
       <c r="AB72" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC72" s="6" t="str">
         <f>IF($AA72="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA72,CaseTypeCol!$A:$A,0)))</f>
@@ -17892,7 +17904,7 @@
         <v>0</v>
       </c>
       <c r="AI72" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ72" s="6" t="str">
         <f>IF($AH72="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH72,CaseTypeCol!$A:$A,0)))</f>
@@ -17943,7 +17955,7 @@
         <v>1</v>
       </c>
       <c r="C73" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="D73" t="s">
         <v>18</v>
@@ -17953,7 +17965,7 @@
         <v>org_user2_2</v>
       </c>
       <c r="F73" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G73" s="19" t="b">
         <f t="shared" ca="1" si="1"/>
@@ -18000,7 +18012,7 @@
         <v>0</v>
       </c>
       <c r="R73" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="S73" t="s">
         <v>123</v>
@@ -18027,7 +18039,7 @@
         <v>142</v>
       </c>
       <c r="AB73" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC73" s="6" t="str">
         <f>IF($AA73="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA73,CaseTypeCol!$A:$A,0)))</f>
@@ -18050,7 +18062,7 @@
         <v>0</v>
       </c>
       <c r="AI73" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ73" s="6" t="str">
         <f>IF($AH73="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH73,CaseTypeCol!$A:$A,0)))</f>
@@ -18101,7 +18113,7 @@
         <v>1</v>
       </c>
       <c r="C74" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="D74" t="s">
         <v>19</v>
@@ -18111,7 +18123,7 @@
         <v>org_user2_3</v>
       </c>
       <c r="F74" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G74" s="19" t="b">
         <f t="shared" ca="1" si="1"/>
@@ -18158,7 +18170,7 @@
         <v>0</v>
       </c>
       <c r="R74" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="S74" t="s">
         <v>119</v>
@@ -18185,7 +18197,7 @@
         <v>142</v>
       </c>
       <c r="AB74" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC74" s="6" t="str">
         <f>IF($AA74="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA74,CaseTypeCol!$A:$A,0)))</f>
@@ -18208,7 +18220,7 @@
         <v>0</v>
       </c>
       <c r="AI74" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ74" s="6" t="str">
         <f>IF($AH74="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH74,CaseTypeCol!$A:$A,0)))</f>
@@ -18259,7 +18271,7 @@
         <v>1</v>
       </c>
       <c r="C75" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="D75" t="s">
         <v>20</v>
@@ -18269,7 +18281,7 @@
         <v>org_user2_4</v>
       </c>
       <c r="F75" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G75" s="19" t="b">
         <f t="shared" ca="1" si="1"/>
@@ -18316,7 +18328,7 @@
         <v>0</v>
       </c>
       <c r="R75" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="S75" t="s">
         <v>119</v>
@@ -18343,7 +18355,7 @@
         <v>142</v>
       </c>
       <c r="AB75" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AC75" s="6" t="str">
         <f>IF($AA75="","",INDEX(CaseTypeCol!$G:$G,MATCH($AA75,CaseTypeCol!$A:$A,0)))</f>
@@ -18366,7 +18378,7 @@
         <v>0</v>
       </c>
       <c r="AI75" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AJ75" s="6" t="str">
         <f>IF($AH75="","",INDEX(CaseTypeCol!$G:$G,MATCH($AH75,CaseTypeCol!$A:$A,0)))</f>
@@ -18458,19 +18470,19 @@
         <v>2</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>4</v>
@@ -18479,16 +18491,16 @@
         <v>5</v>
       </c>
       <c r="J1" s="7" t="s">
+        <v>558</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>560</v>
+      </c>
+      <c r="L1" s="7" t="s">
         <v>559</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="M1" s="8" t="s">
         <v>561</v>
-      </c>
-      <c r="L1" s="7" t="s">
-        <v>560</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>562</v>
       </c>
       <c r="N1" s="7" t="s">
         <v>6</v>
@@ -18506,16 +18518,16 @@
         <v>41</v>
       </c>
       <c r="S1" s="8" t="s">
+        <v>562</v>
+      </c>
+      <c r="T1" s="4" t="s">
         <v>563</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="U1" s="8" t="s">
         <v>564</v>
       </c>
-      <c r="U1" s="8" t="s">
-        <v>565</v>
-      </c>
       <c r="V1" s="8" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
@@ -19312,13 +19324,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>3</v>
@@ -19330,16 +19342,16 @@
         <v>5</v>
       </c>
       <c r="I1" s="7" t="s">
+        <v>558</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>560</v>
+      </c>
+      <c r="K1" s="7" t="s">
         <v>559</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="L1" s="8" t="s">
         <v>561</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>560</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>562</v>
       </c>
       <c r="M1" s="7" t="s">
         <v>6</v>
@@ -19354,25 +19366,25 @@
         <v>9</v>
       </c>
       <c r="Q1" s="8" t="s">
+        <v>568</v>
+      </c>
+      <c r="R1" s="8" t="s">
         <v>569</v>
       </c>
-      <c r="R1" s="8" t="s">
-        <v>570</v>
-      </c>
       <c r="S1" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="T1" s="8" t="s">
         <v>564</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="U1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="V1" s="8" t="s">
         <v>565</v>
       </c>
-      <c r="U1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="V1" s="8" t="s">
-        <v>566</v>
-      </c>
       <c r="W1" s="15" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
@@ -20385,13 +20397,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="D1" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -20412,24 +20424,24 @@
         <v>491</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="M1" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>569</v>
       </c>
-      <c r="N1" s="3" t="s">
-        <v>570</v>
-      </c>
       <c r="O1" s="7" t="s">
         <v>1</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
@@ -20521,13 +20533,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="D1" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -20548,18 +20560,18 @@
         <v>491</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="M1" t="s">
         <v>41</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
@@ -20637,7 +20649,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>441</v>
@@ -20655,27 +20667,27 @@
         <v>41</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="I1" s="5" t="s">
+        <v>671</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>672</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
+        <v>718</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>673</v>
       </c>
-      <c r="K1" s="5" t="s">
-        <v>719</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>674</v>
-      </c>
       <c r="M1" s="17" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B2" t="s">
         <v>443</v>
@@ -20691,7 +20703,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>552</v>
+        <v>785</v>
       </c>
       <c r="G2" t="s">
         <v>43</v>
@@ -20739,7 +20751,7 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>553</v>
+        <v>786</v>
       </c>
       <c r="G3" t="s">
         <v>43</v>
@@ -20774,10 +20786,10 @@
         <v>446</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" si="0"/>
@@ -20787,7 +20799,7 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>721</v>
+        <v>787</v>
       </c>
       <c r="G4" t="s">
         <v>43</v>
@@ -20835,7 +20847,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>554</v>
+        <v>788</v>
       </c>
       <c r="G5" t="s">
         <v>43</v>
@@ -20883,7 +20895,7 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>554</v>
+        <v>788</v>
       </c>
       <c r="G6" t="s">
         <v>46</v>
@@ -20931,7 +20943,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>554</v>
+        <v>788</v>
       </c>
       <c r="G7" t="s">
         <v>49</v>
@@ -20979,7 +20991,7 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>554</v>
+        <v>788</v>
       </c>
       <c r="G8" t="s">
         <v>52</v>
@@ -21027,7 +21039,7 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>554</v>
+        <v>788</v>
       </c>
       <c r="G9" t="s">
         <v>55</v>
@@ -21075,7 +21087,7 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G10" t="s">
         <v>43</v>
@@ -21123,7 +21135,7 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G11" t="s">
         <v>43</v>
@@ -21171,7 +21183,7 @@
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G12" t="s">
         <v>43</v>
@@ -21219,7 +21231,7 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G13" t="s">
         <v>43</v>
@@ -21267,7 +21279,7 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G14" t="s">
         <v>46</v>
@@ -21315,7 +21327,7 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G15" t="s">
         <v>46</v>
@@ -21363,7 +21375,7 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G16" t="s">
         <v>46</v>
@@ -21411,7 +21423,7 @@
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G17" t="s">
         <v>46</v>
@@ -21459,7 +21471,7 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G18" t="s">
         <v>49</v>
@@ -21507,7 +21519,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G19" t="s">
         <v>49</v>
@@ -21555,7 +21567,7 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G20" t="s">
         <v>49</v>
@@ -21603,7 +21615,7 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G21" t="s">
         <v>49</v>
@@ -21651,7 +21663,7 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G22" t="s">
         <v>52</v>
@@ -21699,7 +21711,7 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G23" t="s">
         <v>52</v>
@@ -21747,7 +21759,7 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G24" t="s">
         <v>52</v>
@@ -21795,7 +21807,7 @@
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G25" t="s">
         <v>52</v>
@@ -21843,7 +21855,7 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G26" t="s">
         <v>55</v>
@@ -21891,7 +21903,7 @@
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G27" t="s">
         <v>55</v>
@@ -21939,7 +21951,7 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G28" t="s">
         <v>55</v>
@@ -21987,7 +21999,7 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>555</v>
+        <v>789</v>
       </c>
       <c r="G29" t="s">
         <v>55</v>
@@ -22048,13 +22060,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>441</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>492</v>
@@ -22069,7 +22081,7 @@
         <v>494</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>41</v>
@@ -22099,10 +22111,10 @@
         <v>45743.390918726589</v>
       </c>
       <c r="G2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="H2" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="I2" s="6" t="str">
         <f>INDEX(User!$D:$D,MATCH($H2,User!$A:$A,0))</f>
@@ -22121,10 +22133,10 @@
         <v>497</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="D3" s="6" t="str">
         <f t="shared" ref="D3:D28" si="0">LEFT($C3,LEN($C3)-9)</f>
@@ -22137,7 +22149,7 @@
         <v>45743.390918741461</v>
       </c>
       <c r="G3" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="H3" t="s">
         <v>444</v>
@@ -22175,7 +22187,7 @@
         <v>45743.390918746562</v>
       </c>
       <c r="G4" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="H4" t="s">
         <v>444</v>
@@ -22213,7 +22225,7 @@
         <v>45743.390918763551</v>
       </c>
       <c r="G5" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="H5" t="s">
         <v>444</v>
@@ -22251,7 +22263,7 @@
         <v>45743.390918772537</v>
       </c>
       <c r="G6" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="H6" t="s">
         <v>444</v>
@@ -22289,7 +22301,7 @@
         <v>45743.390918781181</v>
       </c>
       <c r="G7" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="H7" t="s">
         <v>444</v>
@@ -22327,7 +22339,7 @@
         <v>45743.3909187889</v>
       </c>
       <c r="G8" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="H8" t="s">
         <v>444</v>
@@ -22365,7 +22377,7 @@
         <v>45743.390918796598</v>
       </c>
       <c r="G9" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H9" t="s">
         <v>444</v>
@@ -22403,7 +22415,7 @@
         <v>45743.390918801953</v>
       </c>
       <c r="G10" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H10" t="s">
         <v>444</v>
@@ -22441,7 +22453,7 @@
         <v>45743.390918807163</v>
       </c>
       <c r="G11" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H11" t="s">
         <v>444</v>
@@ -22479,7 +22491,7 @@
         <v>45743.3909188123</v>
       </c>
       <c r="G12" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H12" t="s">
         <v>444</v>
@@ -22517,7 +22529,7 @@
         <v>45743.390918817633</v>
       </c>
       <c r="G13" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H13" t="s">
         <v>444</v>
@@ -22555,7 +22567,7 @@
         <v>45743.390918822908</v>
       </c>
       <c r="G14" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H14" t="s">
         <v>444</v>
@@ -22593,7 +22605,7 @@
         <v>45743.390918828743</v>
       </c>
       <c r="G15" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H15" t="s">
         <v>444</v>
@@ -22631,7 +22643,7 @@
         <v>45743.390918834302</v>
       </c>
       <c r="G16" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H16" t="s">
         <v>444</v>
@@ -22669,7 +22681,7 @@
         <v>45743.390918839839</v>
       </c>
       <c r="G17" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H17" t="s">
         <v>444</v>
@@ -22707,7 +22719,7 @@
         <v>45743.390918845187</v>
       </c>
       <c r="G18" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H18" t="s">
         <v>444</v>
@@ -22745,7 +22757,7 @@
         <v>45743.390918851088</v>
       </c>
       <c r="G19" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H19" t="s">
         <v>444</v>
@@ -22783,7 +22795,7 @@
         <v>45743.39091885696</v>
       </c>
       <c r="G20" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H20" t="s">
         <v>444</v>
@@ -22821,7 +22833,7 @@
         <v>45743.390918862962</v>
       </c>
       <c r="G21" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H21" t="s">
         <v>444</v>
@@ -22859,7 +22871,7 @@
         <v>45743.390918868739</v>
       </c>
       <c r="G22" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H22" t="s">
         <v>444</v>
@@ -22897,7 +22909,7 @@
         <v>45743.390918874728</v>
       </c>
       <c r="G23" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H23" t="s">
         <v>444</v>
@@ -22935,7 +22947,7 @@
         <v>45743.390918881109</v>
       </c>
       <c r="G24" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H24" t="s">
         <v>444</v>
@@ -22973,7 +22985,7 @@
         <v>45743.390918887373</v>
       </c>
       <c r="G25" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H25" t="s">
         <v>444</v>
@@ -23011,7 +23023,7 @@
         <v>45743.39091889358</v>
       </c>
       <c r="G26" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H26" t="s">
         <v>444</v>
@@ -23049,7 +23061,7 @@
         <v>45743.390918900091</v>
       </c>
       <c r="G27" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H27" t="s">
         <v>444</v>
@@ -23087,7 +23099,7 @@
         <v>45743.390918906553</v>
       </c>
       <c r="G28" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H28" t="s">
         <v>444</v>
@@ -23161,7 +23173,7 @@
         <v>549</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D2" t="s">
         <v>438</v>
@@ -23182,7 +23194,7 @@
         <v>549</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D3" t="s">
         <v>439</v>
@@ -23203,7 +23215,7 @@
         <v>549</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D4" t="s">
         <v>440</v>
@@ -23302,7 +23314,7 @@
         <v>424</v>
       </c>
       <c r="E2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -23329,7 +23341,7 @@
         <v>424</v>
       </c>
       <c r="E3" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="F3">
         <v>2</v>
@@ -23356,7 +23368,7 @@
         <v>424</v>
       </c>
       <c r="E4" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="F4">
         <v>3</v>
@@ -23383,7 +23395,7 @@
         <v>428</v>
       </c>
       <c r="E5" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -23410,7 +23422,7 @@
         <v>428</v>
       </c>
       <c r="E6" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="F6">
         <v>2</v>
@@ -23437,7 +23449,7 @@
         <v>428</v>
       </c>
       <c r="E7" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="F7">
         <v>3</v>
@@ -23464,7 +23476,7 @@
         <v>432</v>
       </c>
       <c r="E8" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -23491,7 +23503,7 @@
         <v>432</v>
       </c>
       <c r="E9" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="F9">
         <v>2</v>
@@ -23518,7 +23530,7 @@
         <v>432</v>
       </c>
       <c r="E10" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="F10">
         <v>3</v>
@@ -23558,7 +23570,7 @@
         <v>57</v>
       </c>
       <c r="C1" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -23566,7 +23578,7 @@
         <v>121</v>
       </c>
       <c r="B2" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -23574,7 +23586,7 @@
         <v>125</v>
       </c>
       <c r="B3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -23582,7 +23594,7 @@
         <v>129</v>
       </c>
       <c r="B4" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -23590,7 +23602,7 @@
         <v>133</v>
       </c>
       <c r="B5" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -23598,7 +23610,7 @@
         <v>137</v>
       </c>
       <c r="B6" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
   </sheetData>
@@ -23625,7 +23637,7 @@
         <v>57</v>
       </c>
       <c r="C1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -23633,10 +23645,10 @@
         <v>122</v>
       </c>
       <c r="B2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="C2" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -23644,10 +23656,10 @@
         <v>126</v>
       </c>
       <c r="B3" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="C3" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -23655,10 +23667,10 @@
         <v>130</v>
       </c>
       <c r="B4" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C4" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -23666,10 +23678,10 @@
         <v>134</v>
       </c>
       <c r="B5" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C5" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -23677,10 +23689,10 @@
         <v>138</v>
       </c>
       <c r="B6" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="C6" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
   </sheetData>
@@ -23718,7 +23730,7 @@
         <v>115</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>116</v>
@@ -23727,7 +23739,7 @@
         <v>117</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>118</v>

</xml_diff>

<commit_message>
test: casedb.integration.case_access initial genetic_reads and seq columns ref data added test: casedb.unit.case_create_seq created
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_access/test_casedb_case_access.xlsx
+++ b/test/casedb/integration/case_access/test_casedb_case_access.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_access\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A61D31B2-B840-4A5B-BB17-403CEBADC04A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8267D924-D855-4E1E-B377-AF12D20D5D6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3552" yWindow="3552" windowWidth="30960" windowHeight="12120" tabRatio="913" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3456" yWindow="3456" windowWidth="30960" windowHeight="12120" tabRatio="913" firstSheet="3" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Organization" sheetId="17" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2143" uniqueCount="790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2270" uniqueCount="851">
   <si>
     <t>id</t>
   </si>
@@ -2451,6 +2451,189 @@
   </si>
   <si>
     <t>["CASEDB_ORG_USER"]</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-ce77-1fe4-e1e92fc9b431</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-2b6d-f669-ec9d41256fd6</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-81c8-4fce-c4ca38509c66</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>dim4</t>
+  </si>
+  <si>
+    <t>GENETIC_READS</t>
+  </si>
+  <si>
+    <t>GENETIC_SEQUENCE</t>
+  </si>
+  <si>
+    <t>dim4_1_genetic_reads</t>
+  </si>
+  <si>
+    <t>dim4_2_genetic_sequence</t>
+  </si>
+  <si>
+    <t>4_1</t>
+  </si>
+  <si>
+    <t>4_2</t>
+  </si>
+  <si>
+    <t>case_type1_dim4_1_genetic_reads</t>
+  </si>
+  <si>
+    <t>case_type1_dim4_2_genetic_sequence</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-8a7b-7c82-adf57928fa72</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-180c-d818-10c8aed7f4c5</t>
+  </si>
+  <si>
+    <t>case_type2_dim4_1_genetic_reads</t>
+  </si>
+  <si>
+    <t>case_type2_dim4_2_genetic_sequence</t>
+  </si>
+  <si>
+    <t>case_type3_dim4_1_genetic_reads</t>
+  </si>
+  <si>
+    <t>case_type3_dim4_2_genetic_sequence</t>
+  </si>
+  <si>
+    <t>case_type4_dim4_1_genetic_reads</t>
+  </si>
+  <si>
+    <t>case_type4_dim4_2_genetic_sequence</t>
+  </si>
+  <si>
+    <t>case_type5_dim4_1_genetic_reads</t>
+  </si>
+  <si>
+    <t>case_type5_dim4_2_genetic_sequence</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-991b-7f4f-683a81051e65</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-e6df-c1d5-00f9f7cf16f3</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-9857-f307-13b9f5a150d1</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-9436-d94c-4e4ee8856951</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-af63-b674-d9ae3c5f0a08</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-0ab7-4323-aa6aedd4c1cc</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-423c-9007-26ece8e894c8</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-10ef-cde6-dd672b6f1342</t>
+  </si>
+  <si>
+    <t>case_type_col_set1_4_1</t>
+  </si>
+  <si>
+    <t>case_type_col_set1_4_2</t>
+  </si>
+  <si>
+    <t>case_type_col_set2_4_1</t>
+  </si>
+  <si>
+    <t>case_type_col_set2_4_2</t>
+  </si>
+  <si>
+    <t>case_type_col_set3_4_1</t>
+  </si>
+  <si>
+    <t>case_type_col_set3_4_2</t>
+  </si>
+  <si>
+    <t>case_type_col_set4_4_1</t>
+  </si>
+  <si>
+    <t>case_type_col_set4_4_2</t>
+  </si>
+  <si>
+    <t>case_type_col_set5_4_1</t>
+  </si>
+  <si>
+    <t>case_type_col_set5_4_2</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-b12e-cfb7-f4c9c62c8fc6</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-8d4b-cfe4-957f28881a67</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-47cd-cf12-b0da18fd2588</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-eba4-fbce-8c553ccd262a</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-9918-33cd-c862ad905516</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-c7d8-6072-9a0d42887e0f</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-8f84-5827-8c0fedea4c3d</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-2ec3-f155-116a4b0fe44d</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-afc6-e887-8b50ddfd6962</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-869e-506b-15ae88b8c755</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-e0db-f17c-d2593ac2e0ae</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-6c7f-60e3-cac3235d66c9</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-77b4-7251-1482abc4c1de</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-0b05-7141-2f121d4fad38</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-f8d6-367c-7cb258e6eb59</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-134a-0192-ae64f09437ad</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-c767-4e72-46e1afc2b6b3</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-1d66-cdd5-209407b1eac7</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-9737-0c0b-2bfc6e57a6ce</t>
+  </si>
+  <si>
+    <t>019a8753-bed9-c236-1097-01c862c1858d</t>
   </si>
 </sst>
 </file>
@@ -3960,7 +4143,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:T46"/>
+  <dimension ref="A1:T56"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
@@ -4202,16 +4385,16 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>168</v>
+        <v>804</v>
       </c>
       <c r="B11" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D11" t="s">
-        <v>333</v>
+        <v>791</v>
       </c>
       <c r="G11" t="s">
-        <v>352</v>
+        <v>801</v>
       </c>
       <c r="T11" t="s">
         <v>335</v>
@@ -4219,16 +4402,16 @@
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>171</v>
+        <v>803</v>
       </c>
       <c r="B12" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D12" t="s">
-        <v>336</v>
+        <v>790</v>
       </c>
       <c r="G12" t="s">
-        <v>353</v>
+        <v>802</v>
       </c>
       <c r="T12" t="s">
         <v>335</v>
@@ -4236,16 +4419,16 @@
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B13" t="s">
         <v>123</v>
       </c>
       <c r="D13" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="G13" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="T13" t="s">
         <v>335</v>
@@ -4253,16 +4436,16 @@
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="B14" t="s">
         <v>123</v>
       </c>
       <c r="D14" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="G14" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="T14" t="s">
         <v>335</v>
@@ -4270,16 +4453,16 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="B15" t="s">
         <v>123</v>
       </c>
       <c r="D15" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="G15" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="T15" t="s">
         <v>335</v>
@@ -4287,16 +4470,16 @@
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="B16" t="s">
         <v>123</v>
       </c>
       <c r="D16" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="G16" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="T16" t="s">
         <v>335</v>
@@ -4304,16 +4487,16 @@
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="B17" t="s">
         <v>123</v>
       </c>
       <c r="D17" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="G17" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="T17" t="s">
         <v>335</v>
@@ -4321,16 +4504,16 @@
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B18" t="s">
         <v>123</v>
       </c>
       <c r="D18" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="G18" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="T18" t="s">
         <v>335</v>
@@ -4338,16 +4521,16 @@
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="B19" t="s">
         <v>123</v>
       </c>
       <c r="D19" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="G19" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="T19" t="s">
         <v>335</v>
@@ -4355,16 +4538,16 @@
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="B20" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D20" t="s">
-        <v>333</v>
+        <v>348</v>
       </c>
       <c r="G20" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="T20" t="s">
         <v>335</v>
@@ -4372,16 +4555,16 @@
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="B21" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D21" t="s">
-        <v>336</v>
+        <v>350</v>
       </c>
       <c r="G21" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="T21" t="s">
         <v>335</v>
@@ -4389,16 +4572,16 @@
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>200</v>
+        <v>820</v>
       </c>
       <c r="B22" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D22" t="s">
-        <v>338</v>
+        <v>791</v>
       </c>
       <c r="G22" t="s">
-        <v>363</v>
+        <v>805</v>
       </c>
       <c r="T22" t="s">
         <v>335</v>
@@ -4406,16 +4589,16 @@
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>203</v>
+        <v>819</v>
       </c>
       <c r="B23" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D23" t="s">
-        <v>340</v>
+        <v>790</v>
       </c>
       <c r="G23" t="s">
-        <v>364</v>
+        <v>806</v>
       </c>
       <c r="T23" t="s">
         <v>335</v>
@@ -4423,16 +4606,16 @@
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="B24" t="s">
         <v>127</v>
       </c>
       <c r="D24" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="G24" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="T24" t="s">
         <v>335</v>
@@ -4440,16 +4623,16 @@
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="B25" t="s">
         <v>127</v>
       </c>
       <c r="D25" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="G25" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="T25" t="s">
         <v>335</v>
@@ -4457,16 +4640,16 @@
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="B26" t="s">
         <v>127</v>
       </c>
       <c r="D26" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="G26" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="T26" t="s">
         <v>335</v>
@@ -4474,16 +4657,16 @@
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="B27" t="s">
         <v>127</v>
       </c>
       <c r="D27" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="G27" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="T27" t="s">
         <v>335</v>
@@ -4491,16 +4674,16 @@
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="B28" t="s">
         <v>127</v>
       </c>
       <c r="D28" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="G28" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="T28" t="s">
         <v>335</v>
@@ -4508,16 +4691,16 @@
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="B29" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D29" t="s">
-        <v>333</v>
+        <v>344</v>
       </c>
       <c r="G29" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="T29" t="s">
         <v>335</v>
@@ -4525,16 +4708,16 @@
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="B30" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D30" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="G30" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="T30" t="s">
         <v>335</v>
@@ -4542,16 +4725,16 @@
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="B31" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D31" t="s">
-        <v>338</v>
+        <v>348</v>
       </c>
       <c r="G31" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="T31" t="s">
         <v>335</v>
@@ -4559,16 +4742,16 @@
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="B32" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D32" t="s">
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="G32" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="T32" t="s">
         <v>335</v>
@@ -4576,16 +4759,16 @@
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>232</v>
+        <v>818</v>
       </c>
       <c r="B33" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="D33" t="s">
-        <v>342</v>
+        <v>791</v>
       </c>
       <c r="G33" t="s">
-        <v>374</v>
+        <v>807</v>
       </c>
       <c r="T33" t="s">
         <v>335</v>
@@ -4593,16 +4776,16 @@
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>235</v>
+        <v>817</v>
       </c>
       <c r="B34" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="D34" t="s">
-        <v>344</v>
+        <v>790</v>
       </c>
       <c r="G34" t="s">
-        <v>375</v>
+        <v>808</v>
       </c>
       <c r="T34" t="s">
         <v>335</v>
@@ -4610,16 +4793,16 @@
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>238</v>
+        <v>220</v>
       </c>
       <c r="B35" t="s">
         <v>131</v>
       </c>
       <c r="D35" t="s">
-        <v>346</v>
+        <v>333</v>
       </c>
       <c r="G35" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="T35" t="s">
         <v>335</v>
@@ -4627,16 +4810,16 @@
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="B36" t="s">
         <v>131</v>
       </c>
       <c r="D36" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="G36" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="T36" t="s">
         <v>335</v>
@@ -4644,16 +4827,16 @@
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>244</v>
+        <v>226</v>
       </c>
       <c r="B37" t="s">
         <v>131</v>
       </c>
       <c r="D37" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="G37" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="T37" t="s">
         <v>335</v>
@@ -4661,16 +4844,16 @@
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>246</v>
+        <v>229</v>
       </c>
       <c r="B38" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D38" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="G38" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="T38" t="s">
         <v>335</v>
@@ -4678,16 +4861,16 @@
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>249</v>
+        <v>232</v>
       </c>
       <c r="B39" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D39" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="G39" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="T39" t="s">
         <v>335</v>
@@ -4695,16 +4878,16 @@
     </row>
     <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>252</v>
+        <v>235</v>
       </c>
       <c r="B40" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D40" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="G40" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="T40" t="s">
         <v>335</v>
@@ -4712,16 +4895,16 @@
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>255</v>
+        <v>238</v>
       </c>
       <c r="B41" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D41" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="G41" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="T41" t="s">
         <v>335</v>
@@ -4729,16 +4912,16 @@
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>258</v>
+        <v>241</v>
       </c>
       <c r="B42" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D42" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="G42" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="T42" t="s">
         <v>335</v>
@@ -4746,16 +4929,16 @@
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>261</v>
+        <v>244</v>
       </c>
       <c r="B43" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D43" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="G43" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="T43" t="s">
         <v>335</v>
@@ -4763,16 +4946,16 @@
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>264</v>
+        <v>816</v>
       </c>
       <c r="B44" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="D44" t="s">
-        <v>346</v>
+        <v>791</v>
       </c>
       <c r="G44" t="s">
-        <v>385</v>
+        <v>809</v>
       </c>
       <c r="T44" t="s">
         <v>335</v>
@@ -4780,16 +4963,16 @@
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>267</v>
+        <v>815</v>
       </c>
       <c r="B45" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="D45" t="s">
-        <v>348</v>
+        <v>790</v>
       </c>
       <c r="G45" t="s">
-        <v>386</v>
+        <v>810</v>
       </c>
       <c r="T45" t="s">
         <v>335</v>
@@ -4797,18 +4980,188 @@
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>270</v>
+        <v>246</v>
       </c>
       <c r="B46" t="s">
         <v>135</v>
       </c>
       <c r="D46" t="s">
+        <v>333</v>
+      </c>
+      <c r="G46" t="s">
+        <v>379</v>
+      </c>
+      <c r="T46" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>249</v>
+      </c>
+      <c r="B47" t="s">
+        <v>135</v>
+      </c>
+      <c r="D47" t="s">
+        <v>336</v>
+      </c>
+      <c r="G47" t="s">
+        <v>380</v>
+      </c>
+      <c r="T47" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>252</v>
+      </c>
+      <c r="B48" t="s">
+        <v>135</v>
+      </c>
+      <c r="D48" t="s">
+        <v>338</v>
+      </c>
+      <c r="G48" t="s">
+        <v>381</v>
+      </c>
+      <c r="T48" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>255</v>
+      </c>
+      <c r="B49" t="s">
+        <v>135</v>
+      </c>
+      <c r="D49" t="s">
+        <v>340</v>
+      </c>
+      <c r="G49" t="s">
+        <v>382</v>
+      </c>
+      <c r="T49" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>258</v>
+      </c>
+      <c r="B50" t="s">
+        <v>135</v>
+      </c>
+      <c r="D50" t="s">
+        <v>342</v>
+      </c>
+      <c r="G50" t="s">
+        <v>383</v>
+      </c>
+      <c r="T50" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>261</v>
+      </c>
+      <c r="B51" t="s">
+        <v>135</v>
+      </c>
+      <c r="D51" t="s">
+        <v>344</v>
+      </c>
+      <c r="G51" t="s">
+        <v>384</v>
+      </c>
+      <c r="T51" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>264</v>
+      </c>
+      <c r="B52" t="s">
+        <v>135</v>
+      </c>
+      <c r="D52" t="s">
+        <v>346</v>
+      </c>
+      <c r="G52" t="s">
+        <v>385</v>
+      </c>
+      <c r="T52" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>267</v>
+      </c>
+      <c r="B53" t="s">
+        <v>135</v>
+      </c>
+      <c r="D53" t="s">
+        <v>348</v>
+      </c>
+      <c r="G53" t="s">
+        <v>386</v>
+      </c>
+      <c r="T53" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>270</v>
+      </c>
+      <c r="B54" t="s">
+        <v>135</v>
+      </c>
+      <c r="D54" t="s">
         <v>350</v>
       </c>
-      <c r="G46" t="s">
+      <c r="G54" t="s">
         <v>387</v>
       </c>
-      <c r="T46" t="s">
+      <c r="T54" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>814</v>
+      </c>
+      <c r="B55" t="s">
+        <v>119</v>
+      </c>
+      <c r="D55" t="s">
+        <v>791</v>
+      </c>
+      <c r="G55" t="s">
+        <v>811</v>
+      </c>
+      <c r="T55" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>813</v>
+      </c>
+      <c r="B56" t="s">
+        <v>119</v>
+      </c>
+      <c r="D56" t="s">
+        <v>790</v>
+      </c>
+      <c r="G56" t="s">
+        <v>812</v>
+      </c>
+      <c r="T56" t="s">
         <v>335</v>
       </c>
     </row>
@@ -4819,7 +5172,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
@@ -4938,408 +5291,519 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>839</v>
       </c>
       <c r="B11" t="s">
-        <v>280</v>
+        <v>821</v>
       </c>
       <c r="C11" t="s">
-        <v>280</v>
+        <v>821</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>170</v>
+        <v>840</v>
       </c>
       <c r="B12" t="s">
-        <v>281</v>
+        <v>822</v>
       </c>
       <c r="C12" t="s">
-        <v>281</v>
+        <v>822</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>173</v>
+        <v>66</v>
       </c>
       <c r="B13" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C13" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B14" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C14" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B16" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C16" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B17" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C17" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B18" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C18" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B19" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C19" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>68</v>
+        <v>188</v>
       </c>
       <c r="B20" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C20" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="B21" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C21" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>199</v>
+        <v>837</v>
       </c>
       <c r="B22" t="s">
-        <v>291</v>
+        <v>823</v>
       </c>
       <c r="C22" t="s">
-        <v>291</v>
+        <v>823</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>202</v>
+        <v>838</v>
       </c>
       <c r="B23" t="s">
-        <v>292</v>
+        <v>824</v>
       </c>
       <c r="C23" t="s">
-        <v>292</v>
+        <v>824</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>205</v>
+        <v>68</v>
       </c>
       <c r="B24" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="C24" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="B25" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="C25" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="B26" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="C26" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="B27" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="C27" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="B28" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="C28" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>70</v>
+        <v>208</v>
       </c>
       <c r="B29" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="C29" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="B30" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="C30" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="B31" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="C31" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="B32" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="C32" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>231</v>
+        <v>836</v>
       </c>
       <c r="B33" t="s">
-        <v>302</v>
+        <v>825</v>
       </c>
       <c r="C33" t="s">
-        <v>302</v>
+        <v>825</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>234</v>
+        <v>835</v>
       </c>
       <c r="B34" t="s">
-        <v>303</v>
+        <v>826</v>
       </c>
       <c r="C34" t="s">
-        <v>303</v>
+        <v>826</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>237</v>
+        <v>70</v>
       </c>
       <c r="B35" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="C35" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
       <c r="B36" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C36" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>243</v>
+        <v>225</v>
       </c>
       <c r="B37" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="C37" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>72</v>
+        <v>228</v>
       </c>
       <c r="B38" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="C38" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>248</v>
+        <v>231</v>
       </c>
       <c r="B39" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="C39" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>251</v>
+        <v>234</v>
       </c>
       <c r="B40" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="C40" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>254</v>
+        <v>237</v>
       </c>
       <c r="B41" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="C41" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>257</v>
+        <v>240</v>
       </c>
       <c r="B42" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="C42" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="B43" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="C43" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>263</v>
+        <v>834</v>
       </c>
       <c r="B44" t="s">
-        <v>313</v>
+        <v>827</v>
       </c>
       <c r="C44" t="s">
-        <v>313</v>
+        <v>827</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>266</v>
+        <v>833</v>
       </c>
       <c r="B45" t="s">
-        <v>314</v>
+        <v>828</v>
       </c>
       <c r="C45" t="s">
-        <v>314</v>
+        <v>828</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
+        <v>72</v>
+      </c>
+      <c r="B46" t="s">
+        <v>307</v>
+      </c>
+      <c r="C46" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>248</v>
+      </c>
+      <c r="B47" t="s">
+        <v>308</v>
+      </c>
+      <c r="C47" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>251</v>
+      </c>
+      <c r="B48" t="s">
+        <v>309</v>
+      </c>
+      <c r="C48" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>254</v>
+      </c>
+      <c r="B49" t="s">
+        <v>310</v>
+      </c>
+      <c r="C49" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>257</v>
+      </c>
+      <c r="B50" t="s">
+        <v>311</v>
+      </c>
+      <c r="C50" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>260</v>
+      </c>
+      <c r="B51" t="s">
+        <v>312</v>
+      </c>
+      <c r="C51" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>263</v>
+      </c>
+      <c r="B52" t="s">
+        <v>313</v>
+      </c>
+      <c r="C52" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>266</v>
+      </c>
+      <c r="B53" t="s">
+        <v>314</v>
+      </c>
+      <c r="C53" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
         <v>269</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B54" t="s">
         <v>315</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C54" t="s">
         <v>315</v>
       </c>
     </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>832</v>
+      </c>
+      <c r="B55" t="s">
+        <v>829</v>
+      </c>
+      <c r="C55" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>831</v>
+      </c>
+      <c r="B56" t="s">
+        <v>830</v>
+      </c>
+      <c r="C56" t="s">
+        <v>830</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="35.6640625" bestFit="1" customWidth="1"/>
@@ -5419,7 +5883,7 @@
         <v>case_type1_dim1_2_text</v>
       </c>
       <c r="H3" s="6" t="str">
-        <f t="shared" ref="H3:H46" si="0">$B3&amp;"|"&amp;$E3</f>
+        <f t="shared" ref="H3:H56" si="0">$B3&amp;"|"&amp;$E3</f>
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0195d18c-1cab-86f3-5faf-507bfa221cf6</v>
       </c>
     </row>
@@ -5586,830 +6050,1060 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>167</v>
+        <v>841</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>839</v>
       </c>
       <c r="C11" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B11,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set2_1_1</v>
+        <v>case_type_col_set1_4_1</v>
       </c>
       <c r="E11" t="s">
-        <v>168</v>
+        <v>804</v>
       </c>
       <c r="F11" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E11,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type2_dim1_1_text</v>
+        <v>case_type1_dim4_1_genetic_reads</v>
       </c>
       <c r="H11" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cc6-a324-3f72-222014292515|0195d18c-1cad-37c6-0826-9671f313fb2b</v>
+        <v>019a8753-bed9-afc6-e887-8b50ddfd6962|019a8753-bed9-180c-d818-10c8aed7f4c5</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>169</v>
+        <v>842</v>
       </c>
       <c r="B12" t="s">
-        <v>170</v>
+        <v>840</v>
       </c>
       <c r="C12" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B12,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set2_1_2</v>
+        <v>case_type_col_set1_4_2</v>
       </c>
       <c r="E12" t="s">
-        <v>171</v>
+        <v>803</v>
       </c>
       <c r="F12" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E12,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type2_dim1_2_text</v>
+        <v>case_type1_dim4_2_genetic_sequence</v>
       </c>
       <c r="H12" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cc7-243f-f4e7-3dbdfe691c71|0195d18c-1cad-5b48-8a72-25050cbf379e</v>
+        <v>019a8753-bed9-869e-506b-15ae88b8c755|019a8753-bed9-8a7b-7c82-adf57928fa72</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="B13" t="s">
-        <v>173</v>
+        <v>66</v>
       </c>
       <c r="C13" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B13,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set2_1_3</v>
+        <v>case_type_col_set2_1_1</v>
       </c>
       <c r="E13" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="F13" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E13,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type2_dim1_3_text</v>
+        <v>case_type2_dim1_1_text</v>
       </c>
       <c r="H13" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cc7-60b4-b4e6-8ff7fabb2b09|0195d18c-1cad-e18e-a87d-8af6760d00e1</v>
+        <v>0195d18c-1cc6-a324-3f72-222014292515|0195d18c-1cad-37c6-0826-9671f313fb2b</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B14" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C14" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B14,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set2_2_1</v>
+        <v>case_type_col_set2_1_2</v>
       </c>
       <c r="E14" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="F14" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E14,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type2_dim2_1_text</v>
+        <v>case_type2_dim1_2_text</v>
       </c>
       <c r="H14" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cc8-bcf2-c56f-04928f2e3635|0195d18c-1cad-9467-449f-6341c820b944</v>
+        <v>0195d18c-1cc7-243f-f4e7-3dbdfe691c71|0195d18c-1cad-5b48-8a72-25050cbf379e</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="B15" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C15" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B15,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set2_2_2</v>
+        <v>case_type_col_set2_1_3</v>
       </c>
       <c r="E15" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="F15" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E15,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type2_dim2_2_text</v>
+        <v>case_type2_dim1_3_text</v>
       </c>
       <c r="H15" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cc8-18f5-27a5-fd3874e6b78b|0195d18c-1cae-fcea-56fe-4577ada0491d</v>
+        <v>0195d18c-1cc7-60b4-b4e6-8ff7fabb2b09|0195d18c-1cad-e18e-a87d-8af6760d00e1</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="B16" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C16" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B16,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set2_2_3</v>
+        <v>case_type_col_set2_2_1</v>
       </c>
       <c r="E16" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="F16" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E16,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type2_dim2_3_text</v>
+        <v>case_type2_dim2_1_text</v>
       </c>
       <c r="H16" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cc8-5a76-0a72-16117b0a5a5e|0195d18c-1cae-cdba-00d9-e8405172259e</v>
+        <v>0195d18c-1cc8-bcf2-c56f-04928f2e3635|0195d18c-1cad-9467-449f-6341c820b944</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="B17" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="C17" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B17,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set2_3_1</v>
+        <v>case_type_col_set2_2_2</v>
       </c>
       <c r="E17" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="F17" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E17,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type2_dim3_1_text</v>
+        <v>case_type2_dim2_2_text</v>
       </c>
       <c r="H17" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cc9-7181-fd5b-078012e228f2|0195d18c-1cae-faa7-ac0d-22cce7d230ec</v>
+        <v>0195d18c-1cc8-18f5-27a5-fd3874e6b78b|0195d18c-1cae-fcea-56fe-4577ada0491d</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="B18" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="C18" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B18,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set2_3_2</v>
+        <v>case_type_col_set2_2_3</v>
       </c>
       <c r="E18" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="F18" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E18,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type2_dim3_2_text</v>
+        <v>case_type2_dim2_3_text</v>
       </c>
       <c r="H18" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cc9-c61f-4e7e-a00189d3cc75|0195d18c-1cae-45ab-ca21-9cee527b9482</v>
+        <v>0195d18c-1cc8-5a76-0a72-16117b0a5a5e|0195d18c-1cae-cdba-00d9-e8405172259e</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="B19" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C19" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B19,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set2_3_3</v>
+        <v>case_type_col_set2_3_1</v>
       </c>
       <c r="E19" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="F19" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E19,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type2_dim3_3_text</v>
+        <v>case_type2_dim3_1_text</v>
       </c>
       <c r="H19" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cca-878e-2110-0116e848541b|0195d18c-1caf-d364-c3b5-e73ba434270e</v>
+        <v>0195d18c-1cc9-7181-fd5b-078012e228f2|0195d18c-1cae-faa7-ac0d-22cce7d230ec</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B20" t="s">
-        <v>68</v>
+        <v>188</v>
       </c>
       <c r="C20" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B20,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set3_1_1</v>
+        <v>case_type_col_set2_3_2</v>
       </c>
       <c r="E20" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="F20" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E20,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type3_dim1_1_text</v>
+        <v>case_type2_dim3_2_text</v>
       </c>
       <c r="H20" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cca-26c0-66df-979380a43b16|0195d18c-1caf-b3af-f64e-bd18810c4521</v>
+        <v>0195d18c-1cc9-c61f-4e7e-a00189d3cc75|0195d18c-1cae-45ab-ca21-9cee527b9482</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="B21" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C21" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B21,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set3_1_2</v>
+        <v>case_type_col_set2_3_3</v>
       </c>
       <c r="E21" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="F21" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E21,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type3_dim1_2_text</v>
+        <v>case_type2_dim3_3_text</v>
       </c>
       <c r="H21" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1ccb-f06f-162f-a5dc745a5198|0195d18c-1caf-84ca-1737-a8f8788cd464</v>
+        <v>0195d18c-1cca-878e-2110-0116e848541b|0195d18c-1caf-d364-c3b5-e73ba434270e</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>198</v>
+        <v>843</v>
       </c>
       <c r="B22" t="s">
-        <v>199</v>
+        <v>837</v>
       </c>
       <c r="C22" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B22,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set3_1_3</v>
+        <v>case_type_col_set2_4_1</v>
       </c>
       <c r="E22" t="s">
-        <v>200</v>
+        <v>820</v>
       </c>
       <c r="F22" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E22,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type3_dim1_3_text</v>
+        <v>case_type2_dim4_1_genetic_reads</v>
       </c>
       <c r="H22" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1ccb-b068-d845-d61fb54721f1|0195d18c-1cb0-7655-a8bb-f656b1b8b72c</v>
+        <v>019a8753-bed9-8f84-5827-8c0fedea4c3d|019a8753-bed9-10ef-cde6-dd672b6f1342</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>201</v>
+        <v>844</v>
       </c>
       <c r="B23" t="s">
-        <v>202</v>
+        <v>838</v>
       </c>
       <c r="C23" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B23,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set3_2_1</v>
+        <v>case_type_col_set2_4_2</v>
       </c>
       <c r="E23" t="s">
-        <v>203</v>
+        <v>819</v>
       </c>
       <c r="F23" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E23,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type3_dim2_1_text</v>
+        <v>case_type2_dim4_2_genetic_sequence</v>
       </c>
       <c r="H23" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1ccc-f754-4a4f-89cdc532a3be|0195d18c-1cb0-4c24-e2e8-b92cfc74f7cc</v>
+        <v>019a8753-bed9-2ec3-f155-116a4b0fe44d|019a8753-bed9-423c-9007-26ece8e894c8</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="B24" t="s">
-        <v>205</v>
+        <v>68</v>
       </c>
       <c r="C24" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B24,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set3_2_2</v>
+        <v>case_type_col_set3_1_1</v>
       </c>
       <c r="E24" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="F24" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E24,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type3_dim2_2_text</v>
+        <v>case_type3_dim1_1_text</v>
       </c>
       <c r="H24" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1ccc-3f10-cc4e-636793b1e9dd|0195d18c-1cb0-8d34-e3f0-ab091b80ab8f</v>
+        <v>0195d18c-1cca-26c0-66df-979380a43b16|0195d18c-1caf-b3af-f64e-bd18810c4521</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="B25" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="C25" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B25,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set3_2_3</v>
+        <v>case_type_col_set3_1_2</v>
       </c>
       <c r="E25" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="F25" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E25,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type3_dim2_3_text</v>
+        <v>case_type3_dim1_2_text</v>
       </c>
       <c r="H25" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1ccd-3f53-ad72-f2d3c667b246|0195d18c-1cb0-db51-ed28-2a4481c5f1ac</v>
+        <v>0195d18c-1ccb-f06f-162f-a5dc745a5198|0195d18c-1caf-84ca-1737-a8f8788cd464</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="B26" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="C26" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B26,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set3_3_1</v>
+        <v>case_type_col_set3_1_3</v>
       </c>
       <c r="E26" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="F26" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E26,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type3_dim3_1_text</v>
+        <v>case_type3_dim1_3_text</v>
       </c>
       <c r="H26" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1ccd-d664-179c-a1a90c3c886c|0195d18c-1cb1-b5d5-ee26-96c6a9678489</v>
+        <v>0195d18c-1ccb-b068-d845-d61fb54721f1|0195d18c-1cb0-7655-a8bb-f656b1b8b72c</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="B27" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="C27" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B27,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set3_3_2</v>
+        <v>case_type_col_set3_2_1</v>
       </c>
       <c r="E27" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="F27" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E27,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type3_dim3_2_text</v>
+        <v>case_type3_dim2_1_text</v>
       </c>
       <c r="H27" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1ccd-12ae-b807-5b71d1b4e1f1|0195d18c-1cb1-f7bb-aa5b-6f2c6f5d3696</v>
+        <v>0195d18c-1ccc-f754-4a4f-89cdc532a3be|0195d18c-1cb0-4c24-e2e8-b92cfc74f7cc</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="B28" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="C28" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B28,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set3_3_3</v>
+        <v>case_type_col_set3_2_2</v>
       </c>
       <c r="E28" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="F28" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E28,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type3_dim3_3_text</v>
+        <v>case_type3_dim2_2_text</v>
       </c>
       <c r="H28" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cce-3516-017e-cf05c78d4433|0195d18c-1cb1-2097-fae7-ffcb7e109be5</v>
+        <v>0195d18c-1ccc-3f10-cc4e-636793b1e9dd|0195d18c-1cb0-8d34-e3f0-ab091b80ab8f</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="B29" t="s">
-        <v>70</v>
+        <v>208</v>
       </c>
       <c r="C29" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B29,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set4_1_1</v>
+        <v>case_type_col_set3_2_3</v>
       </c>
       <c r="E29" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="F29" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E29,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type4_dim1_1_text</v>
+        <v>case_type3_dim2_3_text</v>
       </c>
       <c r="H29" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cce-585d-e95b-79f3fbfdd12b|0195d18c-1cb2-95e6-139d-1dbe7ffdd3d0</v>
+        <v>0195d18c-1ccd-3f53-ad72-f2d3c667b246|0195d18c-1cb0-db51-ed28-2a4481c5f1ac</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="B30" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="C30" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B30,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set4_1_2</v>
+        <v>case_type_col_set3_3_1</v>
       </c>
       <c r="E30" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="F30" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E30,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type4_dim1_2_text</v>
+        <v>case_type3_dim3_1_text</v>
       </c>
       <c r="H30" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1ccf-c9fa-4e69-800cfa6c5e86|0195d18c-1cb2-995c-625d-dfa62a674ff8</v>
+        <v>0195d18c-1ccd-d664-179c-a1a90c3c886c|0195d18c-1cb1-b5d5-ee26-96c6a9678489</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="B31" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="C31" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B31,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set4_1_3</v>
+        <v>case_type_col_set3_3_2</v>
       </c>
       <c r="E31" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="F31" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E31,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type4_dim1_3_text</v>
+        <v>case_type3_dim3_2_text</v>
       </c>
       <c r="H31" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1ccf-d319-afba-0f13f0d06256|0195d18c-1cb2-7a1f-c2f8-ce2096e4cbbc</v>
+        <v>0195d18c-1ccd-12ae-b807-5b71d1b4e1f1|0195d18c-1cb1-f7bb-aa5b-6f2c6f5d3696</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="B32" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="C32" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B32,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set4_2_1</v>
+        <v>case_type_col_set3_3_3</v>
       </c>
       <c r="E32" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="F32" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E32,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type4_dim2_1_text</v>
+        <v>case_type3_dim3_3_text</v>
       </c>
       <c r="H32" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd0-951a-878d-5fe5fcd0015a|0195d18c-1cb3-b49c-ddc2-f5174414bfdc</v>
+        <v>0195d18c-1cce-3516-017e-cf05c78d4433|0195d18c-1cb1-2097-fae7-ffcb7e109be5</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>230</v>
+        <v>845</v>
       </c>
       <c r="B33" t="s">
-        <v>231</v>
+        <v>836</v>
       </c>
       <c r="C33" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B33,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set4_2_2</v>
+        <v>case_type_col_set3_4_1</v>
       </c>
       <c r="E33" t="s">
-        <v>232</v>
+        <v>818</v>
       </c>
       <c r="F33" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E33,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type4_dim2_2_text</v>
+        <v>case_type3_dim4_1_genetic_reads</v>
       </c>
       <c r="H33" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd0-0128-08ed-42804fabb534|0195d18c-1cb3-9495-0b74-a14fa0378944</v>
+        <v>019a8753-bed9-c7d8-6072-9a0d42887e0f|019a8753-bed9-0ab7-4323-aa6aedd4c1cc</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>233</v>
+        <v>846</v>
       </c>
       <c r="B34" t="s">
-        <v>234</v>
+        <v>835</v>
       </c>
       <c r="C34" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B34,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set4_2_3</v>
+        <v>case_type_col_set3_4_2</v>
       </c>
       <c r="E34" t="s">
-        <v>235</v>
+        <v>817</v>
       </c>
       <c r="F34" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E34,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type4_dim2_3_text</v>
+        <v>case_type3_dim4_2_genetic_sequence</v>
       </c>
       <c r="H34" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd1-9702-2218-87932d7bfde7|0195d18c-1cb3-7165-f2c8-1549624bce57</v>
+        <v>019a8753-bed9-9918-33cd-c862ad905516|019a8753-bed9-af63-b674-d9ae3c5f0a08</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>236</v>
+        <v>219</v>
       </c>
       <c r="B35" t="s">
-        <v>237</v>
+        <v>70</v>
       </c>
       <c r="C35" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B35,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set4_3_1</v>
+        <v>case_type_col_set4_1_1</v>
       </c>
       <c r="E35" t="s">
-        <v>238</v>
+        <v>220</v>
       </c>
       <c r="F35" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E35,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type4_dim3_1_text</v>
+        <v>case_type4_dim1_1_text</v>
       </c>
       <c r="H35" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd1-a4b4-2764-66bf69a9f28c|0195d18c-1cb4-62ef-acc3-d4754efbcff5</v>
+        <v>0195d18c-1cce-585d-e95b-79f3fbfdd12b|0195d18c-1cb2-95e6-139d-1dbe7ffdd3d0</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>239</v>
+        <v>221</v>
       </c>
       <c r="B36" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
       <c r="C36" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B36,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set4_3_2</v>
+        <v>case_type_col_set4_1_2</v>
       </c>
       <c r="E36" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="F36" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E36,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type4_dim3_2_text</v>
+        <v>case_type4_dim1_2_text</v>
       </c>
       <c r="H36" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd2-3359-f0c5-d09dfe10cbd9|0195d18c-1cb4-4080-ce72-0ae401b350e2</v>
+        <v>0195d18c-1ccf-c9fa-4e69-800cfa6c5e86|0195d18c-1cb2-995c-625d-dfa62a674ff8</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>242</v>
+        <v>224</v>
       </c>
       <c r="B37" t="s">
-        <v>243</v>
+        <v>225</v>
       </c>
       <c r="C37" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B37,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set4_3_3</v>
+        <v>case_type_col_set4_1_3</v>
       </c>
       <c r="E37" t="s">
-        <v>244</v>
+        <v>226</v>
       </c>
       <c r="F37" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E37,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type4_dim3_3_text</v>
+        <v>case_type4_dim1_3_text</v>
       </c>
       <c r="H37" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd2-c028-2759-dfa197e2e6c0|0195d18c-1cb4-7eca-c0f5-e64333747c9b</v>
+        <v>0195d18c-1ccf-d319-afba-0f13f0d06256|0195d18c-1cb2-7a1f-c2f8-ce2096e4cbbc</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>245</v>
+        <v>227</v>
       </c>
       <c r="B38" t="s">
-        <v>72</v>
+        <v>228</v>
       </c>
       <c r="C38" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B38,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set5_1_1</v>
+        <v>case_type_col_set4_2_1</v>
       </c>
       <c r="E38" t="s">
-        <v>246</v>
+        <v>229</v>
       </c>
       <c r="F38" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E38,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type5_dim1_1_text</v>
+        <v>case_type4_dim2_1_text</v>
       </c>
       <c r="H38" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd3-02c7-4a0d-80f544cc425a|0195d18c-1cb5-c3e7-b945-7d438ce70962</v>
+        <v>0195d18c-1cd0-951a-878d-5fe5fcd0015a|0195d18c-1cb3-b49c-ddc2-f5174414bfdc</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>247</v>
+        <v>230</v>
       </c>
       <c r="B39" t="s">
-        <v>248</v>
+        <v>231</v>
       </c>
       <c r="C39" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B39,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set5_1_2</v>
+        <v>case_type_col_set4_2_2</v>
       </c>
       <c r="E39" t="s">
-        <v>249</v>
+        <v>232</v>
       </c>
       <c r="F39" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E39,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type5_dim1_2_text</v>
+        <v>case_type4_dim2_2_text</v>
       </c>
       <c r="H39" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd3-acd1-2f6c-f9db7a3cd290|0195d18c-1cb5-8fdb-b13a-19f20c06817d</v>
+        <v>0195d18c-1cd0-0128-08ed-42804fabb534|0195d18c-1cb3-9495-0b74-a14fa0378944</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>250</v>
+        <v>233</v>
       </c>
       <c r="B40" t="s">
-        <v>251</v>
+        <v>234</v>
       </c>
       <c r="C40" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B40,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set5_1_3</v>
+        <v>case_type_col_set4_2_3</v>
       </c>
       <c r="E40" t="s">
-        <v>252</v>
+        <v>235</v>
       </c>
       <c r="F40" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E40,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type5_dim1_3_text</v>
+        <v>case_type4_dim2_3_text</v>
       </c>
       <c r="H40" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd4-44f9-ea4c-4ab401e03f8f|0195d18c-1cb5-5dbb-4903-872ca139254e</v>
+        <v>0195d18c-1cd1-9702-2218-87932d7bfde7|0195d18c-1cb3-7165-f2c8-1549624bce57</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>253</v>
+        <v>236</v>
       </c>
       <c r="B41" t="s">
-        <v>254</v>
+        <v>237</v>
       </c>
       <c r="C41" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B41,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set5_2_1</v>
+        <v>case_type_col_set4_3_1</v>
       </c>
       <c r="E41" t="s">
-        <v>255</v>
+        <v>238</v>
       </c>
       <c r="F41" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E41,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type5_dim2_1_text</v>
+        <v>case_type4_dim3_1_text</v>
       </c>
       <c r="H41" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd4-a35d-3e85-41eb9f24a911|0195d18c-1cb6-9ffa-e835-0b70cc4b0ae9</v>
+        <v>0195d18c-1cd1-a4b4-2764-66bf69a9f28c|0195d18c-1cb4-62ef-acc3-d4754efbcff5</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>256</v>
+        <v>239</v>
       </c>
       <c r="B42" t="s">
-        <v>257</v>
+        <v>240</v>
       </c>
       <c r="C42" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B42,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set5_2_2</v>
+        <v>case_type_col_set4_3_2</v>
       </c>
       <c r="E42" t="s">
-        <v>258</v>
+        <v>241</v>
       </c>
       <c r="F42" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E42,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type5_dim2_2_text</v>
+        <v>case_type4_dim3_2_text</v>
       </c>
       <c r="H42" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd5-e8f4-76f8-56e13a8aec12|0195d18c-1cb6-a2b9-4827-77425c5ab615</v>
+        <v>0195d18c-1cd2-3359-f0c5-d09dfe10cbd9|0195d18c-1cb4-4080-ce72-0ae401b350e2</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>259</v>
+        <v>242</v>
       </c>
       <c r="B43" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="C43" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B43,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set5_2_3</v>
+        <v>case_type_col_set4_3_3</v>
       </c>
       <c r="E43" t="s">
-        <v>261</v>
+        <v>244</v>
       </c>
       <c r="F43" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E43,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type5_dim2_3_text</v>
+        <v>case_type4_dim3_3_text</v>
       </c>
       <c r="H43" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd6-da43-ec75-25feee641928|0195d18c-1cb6-04b0-5474-a6411b693a97</v>
+        <v>0195d18c-1cd2-c028-2759-dfa197e2e6c0|0195d18c-1cb4-7eca-c0f5-e64333747c9b</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>262</v>
+        <v>848</v>
       </c>
       <c r="B44" t="s">
-        <v>263</v>
+        <v>834</v>
       </c>
       <c r="C44" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B44,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set5_3_1</v>
+        <v>case_type_col_set4_4_1</v>
       </c>
       <c r="E44" t="s">
-        <v>264</v>
+        <v>816</v>
       </c>
       <c r="F44" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E44,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type5_dim3_1_text</v>
+        <v>case_type4_dim4_1_genetic_reads</v>
       </c>
       <c r="H44" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd6-2f81-aefd-93fce854296f|0195d18c-1cb7-05e5-fd6b-6914a124e649</v>
+        <v>019a8753-bed9-eba4-fbce-8c553ccd262a|019a8753-bed9-9436-d94c-4e4ee8856951</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>265</v>
+        <v>847</v>
       </c>
       <c r="B45" t="s">
-        <v>266</v>
+        <v>833</v>
       </c>
       <c r="C45" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B45,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set5_3_2</v>
+        <v>case_type_col_set4_4_2</v>
       </c>
       <c r="E45" t="s">
-        <v>267</v>
+        <v>815</v>
       </c>
       <c r="F45" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E45,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type5_dim3_2_text</v>
+        <v>case_type4_dim4_2_genetic_sequence</v>
       </c>
       <c r="H45" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0195d18c-1cd7-22bb-71ce-9110669bbfef|0195d18c-1cb7-44c6-2f56-594e12327604</v>
+        <v>019a8753-bed9-47cd-cf12-b0da18fd2588|019a8753-bed9-9857-f307-13b9f5a150d1</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>268</v>
+        <v>245</v>
       </c>
       <c r="B46" t="s">
-        <v>269</v>
+        <v>72</v>
       </c>
       <c r="C46" s="6" t="str">
         <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B46,CaseTypeColSet!$A:$A,0))</f>
-        <v>case_type_col_set5_3_3</v>
+        <v>case_type_col_set5_1_1</v>
       </c>
       <c r="E46" t="s">
-        <v>270</v>
+        <v>246</v>
       </c>
       <c r="F46" s="6" t="str">
         <f>INDEX(CaseTypeCol!$G:$G,MATCH($E46,CaseTypeCol!$A:$A,0))</f>
-        <v>case_type5_dim3_3_text</v>
+        <v>case_type5_dim1_1_text</v>
       </c>
       <c r="H46" s="6" t="str">
         <f t="shared" si="0"/>
+        <v>0195d18c-1cd3-02c7-4a0d-80f544cc425a|0195d18c-1cb5-c3e7-b945-7d438ce70962</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>247</v>
+      </c>
+      <c r="B47" t="s">
+        <v>248</v>
+      </c>
+      <c r="C47" s="6" t="str">
+        <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B47,CaseTypeColSet!$A:$A,0))</f>
+        <v>case_type_col_set5_1_2</v>
+      </c>
+      <c r="E47" t="s">
+        <v>249</v>
+      </c>
+      <c r="F47" s="6" t="str">
+        <f>INDEX(CaseTypeCol!$G:$G,MATCH($E47,CaseTypeCol!$A:$A,0))</f>
+        <v>case_type5_dim1_2_text</v>
+      </c>
+      <c r="H47" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>0195d18c-1cd3-acd1-2f6c-f9db7a3cd290|0195d18c-1cb5-8fdb-b13a-19f20c06817d</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>250</v>
+      </c>
+      <c r="B48" t="s">
+        <v>251</v>
+      </c>
+      <c r="C48" s="6" t="str">
+        <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B48,CaseTypeColSet!$A:$A,0))</f>
+        <v>case_type_col_set5_1_3</v>
+      </c>
+      <c r="E48" t="s">
+        <v>252</v>
+      </c>
+      <c r="F48" s="6" t="str">
+        <f>INDEX(CaseTypeCol!$G:$G,MATCH($E48,CaseTypeCol!$A:$A,0))</f>
+        <v>case_type5_dim1_3_text</v>
+      </c>
+      <c r="H48" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>0195d18c-1cd4-44f9-ea4c-4ab401e03f8f|0195d18c-1cb5-5dbb-4903-872ca139254e</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>253</v>
+      </c>
+      <c r="B49" t="s">
+        <v>254</v>
+      </c>
+      <c r="C49" s="6" t="str">
+        <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B49,CaseTypeColSet!$A:$A,0))</f>
+        <v>case_type_col_set5_2_1</v>
+      </c>
+      <c r="E49" t="s">
+        <v>255</v>
+      </c>
+      <c r="F49" s="6" t="str">
+        <f>INDEX(CaseTypeCol!$G:$G,MATCH($E49,CaseTypeCol!$A:$A,0))</f>
+        <v>case_type5_dim2_1_text</v>
+      </c>
+      <c r="H49" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>0195d18c-1cd4-a35d-3e85-41eb9f24a911|0195d18c-1cb6-9ffa-e835-0b70cc4b0ae9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>256</v>
+      </c>
+      <c r="B50" t="s">
+        <v>257</v>
+      </c>
+      <c r="C50" s="6" t="str">
+        <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B50,CaseTypeColSet!$A:$A,0))</f>
+        <v>case_type_col_set5_2_2</v>
+      </c>
+      <c r="E50" t="s">
+        <v>258</v>
+      </c>
+      <c r="F50" s="6" t="str">
+        <f>INDEX(CaseTypeCol!$G:$G,MATCH($E50,CaseTypeCol!$A:$A,0))</f>
+        <v>case_type5_dim2_2_text</v>
+      </c>
+      <c r="H50" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>0195d18c-1cd5-e8f4-76f8-56e13a8aec12|0195d18c-1cb6-a2b9-4827-77425c5ab615</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>259</v>
+      </c>
+      <c r="B51" t="s">
+        <v>260</v>
+      </c>
+      <c r="C51" s="6" t="str">
+        <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B51,CaseTypeColSet!$A:$A,0))</f>
+        <v>case_type_col_set5_2_3</v>
+      </c>
+      <c r="E51" t="s">
+        <v>261</v>
+      </c>
+      <c r="F51" s="6" t="str">
+        <f>INDEX(CaseTypeCol!$G:$G,MATCH($E51,CaseTypeCol!$A:$A,0))</f>
+        <v>case_type5_dim2_3_text</v>
+      </c>
+      <c r="H51" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>0195d18c-1cd6-da43-ec75-25feee641928|0195d18c-1cb6-04b0-5474-a6411b693a97</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>262</v>
+      </c>
+      <c r="B52" t="s">
+        <v>263</v>
+      </c>
+      <c r="C52" s="6" t="str">
+        <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B52,CaseTypeColSet!$A:$A,0))</f>
+        <v>case_type_col_set5_3_1</v>
+      </c>
+      <c r="E52" t="s">
+        <v>264</v>
+      </c>
+      <c r="F52" s="6" t="str">
+        <f>INDEX(CaseTypeCol!$G:$G,MATCH($E52,CaseTypeCol!$A:$A,0))</f>
+        <v>case_type5_dim3_1_text</v>
+      </c>
+      <c r="H52" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>0195d18c-1cd6-2f81-aefd-93fce854296f|0195d18c-1cb7-05e5-fd6b-6914a124e649</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>265</v>
+      </c>
+      <c r="B53" t="s">
+        <v>266</v>
+      </c>
+      <c r="C53" s="6" t="str">
+        <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B53,CaseTypeColSet!$A:$A,0))</f>
+        <v>case_type_col_set5_3_2</v>
+      </c>
+      <c r="E53" t="s">
+        <v>267</v>
+      </c>
+      <c r="F53" s="6" t="str">
+        <f>INDEX(CaseTypeCol!$G:$G,MATCH($E53,CaseTypeCol!$A:$A,0))</f>
+        <v>case_type5_dim3_2_text</v>
+      </c>
+      <c r="H53" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>0195d18c-1cd7-22bb-71ce-9110669bbfef|0195d18c-1cb7-44c6-2f56-594e12327604</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>268</v>
+      </c>
+      <c r="B54" t="s">
+        <v>269</v>
+      </c>
+      <c r="C54" s="6" t="str">
+        <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B54,CaseTypeColSet!$A:$A,0))</f>
+        <v>case_type_col_set5_3_3</v>
+      </c>
+      <c r="E54" t="s">
+        <v>270</v>
+      </c>
+      <c r="F54" s="6" t="str">
+        <f>INDEX(CaseTypeCol!$G:$G,MATCH($E54,CaseTypeCol!$A:$A,0))</f>
+        <v>case_type5_dim3_3_text</v>
+      </c>
+      <c r="H54" s="6" t="str">
+        <f t="shared" si="0"/>
         <v>0195d18c-1cd7-b95b-ced6-589a63e3e6eb|0195d18c-1cb7-e7f7-a41d-bacd0f861a06</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>850</v>
+      </c>
+      <c r="B55" t="s">
+        <v>832</v>
+      </c>
+      <c r="C55" s="6" t="str">
+        <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B55,CaseTypeColSet!$A:$A,0))</f>
+        <v>case_type_col_set5_4_1</v>
+      </c>
+      <c r="E55" t="s">
+        <v>814</v>
+      </c>
+      <c r="F55" s="6" t="str">
+        <f>INDEX(CaseTypeCol!$G:$G,MATCH($E55,CaseTypeCol!$A:$A,0))</f>
+        <v>case_type5_dim4_1_genetic_reads</v>
+      </c>
+      <c r="H55" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>019a8753-bed9-8d4b-cfe4-957f28881a67|019a8753-bed9-e6df-c1d5-00f9f7cf16f3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>849</v>
+      </c>
+      <c r="B56" t="s">
+        <v>831</v>
+      </c>
+      <c r="C56" s="6" t="str">
+        <f>INDEX(CaseTypeColSet!$B:$B,MATCH($B56,CaseTypeColSet!$A:$A,0))</f>
+        <v>case_type_col_set5_4_2</v>
+      </c>
+      <c r="E56" t="s">
+        <v>813</v>
+      </c>
+      <c r="F56" s="6" t="str">
+        <f>INDEX(CaseTypeCol!$G:$G,MATCH($E56,CaseTypeCol!$A:$A,0))</f>
+        <v>case_type5_dim4_2_genetic_sequence</v>
+      </c>
+      <c r="H56" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>019a8753-bed9-b12e-cfb7-f4c9c62c8fc6|019a8753-bed9-991b-7f4f-683a81051e65</v>
       </c>
     </row>
   </sheetData>
@@ -18435,7 +19129,6 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6F0F389-1562-4A7F-BB5E-AAA96B2F3DDB}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:V11"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -18606,7 +19299,7 @@
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653|0195d18c-1ca2-a23d-1f64-00271f63199c</v>
       </c>
     </row>
-    <row r="3" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -18682,7 +19375,7 @@
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3|0195d18c-1ca2-2a29-96a5-37c6bf87f586</v>
       </c>
     </row>
-    <row r="4" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>74</v>
       </c>
@@ -18758,7 +19451,7 @@
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037|0195d18c-1ca2-3a4f-1878-fbe3282c9c76</v>
       </c>
     </row>
-    <row r="5" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>75</v>
       </c>
@@ -18834,7 +19527,7 @@
         <v>0195d18c-1c92-d419-4c71-a570f428499b|0195d18c-1ca2-e55a-608d-a42fc6f948e1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>76</v>
       </c>
@@ -18983,7 +19676,7 @@
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653|0195d18c-1ca3-f309-f6f1-e4807afe3802</v>
       </c>
     </row>
-    <row r="8" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>78</v>
       </c>
@@ -19056,7 +19749,7 @@
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3|0195d18c-1ca3-db40-a2a8-6dc905d6c1e9</v>
       </c>
     </row>
-    <row r="9" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>79</v>
       </c>
@@ -19129,7 +19822,7 @@
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037|0195d18c-1ca3-da0a-44bb-877b3a1eb73e</v>
       </c>
     </row>
-    <row r="10" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>80</v>
       </c>
@@ -19202,7 +19895,7 @@
         <v>0195d18c-1c92-d419-4c71-a570f428499b|0195d18c-1ca3-4d34-d0e9-8f024ad8651a</v>
       </c>
     </row>
-    <row r="11" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>81</v>
       </c>
@@ -19276,13 +19969,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U11" xr:uid="{A6F0F389-1562-4A7F-BB5E-AAA96B2F3DDB}">
-    <filterColumn colId="18">
-      <filters>
-        <filter val="org1"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:U11" xr:uid="{A6F0F389-1562-4A7F-BB5E-AAA96B2F3DDB}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23127,7 +23814,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
@@ -23228,6 +23915,27 @@
         <v>335</v>
       </c>
     </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>792</v>
+      </c>
+      <c r="B5" t="s">
+        <v>549</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>793</v>
+      </c>
+      <c r="D5" t="s">
+        <v>794</v>
+      </c>
+      <c r="G5" s="6" t="str">
+        <f>"dim"&amp;$C5&amp;"("&amp;$B5&amp;")"</f>
+        <v>dim4(TEXT)</v>
+      </c>
+      <c r="H5" t="s">
+        <v>335</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23235,7 +23943,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
@@ -23353,7 +24061,7 @@
         <v>549</v>
       </c>
       <c r="O3" s="13" t="str">
-        <f t="shared" ref="O3:O10" si="0">"col"&amp;$E3&amp;"("&amp;$H3&amp;")"</f>
+        <f t="shared" ref="O3:O12" si="0">"col"&amp;$E3&amp;"("&amp;$H3&amp;")"</f>
         <v>col1_2(TEXT)</v>
       </c>
       <c r="P3" t="s">
@@ -23546,6 +24254,60 @@
         <v>col3_3(TEXT)</v>
       </c>
       <c r="P10" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>791</v>
+      </c>
+      <c r="B11" t="s">
+        <v>792</v>
+      </c>
+      <c r="E11" t="s">
+        <v>799</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>797</v>
+      </c>
+      <c r="H11" t="s">
+        <v>795</v>
+      </c>
+      <c r="O11" s="13" t="str">
+        <f>"col"&amp;$E11&amp;"("&amp;$H11&amp;")"</f>
+        <v>col4_1(GENETIC_READS)</v>
+      </c>
+      <c r="P11" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>790</v>
+      </c>
+      <c r="B12" t="s">
+        <v>792</v>
+      </c>
+      <c r="E12" t="s">
+        <v>800</v>
+      </c>
+      <c r="F12">
+        <v>2</v>
+      </c>
+      <c r="G12" t="s">
+        <v>798</v>
+      </c>
+      <c r="H12" t="s">
+        <v>796</v>
+      </c>
+      <c r="O12" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>col4_2(GENETIC_SEQUENCE)</v>
+      </c>
+      <c r="P12" t="s">
         <v>335</v>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: Modified code and tests to correctly handle new ConceptSet/RefCol changes
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_access/test_casedb_case_access.xlsx
+++ b/test/casedb/integration/case_access/test_casedb_case_access.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_access\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\streevdm\gen-epix\gen-epix-api\test\casedb\integration\case_access\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{806799F4-FA30-4822-B1EF-7DBCBB5E54AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B51DA8D6-D024-482C-BC2D-6ECE9DB225A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4260" yWindow="1965" windowWidth="21600" windowHeight="11235" tabRatio="913" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Organization" sheetId="17" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2499" uniqueCount="908">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2502" uniqueCount="911">
   <si>
     <t>id</t>
   </si>
@@ -2806,6 +2806,15 @@
   </si>
   <si>
     <t>dm.write_col_set.name</t>
+  </si>
+  <si>
+    <t>regex</t>
+  </si>
+  <si>
+    <t>schema_definition</t>
+  </si>
+  <si>
+    <t>schema_uri</t>
   </si>
 </sst>
 </file>
@@ -3309,14 +3318,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3327,7 +3336,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -3338,7 +3347,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>46</v>
       </c>
@@ -3349,7 +3358,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -3360,7 +3369,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>52</v>
       </c>
@@ -3371,7 +3380,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>55</v>
       </c>
@@ -3390,16 +3399,16 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3416,7 +3425,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -3438,18 +3447,18 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.7109375" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3472,7 +3481,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>61</v>
       </c>
@@ -3490,7 +3499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>63</v>
       </c>
@@ -3508,7 +3517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>65</v>
       </c>
@@ -3526,7 +3535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>67</v>
       </c>
@@ -3544,7 +3553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>69</v>
       </c>
@@ -3562,7 +3571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>90</v>
       </c>
@@ -3580,7 +3589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>92</v>
       </c>
@@ -3598,7 +3607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>94</v>
       </c>
@@ -3616,7 +3625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -3634,7 +3643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>98</v>
       </c>
@@ -3652,7 +3661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>100</v>
       </c>
@@ -3670,7 +3679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>102</v>
       </c>
@@ -3688,7 +3697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>104</v>
       </c>
@@ -3706,7 +3715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>106</v>
       </c>
@@ -3724,7 +3733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>108</v>
       </c>
@@ -3751,18 +3760,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" style="6"/>
+    <col min="7" max="7" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3788,7 +3797,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>291</v>
       </c>
@@ -3811,7 +3820,7 @@
         <v>0195d18c-1cb8-5af5-9939-74dc8b5d3b5b|0195d18c-1ca6-fd99-9d76-fcfa0c0cf400</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>292</v>
       </c>
@@ -3831,7 +3840,7 @@
       </c>
       <c r="H3"/>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>293</v>
       </c>
@@ -3851,7 +3860,7 @@
       </c>
       <c r="H4"/>
     </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>294</v>
       </c>
@@ -3871,7 +3880,7 @@
       </c>
       <c r="H5"/>
     </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>295</v>
       </c>
@@ -3891,7 +3900,7 @@
       </c>
       <c r="H6"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>296</v>
       </c>
@@ -3914,7 +3923,7 @@
         <v>0195d18c-1cbb-d7b8-d852-987a801e0ad5|0195d18c-1ca6-fd99-9d76-fcfa0c0cf400</v>
       </c>
     </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>297</v>
       </c>
@@ -3934,7 +3943,7 @@
       </c>
       <c r="H8"/>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>298</v>
       </c>
@@ -3954,7 +3963,7 @@
       </c>
       <c r="H9"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>299</v>
       </c>
@@ -3977,7 +3986,7 @@
         <v>0195d18c-1cbb-5047-ab67-71cb2cb84047|0195d18c-1ca6-fd99-9d76-fcfa0c0cf400</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>300</v>
       </c>
@@ -4000,7 +4009,7 @@
         <v>0195d18c-1cbc-41fb-3ad7-2eed31140bd6|0195d18c-1ca6-fd99-9d76-fcfa0c0cf400</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>301</v>
       </c>
@@ -4020,7 +4029,7 @@
       </c>
       <c r="H12"/>
     </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>302</v>
       </c>
@@ -4040,7 +4049,7 @@
       </c>
       <c r="H13"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>303</v>
       </c>
@@ -4063,7 +4072,7 @@
         <v>0195d18c-1cbc-cf9a-b28d-bd77d3b30365|0195d18c-1ca6-fd99-9d76-fcfa0c0cf400</v>
       </c>
     </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>304</v>
       </c>
@@ -4083,7 +4092,7 @@
       </c>
       <c r="H15"/>
     </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>305</v>
       </c>
@@ -4103,7 +4112,7 @@
       </c>
       <c r="H16"/>
     </row>
-    <row r="17" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>306</v>
       </c>
@@ -4122,7 +4131,7 @@
         <v>case_type4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>307</v>
       </c>
@@ -4141,7 +4150,7 @@
         <v>case_type2</v>
       </c>
     </row>
-    <row r="19" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>308</v>
       </c>
@@ -4160,7 +4169,7 @@
         <v>case_type5</v>
       </c>
     </row>
-    <row r="20" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>309</v>
       </c>
@@ -4179,7 +4188,7 @@
         <v>case_type2</v>
       </c>
     </row>
-    <row r="21" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>310</v>
       </c>
@@ -4198,7 +4207,7 @@
         <v>case_type3</v>
       </c>
     </row>
-    <row r="22" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>311</v>
       </c>
@@ -4217,7 +4226,7 @@
         <v>case_type4</v>
       </c>
     </row>
-    <row r="23" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>312</v>
       </c>
@@ -4236,7 +4245,7 @@
         <v>case_type3</v>
       </c>
     </row>
-    <row r="24" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>313</v>
       </c>
@@ -4255,7 +4264,7 @@
         <v>case_type5</v>
       </c>
     </row>
-    <row r="25" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>314</v>
       </c>
@@ -4274,7 +4283,7 @@
         <v>case_type5</v>
       </c>
     </row>
-    <row r="26" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>315</v>
       </c>
@@ -4308,21 +4317,21 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{255ABC7C-6CF8-4305-B66D-D3F56E6B0FAE}">
   <dimension ref="A1:J56"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="49.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="49.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4354,7 +4363,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>814</v>
       </c>
@@ -4385,7 +4394,7 @@
         <v>dim1_1_1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>813</v>
       </c>
@@ -4416,7 +4425,7 @@
         <v>dim1_1_2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>812</v>
       </c>
@@ -4447,7 +4456,7 @@
         <v>dim1_1_3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>811</v>
       </c>
@@ -4478,7 +4487,7 @@
         <v>dim1_2_1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>810</v>
       </c>
@@ -4509,7 +4518,7 @@
         <v>dim1_2_2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>809</v>
       </c>
@@ -4540,7 +4549,7 @@
         <v>dim1_2_3</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>808</v>
       </c>
@@ -4571,7 +4580,7 @@
         <v>dim1_3_1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>807</v>
       </c>
@@ -4602,7 +4611,7 @@
         <v>dim1_3_2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>806</v>
       </c>
@@ -4633,7 +4642,7 @@
         <v>dim1_3_3</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>805</v>
       </c>
@@ -4664,7 +4673,7 @@
         <v>dim1_4_1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>804</v>
       </c>
@@ -4695,7 +4704,7 @@
         <v>dim1_4_2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>803</v>
       </c>
@@ -4726,7 +4735,7 @@
         <v>dim2_1_1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>802</v>
       </c>
@@ -4757,7 +4766,7 @@
         <v>dim2_1_2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>801</v>
       </c>
@@ -4788,7 +4797,7 @@
         <v>dim2_1_3</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>800</v>
       </c>
@@ -4819,7 +4828,7 @@
         <v>dim2_2_1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>799</v>
       </c>
@@ -4850,7 +4859,7 @@
         <v>dim2_2_2</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>798</v>
       </c>
@@ -4881,7 +4890,7 @@
         <v>dim2_2_3</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>797</v>
       </c>
@@ -4912,7 +4921,7 @@
         <v>dim2_3_1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>796</v>
       </c>
@@ -4943,7 +4952,7 @@
         <v>dim2_3_2</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>795</v>
       </c>
@@ -4974,7 +4983,7 @@
         <v>dim2_3_3</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>794</v>
       </c>
@@ -5005,7 +5014,7 @@
         <v>dim2_4_1</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>793</v>
       </c>
@@ -5036,7 +5045,7 @@
         <v>dim2_4_2</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>792</v>
       </c>
@@ -5067,7 +5076,7 @@
         <v>dim3_1_1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>791</v>
       </c>
@@ -5098,7 +5107,7 @@
         <v>dim3_1_2</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>790</v>
       </c>
@@ -5129,7 +5138,7 @@
         <v>dim3_1_3</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>789</v>
       </c>
@@ -5160,7 +5169,7 @@
         <v>dim3_2_1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>788</v>
       </c>
@@ -5191,7 +5200,7 @@
         <v>dim3_2_2</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>787</v>
       </c>
@@ -5222,7 +5231,7 @@
         <v>dim3_2_3</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>786</v>
       </c>
@@ -5253,7 +5262,7 @@
         <v>dim3_3_1</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>785</v>
       </c>
@@ -5284,7 +5293,7 @@
         <v>dim3_3_2</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>784</v>
       </c>
@@ -5315,7 +5324,7 @@
         <v>dim3_3_3</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>783</v>
       </c>
@@ -5346,7 +5355,7 @@
         <v>dim3_4_1</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>782</v>
       </c>
@@ -5377,7 +5386,7 @@
         <v>dim3_4_2</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>781</v>
       </c>
@@ -5408,7 +5417,7 @@
         <v>dim4_1_1</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>780</v>
       </c>
@@ -5439,7 +5448,7 @@
         <v>dim4_1_2</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>779</v>
       </c>
@@ -5470,7 +5479,7 @@
         <v>dim4_1_3</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>778</v>
       </c>
@@ -5501,7 +5510,7 @@
         <v>dim4_2_1</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>777</v>
       </c>
@@ -5532,7 +5541,7 @@
         <v>dim4_2_2</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>776</v>
       </c>
@@ -5563,7 +5572,7 @@
         <v>dim4_2_3</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>775</v>
       </c>
@@ -5594,7 +5603,7 @@
         <v>dim4_3_1</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>774</v>
       </c>
@@ -5625,7 +5634,7 @@
         <v>dim4_3_2</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>773</v>
       </c>
@@ -5656,7 +5665,7 @@
         <v>dim4_3_3</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>772</v>
       </c>
@@ -5687,7 +5696,7 @@
         <v>dim4_4_1</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>771</v>
       </c>
@@ -5718,7 +5727,7 @@
         <v>dim4_4_2</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>770</v>
       </c>
@@ -5749,7 +5758,7 @@
         <v>dim5_1_1</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>769</v>
       </c>
@@ -5780,7 +5789,7 @@
         <v>dim5_1_2</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>768</v>
       </c>
@@ -5811,7 +5820,7 @@
         <v>dim5_1_3</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>767</v>
       </c>
@@ -5842,7 +5851,7 @@
         <v>dim5_2_1</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>766</v>
       </c>
@@ -5873,7 +5882,7 @@
         <v>dim5_2_2</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>765</v>
       </c>
@@ -5904,7 +5913,7 @@
         <v>dim5_2_3</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>764</v>
       </c>
@@ -5935,7 +5944,7 @@
         <v>dim5_3_1</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>763</v>
       </c>
@@ -5966,7 +5975,7 @@
         <v>dim5_3_2</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>762</v>
       </c>
@@ -5997,7 +6006,7 @@
         <v>dim5_3_3</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>761</v>
       </c>
@@ -6028,7 +6037,7 @@
         <v>dim5_4_1</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>760</v>
       </c>
@@ -6068,31 +6077,30 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:U56"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="29.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="38.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="29.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="38.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="4.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="13" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="7" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="31.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6157,7 +6165,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>138</v>
       </c>
@@ -6193,7 +6201,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>141</v>
       </c>
@@ -6229,7 +6237,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>144</v>
       </c>
@@ -6265,7 +6273,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>147</v>
       </c>
@@ -6301,7 +6309,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>150</v>
       </c>
@@ -6337,7 +6345,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>153</v>
       </c>
@@ -6373,7 +6381,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>156</v>
       </c>
@@ -6409,7 +6417,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>159</v>
       </c>
@@ -6445,7 +6453,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>162</v>
       </c>
@@ -6481,7 +6489,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>663</v>
       </c>
@@ -6517,7 +6525,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>662</v>
       </c>
@@ -6553,7 +6561,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>164</v>
       </c>
@@ -6589,7 +6597,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>167</v>
       </c>
@@ -6625,7 +6633,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>170</v>
       </c>
@@ -6661,7 +6669,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>173</v>
       </c>
@@ -6697,7 +6705,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>176</v>
       </c>
@@ -6733,7 +6741,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>179</v>
       </c>
@@ -6769,7 +6777,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>182</v>
       </c>
@@ -6805,7 +6813,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>185</v>
       </c>
@@ -6841,7 +6849,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>188</v>
       </c>
@@ -6877,7 +6885,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>671</v>
       </c>
@@ -6913,7 +6921,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>670</v>
       </c>
@@ -6949,7 +6957,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>190</v>
       </c>
@@ -6985,7 +6993,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>193</v>
       </c>
@@ -7021,7 +7029,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>196</v>
       </c>
@@ -7057,7 +7065,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>199</v>
       </c>
@@ -7093,7 +7101,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>202</v>
       </c>
@@ -7129,7 +7137,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>205</v>
       </c>
@@ -7165,7 +7173,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>208</v>
       </c>
@@ -7201,7 +7209,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>211</v>
       </c>
@@ -7237,7 +7245,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>214</v>
       </c>
@@ -7273,7 +7281,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>669</v>
       </c>
@@ -7309,7 +7317,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>668</v>
       </c>
@@ -7345,7 +7353,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>216</v>
       </c>
@@ -7381,7 +7389,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>219</v>
       </c>
@@ -7417,7 +7425,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>222</v>
       </c>
@@ -7453,7 +7461,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>225</v>
       </c>
@@ -7489,7 +7497,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>228</v>
       </c>
@@ -7525,7 +7533,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>231</v>
       </c>
@@ -7561,7 +7569,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>234</v>
       </c>
@@ -7597,7 +7605,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>237</v>
       </c>
@@ -7633,7 +7641,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>240</v>
       </c>
@@ -7669,7 +7677,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>667</v>
       </c>
@@ -7705,7 +7713,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>666</v>
       </c>
@@ -7741,7 +7749,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>242</v>
       </c>
@@ -7777,7 +7785,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>245</v>
       </c>
@@ -7813,7 +7821,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>248</v>
       </c>
@@ -7849,7 +7857,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>251</v>
       </c>
@@ -7885,7 +7893,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>254</v>
       </c>
@@ -7921,7 +7929,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>257</v>
       </c>
@@ -7957,7 +7965,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>260</v>
       </c>
@@ -7993,7 +8001,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>263</v>
       </c>
@@ -8029,7 +8037,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>266</v>
       </c>
@@ -8065,7 +8073,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>665</v>
       </c>
@@ -8101,7 +8109,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>664</v>
       </c>
@@ -8145,58 +8153,58 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E0C7C33-6768-4AAE-A57E-F80585DED472}">
   <dimension ref="A1:AU75"/>
-  <sheetFormatPr defaultColWidth="5.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="5.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.44140625" customWidth="1"/>
-    <col min="3" max="3" width="36.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.42578125" customWidth="1"/>
+    <col min="3" max="3" width="36.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.6640625" style="19" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="35.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="29.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="37.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="62.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="41.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="37.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="62.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="41.7109375" style="6" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="45" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="30.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="56.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="30.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="56.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="35" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="38.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="36.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="23.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="28.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="34.44140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="38.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="38.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="36.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="23.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="28.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="34.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="38.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="12" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="34.6640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="35.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="66.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="66.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="59.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="35.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="66.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="66.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="59.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="60" style="6" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="35.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="66.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="66.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="59.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="35.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="66.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="66.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="59.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="60" style="6" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="35.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="66.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="66.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="59.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="35.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="66.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="66.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="59.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="47" max="47" width="60" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>471</v>
       </c>
@@ -8339,7 +8347,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -8494,7 +8502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -8649,7 +8657,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -8804,7 +8812,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -8959,7 +8967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -9114,7 +9122,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -9269,7 +9277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -9424,7 +9432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -9579,7 +9587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -9734,7 +9742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -9889,7 +9897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -10044,7 +10052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -10199,7 +10207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -10354,7 +10362,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -10509,7 +10517,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -10664,7 +10672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -10819,7 +10827,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -10974,7 +10982,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -11129,7 +11137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -11284,7 +11292,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -11439,7 +11447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -11594,7 +11602,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -11749,7 +11757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -11904,7 +11912,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -12059,7 +12067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -12214,7 +12222,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -12369,7 +12377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -12524,7 +12532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -12679,7 +12687,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -12834,7 +12842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -12989,7 +12997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -13144,7 +13152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -13299,7 +13307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -13466,7 +13474,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -13624,7 +13632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -13782,7 +13790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -13940,7 +13948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -14098,7 +14106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -14256,7 +14264,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -14414,7 +14422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -14572,7 +14580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -14730,7 +14738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -14888,7 +14896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -15043,7 +15051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -15198,7 +15206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -15356,7 +15364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -15514,7 +15522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -15672,7 +15680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -15830,7 +15838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -15988,7 +15996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -16146,7 +16154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -16304,7 +16312,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -16462,7 +16470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -16629,7 +16637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -16796,7 +16804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -16963,7 +16971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -17124,7 +17132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -17285,7 +17293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -17446,7 +17454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -17604,7 +17612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -17762,7 +17770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -17920,7 +17928,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -18078,7 +18086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -18239,7 +18247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -18400,7 +18408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -18561,7 +18569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -18722,7 +18730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -18883,7 +18891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -19044,7 +19052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -19205,7 +19213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -19366,7 +19374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -19524,7 +19532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -19682,7 +19690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -19840,7 +19848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -20013,13 +20021,13 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:C56"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="21.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -20030,7 +20038,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>62</v>
       </c>
@@ -20041,7 +20049,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>140</v>
       </c>
@@ -20052,7 +20060,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>143</v>
       </c>
@@ -20063,7 +20071,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>146</v>
       </c>
@@ -20074,7 +20082,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>149</v>
       </c>
@@ -20085,7 +20093,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>152</v>
       </c>
@@ -20096,7 +20104,7 @@
         <v>854</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>155</v>
       </c>
@@ -20107,7 +20115,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>158</v>
       </c>
@@ -20118,7 +20126,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>161</v>
       </c>
@@ -20129,7 +20137,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>680</v>
       </c>
@@ -20140,7 +20148,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>681</v>
       </c>
@@ -20151,7 +20159,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>64</v>
       </c>
@@ -20162,7 +20170,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>166</v>
       </c>
@@ -20173,7 +20181,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>169</v>
       </c>
@@ -20184,7 +20192,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>172</v>
       </c>
@@ -20195,7 +20203,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>175</v>
       </c>
@@ -20206,7 +20214,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>178</v>
       </c>
@@ -20217,7 +20225,7 @@
         <v>865</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>181</v>
       </c>
@@ -20228,7 +20236,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>184</v>
       </c>
@@ -20239,7 +20247,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>187</v>
       </c>
@@ -20250,7 +20258,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>678</v>
       </c>
@@ -20261,7 +20269,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>679</v>
       </c>
@@ -20272,7 +20280,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>66</v>
       </c>
@@ -20283,7 +20291,7 @@
         <v>871</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>192</v>
       </c>
@@ -20294,7 +20302,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>195</v>
       </c>
@@ -20305,7 +20313,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>198</v>
       </c>
@@ -20316,7 +20324,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>201</v>
       </c>
@@ -20327,7 +20335,7 @@
         <v>875</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>204</v>
       </c>
@@ -20338,7 +20346,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>207</v>
       </c>
@@ -20349,7 +20357,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>210</v>
       </c>
@@ -20360,7 +20368,7 @@
         <v>878</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>213</v>
       </c>
@@ -20371,7 +20379,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>677</v>
       </c>
@@ -20382,7 +20390,7 @@
         <v>880</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>676</v>
       </c>
@@ -20393,7 +20401,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>68</v>
       </c>
@@ -20404,7 +20412,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>218</v>
       </c>
@@ -20415,7 +20423,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>221</v>
       </c>
@@ -20426,7 +20434,7 @@
         <v>884</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>224</v>
       </c>
@@ -20437,7 +20445,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>227</v>
       </c>
@@ -20448,7 +20456,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>230</v>
       </c>
@@ -20459,7 +20467,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>233</v>
       </c>
@@ -20470,7 +20478,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>236</v>
       </c>
@@ -20481,7 +20489,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>239</v>
       </c>
@@ -20492,7 +20500,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>675</v>
       </c>
@@ -20503,7 +20511,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>674</v>
       </c>
@@ -20514,7 +20522,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>70</v>
       </c>
@@ -20525,7 +20533,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>244</v>
       </c>
@@ -20536,7 +20544,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>247</v>
       </c>
@@ -20547,7 +20555,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>250</v>
       </c>
@@ -20558,7 +20566,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>253</v>
       </c>
@@ -20569,7 +20577,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>256</v>
       </c>
@@ -20580,7 +20588,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>259</v>
       </c>
@@ -20591,7 +20599,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>262</v>
       </c>
@@ -20602,7 +20610,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>265</v>
       </c>
@@ -20613,7 +20621,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>673</v>
       </c>
@@ -20624,7 +20632,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>672</v>
       </c>
@@ -20644,18 +20652,18 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H56"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.6640625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" style="6"/>
+    <col min="5" max="5" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.7109375" style="6" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -20681,7 +20689,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>137</v>
       </c>
@@ -20704,7 +20712,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0195d18c-1caa-1722-0366-f73bd3f09ee8</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>139</v>
       </c>
@@ -20727,7 +20735,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0195d18c-1cab-86f3-5faf-507bfa221cf6</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>142</v>
       </c>
@@ -20750,7 +20758,7 @@
         <v>0195d18c-1cc2-37d1-f6c3-0e7c8d6b1f07|0195d18c-1cab-b4e5-a81b-6acdcc710af2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>145</v>
       </c>
@@ -20773,7 +20781,7 @@
         <v>0195d18c-1cc2-7cf5-8b5c-03f41714d8b8|0195d18c-1cab-3208-7ccc-820a8c522208</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>148</v>
       </c>
@@ -20796,7 +20804,7 @@
         <v>0195d18c-1cc2-50aa-7113-6b261eaeec7a|0195d18c-1cab-767e-81b1-986e918827fb</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>151</v>
       </c>
@@ -20819,7 +20827,7 @@
         <v>0195d18c-1cc3-0cbc-2362-c1cfe3fdec5a|0195d18c-1cab-22f7-dda1-cc74cee303ca</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>154</v>
       </c>
@@ -20842,7 +20850,7 @@
         <v>0195d18c-1cc3-e9c0-5858-8bf9d9d8c36f|0195d18c-1cac-4ed2-2296-a46fa423ce99</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>157</v>
       </c>
@@ -20865,7 +20873,7 @@
         <v>0195d18c-1cc4-9f18-3767-29d288f47190|0195d18c-1cac-9221-a9c7-72e70e09dea9</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>160</v>
       </c>
@@ -20888,7 +20896,7 @@
         <v>0195d18c-1cc5-2ea3-8102-7b410f3146c8|0195d18c-1cac-4d0a-db2e-5a54065df180</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>682</v>
       </c>
@@ -20911,7 +20919,7 @@
         <v>019a8753-bed9-afc6-e887-8b50ddfd6962|019a8753-bed9-180c-d818-10c8aed7f4c5</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>683</v>
       </c>
@@ -20934,7 +20942,7 @@
         <v>019a8753-bed9-869e-506b-15ae88b8c755|019a8753-bed9-8a7b-7c82-adf57928fa72</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>163</v>
       </c>
@@ -20957,7 +20965,7 @@
         <v>0195d18c-1cc6-a324-3f72-222014292515|0195d18c-1cad-37c6-0826-9671f313fb2b</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>165</v>
       </c>
@@ -20980,7 +20988,7 @@
         <v>0195d18c-1cc7-243f-f4e7-3dbdfe691c71|0195d18c-1cad-5b48-8a72-25050cbf379e</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>168</v>
       </c>
@@ -21003,7 +21011,7 @@
         <v>0195d18c-1cc7-60b4-b4e6-8ff7fabb2b09|0195d18c-1cad-e18e-a87d-8af6760d00e1</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>171</v>
       </c>
@@ -21026,7 +21034,7 @@
         <v>0195d18c-1cc8-bcf2-c56f-04928f2e3635|0195d18c-1cad-9467-449f-6341c820b944</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>174</v>
       </c>
@@ -21049,7 +21057,7 @@
         <v>0195d18c-1cc8-18f5-27a5-fd3874e6b78b|0195d18c-1cae-fcea-56fe-4577ada0491d</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>177</v>
       </c>
@@ -21072,7 +21080,7 @@
         <v>0195d18c-1cc8-5a76-0a72-16117b0a5a5e|0195d18c-1cae-cdba-00d9-e8405172259e</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>180</v>
       </c>
@@ -21095,7 +21103,7 @@
         <v>0195d18c-1cc9-7181-fd5b-078012e228f2|0195d18c-1cae-faa7-ac0d-22cce7d230ec</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>183</v>
       </c>
@@ -21118,7 +21126,7 @@
         <v>0195d18c-1cc9-c61f-4e7e-a00189d3cc75|0195d18c-1cae-45ab-ca21-9cee527b9482</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>186</v>
       </c>
@@ -21141,7 +21149,7 @@
         <v>0195d18c-1cca-878e-2110-0116e848541b|0195d18c-1caf-d364-c3b5-e73ba434270e</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>684</v>
       </c>
@@ -21164,7 +21172,7 @@
         <v>019a8753-bed9-8f84-5827-8c0fedea4c3d|019a8753-bed9-10ef-cde6-dd672b6f1342</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>685</v>
       </c>
@@ -21187,7 +21195,7 @@
         <v>019a8753-bed9-2ec3-f155-116a4b0fe44d|019a8753-bed9-423c-9007-26ece8e894c8</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>189</v>
       </c>
@@ -21210,7 +21218,7 @@
         <v>0195d18c-1cca-26c0-66df-979380a43b16|0195d18c-1caf-b3af-f64e-bd18810c4521</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>191</v>
       </c>
@@ -21233,7 +21241,7 @@
         <v>0195d18c-1ccb-f06f-162f-a5dc745a5198|0195d18c-1caf-84ca-1737-a8f8788cd464</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>194</v>
       </c>
@@ -21256,7 +21264,7 @@
         <v>0195d18c-1ccb-b068-d845-d61fb54721f1|0195d18c-1cb0-7655-a8bb-f656b1b8b72c</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>197</v>
       </c>
@@ -21279,7 +21287,7 @@
         <v>0195d18c-1ccc-f754-4a4f-89cdc532a3be|0195d18c-1cb0-4c24-e2e8-b92cfc74f7cc</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>200</v>
       </c>
@@ -21302,7 +21310,7 @@
         <v>0195d18c-1ccc-3f10-cc4e-636793b1e9dd|0195d18c-1cb0-8d34-e3f0-ab091b80ab8f</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>203</v>
       </c>
@@ -21325,7 +21333,7 @@
         <v>0195d18c-1ccd-3f53-ad72-f2d3c667b246|0195d18c-1cb0-db51-ed28-2a4481c5f1ac</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>206</v>
       </c>
@@ -21348,7 +21356,7 @@
         <v>0195d18c-1ccd-d664-179c-a1a90c3c886c|0195d18c-1cb1-b5d5-ee26-96c6a9678489</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>209</v>
       </c>
@@ -21371,7 +21379,7 @@
         <v>0195d18c-1ccd-12ae-b807-5b71d1b4e1f1|0195d18c-1cb1-f7bb-aa5b-6f2c6f5d3696</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>212</v>
       </c>
@@ -21394,7 +21402,7 @@
         <v>0195d18c-1cce-3516-017e-cf05c78d4433|0195d18c-1cb1-2097-fae7-ffcb7e109be5</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>686</v>
       </c>
@@ -21417,7 +21425,7 @@
         <v>019a8753-bed9-c7d8-6072-9a0d42887e0f|019a8753-bed9-0ab7-4323-aa6aedd4c1cc</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>687</v>
       </c>
@@ -21440,7 +21448,7 @@
         <v>019a8753-bed9-9918-33cd-c862ad905516|019a8753-bed9-af63-b674-d9ae3c5f0a08</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>215</v>
       </c>
@@ -21463,7 +21471,7 @@
         <v>0195d18c-1cce-585d-e95b-79f3fbfdd12b|0195d18c-1cb2-95e6-139d-1dbe7ffdd3d0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>217</v>
       </c>
@@ -21486,7 +21494,7 @@
         <v>0195d18c-1ccf-c9fa-4e69-800cfa6c5e86|0195d18c-1cb2-995c-625d-dfa62a674ff8</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>220</v>
       </c>
@@ -21509,7 +21517,7 @@
         <v>0195d18c-1ccf-d319-afba-0f13f0d06256|0195d18c-1cb2-7a1f-c2f8-ce2096e4cbbc</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>223</v>
       </c>
@@ -21532,7 +21540,7 @@
         <v>0195d18c-1cd0-951a-878d-5fe5fcd0015a|0195d18c-1cb3-b49c-ddc2-f5174414bfdc</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>226</v>
       </c>
@@ -21555,7 +21563,7 @@
         <v>0195d18c-1cd0-0128-08ed-42804fabb534|0195d18c-1cb3-9495-0b74-a14fa0378944</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>229</v>
       </c>
@@ -21578,7 +21586,7 @@
         <v>0195d18c-1cd1-9702-2218-87932d7bfde7|0195d18c-1cb3-7165-f2c8-1549624bce57</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>232</v>
       </c>
@@ -21601,7 +21609,7 @@
         <v>0195d18c-1cd1-a4b4-2764-66bf69a9f28c|0195d18c-1cb4-62ef-acc3-d4754efbcff5</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>235</v>
       </c>
@@ -21624,7 +21632,7 @@
         <v>0195d18c-1cd2-3359-f0c5-d09dfe10cbd9|0195d18c-1cb4-4080-ce72-0ae401b350e2</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>238</v>
       </c>
@@ -21647,7 +21655,7 @@
         <v>0195d18c-1cd2-c028-2759-dfa197e2e6c0|0195d18c-1cb4-7eca-c0f5-e64333747c9b</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>689</v>
       </c>
@@ -21670,7 +21678,7 @@
         <v>019a8753-bed9-eba4-fbce-8c553ccd262a|019a8753-bed9-9436-d94c-4e4ee8856951</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>688</v>
       </c>
@@ -21693,7 +21701,7 @@
         <v>019a8753-bed9-47cd-cf12-b0da18fd2588|019a8753-bed9-9857-f307-13b9f5a150d1</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>241</v>
       </c>
@@ -21716,7 +21724,7 @@
         <v>0195d18c-1cd3-02c7-4a0d-80f544cc425a|0195d18c-1cb5-c3e7-b945-7d438ce70962</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>243</v>
       </c>
@@ -21739,7 +21747,7 @@
         <v>0195d18c-1cd3-acd1-2f6c-f9db7a3cd290|0195d18c-1cb5-8fdb-b13a-19f20c06817d</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>246</v>
       </c>
@@ -21762,7 +21770,7 @@
         <v>0195d18c-1cd4-44f9-ea4c-4ab401e03f8f|0195d18c-1cb5-5dbb-4903-872ca139254e</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>249</v>
       </c>
@@ -21785,7 +21793,7 @@
         <v>0195d18c-1cd4-a35d-3e85-41eb9f24a911|0195d18c-1cb6-9ffa-e835-0b70cc4b0ae9</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>252</v>
       </c>
@@ -21808,7 +21816,7 @@
         <v>0195d18c-1cd5-e8f4-76f8-56e13a8aec12|0195d18c-1cb6-a2b9-4827-77425c5ab615</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>255</v>
       </c>
@@ -21831,7 +21839,7 @@
         <v>0195d18c-1cd6-da43-ec75-25feee641928|0195d18c-1cb6-04b0-5474-a6411b693a97</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>258</v>
       </c>
@@ -21854,7 +21862,7 @@
         <v>0195d18c-1cd6-2f81-aefd-93fce854296f|0195d18c-1cb7-05e5-fd6b-6914a124e649</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>261</v>
       </c>
@@ -21877,7 +21885,7 @@
         <v>0195d18c-1cd7-22bb-71ce-9110669bbfef|0195d18c-1cb7-44c6-2f56-594e12327604</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>264</v>
       </c>
@@ -21900,7 +21908,7 @@
         <v>0195d18c-1cd7-b95b-ced6-589a63e3e6eb|0195d18c-1cb7-e7f7-a41d-bacd0f861a06</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>691</v>
       </c>
@@ -21923,7 +21931,7 @@
         <v>019a8753-bed9-8d4b-cfe4-957f28881a67|019a8753-bed9-e6df-c1d5-00f9f7cf16f3</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>690</v>
       </c>
@@ -21954,17 +21962,17 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -21984,7 +21992,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -22006,7 +22014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -22028,7 +22036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>48</v>
       </c>
@@ -22050,7 +22058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -22072,7 +22080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -22102,32 +22110,32 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6F0F389-1562-4A7F-BB5E-AAA96B2F3DDB}">
   <dimension ref="A1:V11"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="35.6640625" customWidth="1"/>
-    <col min="13" max="13" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="35.7109375" customWidth="1"/>
+    <col min="13" max="13" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="36" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.44140625" customWidth="1"/>
+    <col min="19" max="19" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -22195,7 +22203,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>60</v>
       </c>
@@ -22271,7 +22279,7 @@
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653|0195d18c-1ca2-a23d-1f64-00271f63199c</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -22347,7 +22355,7 @@
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3|0195d18c-1ca2-2a29-96a5-37c6bf87f586</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>72</v>
       </c>
@@ -22423,7 +22431,7 @@
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037|0195d18c-1ca2-3a4f-1878-fbe3282c9c76</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>73</v>
       </c>
@@ -22499,7 +22507,7 @@
         <v>0195d18c-1c92-d419-4c71-a570f428499b|0195d18c-1ca2-e55a-608d-a42fc6f948e1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>74</v>
       </c>
@@ -22575,7 +22583,7 @@
         <v>0195d18c-1c93-02a2-6920-7e4dbfb73ce0|0195d18c-1ca2-b728-a2a1-d2a4cf7b8eb8</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>75</v>
       </c>
@@ -22648,7 +22656,7 @@
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653|0195d18c-1ca3-f309-f6f1-e4807afe3802</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>76</v>
       </c>
@@ -22721,7 +22729,7 @@
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3|0195d18c-1ca3-db40-a2a8-6dc905d6c1e9</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -22794,7 +22802,7 @@
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037|0195d18c-1ca3-da0a-44bb-877b3a1eb73e</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>78</v>
       </c>
@@ -22867,7 +22875,7 @@
         <v>0195d18c-1c92-d419-4c71-a570f428499b|0195d18c-1ca3-4d34-d0e9-8f024ad8651a</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>79</v>
       </c>
@@ -22949,14 +22957,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -22967,7 +22975,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -22979,7 +22987,7 @@
         <v>dc1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -22991,7 +22999,7 @@
         <v>dc2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -23003,7 +23011,7 @@
         <v>dc3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -23015,7 +23023,7 @@
         <v>dc4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -23027,7 +23035,7 @@
         <v>dc5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -23039,7 +23047,7 @@
         <v>dc6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -23051,7 +23059,7 @@
         <v>dc7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -23063,7 +23071,7 @@
         <v>dc8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -23075,7 +23083,7 @@
         <v>dc9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -23087,7 +23095,7 @@
         <v>dc10</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -23108,32 +23116,32 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{413B6EDF-4214-4325-A1BD-732A42D052EA}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:W11"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="35.6640625" customWidth="1"/>
-    <col min="12" max="12" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="25.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="42.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="35.7109375" customWidth="1"/>
+    <col min="12" max="12" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="42.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="36" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -23204,7 +23212,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>60</v>
       </c>
@@ -23285,7 +23293,7 @@
         <v>0195d18c-1c98-7e0b-0c91-8cafbdb2c852|0195d18c-1ca2-a23d-1f64-00271f63199c</v>
       </c>
     </row>
-    <row r="3" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -23366,7 +23374,7 @@
         <v>0195d18c-1c9a-1178-0519-9124131763a6|0195d18c-1ca2-2a29-96a5-37c6bf87f586</v>
       </c>
     </row>
-    <row r="4" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>72</v>
       </c>
@@ -23447,7 +23455,7 @@
         <v>0195d18c-1c9c-0d8f-435a-5ca8b45939b8|0195d18c-1ca2-3a4f-1878-fbe3282c9c76</v>
       </c>
     </row>
-    <row r="5" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>73</v>
       </c>
@@ -23528,7 +23536,7 @@
         <v>0195d18c-1c9e-1c4a-1311-4f22f0d59f61|0195d18c-1ca2-e55a-608d-a42fc6f948e1</v>
       </c>
     </row>
-    <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>74</v>
       </c>
@@ -23609,7 +23617,7 @@
         <v>0195d18c-1ca0-e0db-7a87-6237ad6380c8|0195d18c-1ca2-b728-a2a1-d2a4cf7b8eb8</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>75</v>
       </c>
@@ -23690,7 +23698,7 @@
         <v>0195d18c-1c98-7e0b-0c91-8cafbdb2c852|0195d18c-1ca3-f309-f6f1-e4807afe3802</v>
       </c>
     </row>
-    <row r="8" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>76</v>
       </c>
@@ -23771,7 +23779,7 @@
         <v>0195d18c-1c9a-1178-0519-9124131763a6|0195d18c-1ca3-db40-a2a8-6dc905d6c1e9</v>
       </c>
     </row>
-    <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -23852,7 +23860,7 @@
         <v>0195d18c-1c9c-0d8f-435a-5ca8b45939b8|0195d18c-1ca3-da0a-44bb-877b3a1eb73e</v>
       </c>
     </row>
-    <row r="10" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>78</v>
       </c>
@@ -23933,7 +23941,7 @@
         <v>0195d18c-1c9e-1c4a-1311-4f22f0d59f61|0195d18c-1ca3-4d34-d0e9-8f024ad8651a</v>
       </c>
     </row>
-    <row r="11" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>79</v>
       </c>
@@ -24029,26 +24037,26 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46B1A0CE-352C-4E69-8986-540397C3CD9D}">
   <dimension ref="A1:P2"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="35.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="27.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="36" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="35.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -24098,7 +24106,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>453</v>
       </c>
@@ -24166,25 +24174,25 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21E03A8B-A0A1-46B6-957F-B8B3E001E975}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="27.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="36" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -24228,7 +24236,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>453</v>
       </c>
@@ -24288,22 +24296,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:M29"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.33203125" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.28515625" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="36" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="14.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -24344,7 +24352,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>586</v>
       </c>
@@ -24392,7 +24400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>337</v>
       </c>
@@ -24440,7 +24448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>339</v>
       </c>
@@ -24488,7 +24496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -24536,7 +24544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>47</v>
       </c>
@@ -24584,7 +24592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>50</v>
       </c>
@@ -24632,7 +24640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>53</v>
       </c>
@@ -24680,7 +24688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>56</v>
       </c>
@@ -24728,7 +24736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -24776,7 +24784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -24824,7 +24832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -24872,7 +24880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -24920,7 +24928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -24968,7 +24976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -25016,7 +25024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -25064,7 +25072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -25112,7 +25120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -25160,7 +25168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -25208,7 +25216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -25256,7 +25264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -25304,7 +25312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -25352,7 +25360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -25400,7 +25408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>31</v>
       </c>
@@ -25448,7 +25456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -25496,7 +25504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>34</v>
       </c>
@@ -25544,7 +25552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -25592,7 +25600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -25640,7 +25648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -25700,21 +25708,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:K28"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="27" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" style="6" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="36" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -25749,7 +25757,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>385</v>
       </c>
@@ -25787,7 +25795,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>387</v>
       </c>
@@ -25825,7 +25833,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>389</v>
       </c>
@@ -25863,7 +25871,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>391</v>
       </c>
@@ -25901,7 +25909,7 @@
         <v>org2</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>393</v>
       </c>
@@ -25939,7 +25947,7 @@
         <v>org3</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>395</v>
       </c>
@@ -25977,7 +25985,7 @@
         <v>org4</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>397</v>
       </c>
@@ -26015,7 +26023,7 @@
         <v>org5</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>399</v>
       </c>
@@ -26053,7 +26061,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>401</v>
       </c>
@@ -26091,7 +26099,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>403</v>
       </c>
@@ -26129,7 +26137,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>405</v>
       </c>
@@ -26167,7 +26175,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>407</v>
       </c>
@@ -26205,7 +26213,7 @@
         <v>org2</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>409</v>
       </c>
@@ -26243,7 +26251,7 @@
         <v>org2</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>411</v>
       </c>
@@ -26281,7 +26289,7 @@
         <v>org2</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>413</v>
       </c>
@@ -26319,7 +26327,7 @@
         <v>org2</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>415</v>
       </c>
@@ -26357,7 +26365,7 @@
         <v>org3</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>417</v>
       </c>
@@ -26395,7 +26403,7 @@
         <v>org3</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>419</v>
       </c>
@@ -26433,7 +26441,7 @@
         <v>org3</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>421</v>
       </c>
@@ -26471,7 +26479,7 @@
         <v>org3</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>423</v>
       </c>
@@ -26509,7 +26517,7 @@
         <v>org4</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>425</v>
       </c>
@@ -26547,7 +26555,7 @@
         <v>org4</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>427</v>
       </c>
@@ -26585,7 +26593,7 @@
         <v>org4</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>429</v>
       </c>
@@ -26623,7 +26631,7 @@
         <v>org4</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>431</v>
       </c>
@@ -26661,7 +26669,7 @@
         <v>org5</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>433</v>
       </c>
@@ -26699,7 +26707,7 @@
         <v>org5</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>435</v>
       </c>
@@ -26737,7 +26745,7 @@
         <v>org5</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>437</v>
       </c>
@@ -26787,18 +26795,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -26824,7 +26832,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>326</v>
       </c>
@@ -26852,7 +26860,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>327</v>
       </c>
@@ -26880,7 +26888,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>328</v>
       </c>
@@ -26908,7 +26916,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>655</v>
       </c>
@@ -26943,28 +26951,28 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:P12"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:S12"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.6640625" style="13" customWidth="1"/>
-    <col min="16" max="16" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="26.28515625" style="13" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -27013,8 +27021,17 @@
       <c r="P1" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q1" t="s">
+        <v>908</v>
+      </c>
+      <c r="R1" t="s">
+        <v>909</v>
+      </c>
+      <c r="S1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>281</v>
       </c>
@@ -27041,7 +27058,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>283</v>
       </c>
@@ -27068,7 +27085,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>284</v>
       </c>
@@ -27095,7 +27112,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>285</v>
       </c>
@@ -27122,7 +27139,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>286</v>
       </c>
@@ -27149,7 +27166,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>287</v>
       </c>
@@ -27176,7 +27193,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>288</v>
       </c>
@@ -27203,7 +27220,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>289</v>
       </c>
@@ -27230,7 +27247,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>290</v>
       </c>
@@ -27257,7 +27274,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>654</v>
       </c>
@@ -27284,7 +27301,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>653</v>
       </c>
@@ -27319,12 +27336,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BFE9DBA-4D09-4E45-A394-72AC78245E1D}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -27335,7 +27352,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>119</v>
       </c>
@@ -27343,7 +27360,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>123</v>
       </c>
@@ -27351,7 +27368,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>127</v>
       </c>
@@ -27359,7 +27376,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>131</v>
       </c>
@@ -27367,7 +27384,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>135</v>
       </c>
@@ -27384,14 +27401,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFBF5204-3F7C-438F-A194-7543BC84CF2A}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -27402,7 +27419,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>120</v>
       </c>
@@ -27413,7 +27430,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>124</v>
       </c>
@@ -27424,7 +27441,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>128</v>
       </c>
@@ -27435,7 +27452,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>132</v>
       </c>
@@ -27446,7 +27463,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>136</v>
       </c>
@@ -27466,19 +27483,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.6640625" style="13" customWidth="1"/>
+    <col min="4" max="4" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.7109375" style="13" customWidth="1"/>
     <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="35.33203125" style="13" customWidth="1"/>
+    <col min="7" max="7" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.28515625" style="13" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -27507,7 +27524,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>117</v>
       </c>
@@ -27529,7 +27546,7 @@
         <v>etiological_agent1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>121</v>
       </c>
@@ -27551,7 +27568,7 @@
         <v>etiological_agent2</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>125</v>
       </c>
@@ -27573,7 +27590,7 @@
         <v>etiological_agent3</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>129</v>
       </c>
@@ -27595,7 +27612,7 @@
         <v>etiological_agent4</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>133</v>
       </c>

</xml_diff>

<commit_message>
feat: Introduced new Protocol model to replace all existing protocols (#467)
Co-authored-by: Ivo van Walle <ivo.van.walle@rivm.nl>
Co-authored-by: raaijmag <gino.raaijmakers@rivm.nl>
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_access/test_casedb_case_access.xlsx
+++ b/test/casedb/integration/case_access/test_casedb_case_access.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_access\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\streevdm\gen-epix\gen-epix-api\test\casedb\integration\case_access\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{806799F4-FA30-4822-B1EF-7DBCBB5E54AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B51DA8D6-D024-482C-BC2D-6ECE9DB225A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4260" yWindow="1965" windowWidth="21600" windowHeight="11235" tabRatio="913" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Organization" sheetId="17" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2499" uniqueCount="908">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2502" uniqueCount="911">
   <si>
     <t>id</t>
   </si>
@@ -2806,6 +2806,15 @@
   </si>
   <si>
     <t>dm.write_col_set.name</t>
+  </si>
+  <si>
+    <t>regex</t>
+  </si>
+  <si>
+    <t>schema_definition</t>
+  </si>
+  <si>
+    <t>schema_uri</t>
   </si>
 </sst>
 </file>
@@ -3309,14 +3318,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3327,7 +3336,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -3338,7 +3347,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>46</v>
       </c>
@@ -3349,7 +3358,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -3360,7 +3369,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>52</v>
       </c>
@@ -3371,7 +3380,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>55</v>
       </c>
@@ -3390,16 +3399,16 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3416,7 +3425,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -3438,18 +3447,18 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.7109375" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3472,7 +3481,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>61</v>
       </c>
@@ -3490,7 +3499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>63</v>
       </c>
@@ -3508,7 +3517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>65</v>
       </c>
@@ -3526,7 +3535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>67</v>
       </c>
@@ -3544,7 +3553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>69</v>
       </c>
@@ -3562,7 +3571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>90</v>
       </c>
@@ -3580,7 +3589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>92</v>
       </c>
@@ -3598,7 +3607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>94</v>
       </c>
@@ -3616,7 +3625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -3634,7 +3643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>98</v>
       </c>
@@ -3652,7 +3661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>100</v>
       </c>
@@ -3670,7 +3679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>102</v>
       </c>
@@ -3688,7 +3697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>104</v>
       </c>
@@ -3706,7 +3715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>106</v>
       </c>
@@ -3724,7 +3733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>108</v>
       </c>
@@ -3751,18 +3760,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" style="6"/>
+    <col min="7" max="7" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3788,7 +3797,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>291</v>
       </c>
@@ -3811,7 +3820,7 @@
         <v>0195d18c-1cb8-5af5-9939-74dc8b5d3b5b|0195d18c-1ca6-fd99-9d76-fcfa0c0cf400</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>292</v>
       </c>
@@ -3831,7 +3840,7 @@
       </c>
       <c r="H3"/>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>293</v>
       </c>
@@ -3851,7 +3860,7 @@
       </c>
       <c r="H4"/>
     </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>294</v>
       </c>
@@ -3871,7 +3880,7 @@
       </c>
       <c r="H5"/>
     </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>295</v>
       </c>
@@ -3891,7 +3900,7 @@
       </c>
       <c r="H6"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>296</v>
       </c>
@@ -3914,7 +3923,7 @@
         <v>0195d18c-1cbb-d7b8-d852-987a801e0ad5|0195d18c-1ca6-fd99-9d76-fcfa0c0cf400</v>
       </c>
     </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>297</v>
       </c>
@@ -3934,7 +3943,7 @@
       </c>
       <c r="H8"/>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>298</v>
       </c>
@@ -3954,7 +3963,7 @@
       </c>
       <c r="H9"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>299</v>
       </c>
@@ -3977,7 +3986,7 @@
         <v>0195d18c-1cbb-5047-ab67-71cb2cb84047|0195d18c-1ca6-fd99-9d76-fcfa0c0cf400</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>300</v>
       </c>
@@ -4000,7 +4009,7 @@
         <v>0195d18c-1cbc-41fb-3ad7-2eed31140bd6|0195d18c-1ca6-fd99-9d76-fcfa0c0cf400</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>301</v>
       </c>
@@ -4020,7 +4029,7 @@
       </c>
       <c r="H12"/>
     </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>302</v>
       </c>
@@ -4040,7 +4049,7 @@
       </c>
       <c r="H13"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>303</v>
       </c>
@@ -4063,7 +4072,7 @@
         <v>0195d18c-1cbc-cf9a-b28d-bd77d3b30365|0195d18c-1ca6-fd99-9d76-fcfa0c0cf400</v>
       </c>
     </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>304</v>
       </c>
@@ -4083,7 +4092,7 @@
       </c>
       <c r="H15"/>
     </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>305</v>
       </c>
@@ -4103,7 +4112,7 @@
       </c>
       <c r="H16"/>
     </row>
-    <row r="17" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>306</v>
       </c>
@@ -4122,7 +4131,7 @@
         <v>case_type4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>307</v>
       </c>
@@ -4141,7 +4150,7 @@
         <v>case_type2</v>
       </c>
     </row>
-    <row r="19" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>308</v>
       </c>
@@ -4160,7 +4169,7 @@
         <v>case_type5</v>
       </c>
     </row>
-    <row r="20" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>309</v>
       </c>
@@ -4179,7 +4188,7 @@
         <v>case_type2</v>
       </c>
     </row>
-    <row r="21" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>310</v>
       </c>
@@ -4198,7 +4207,7 @@
         <v>case_type3</v>
       </c>
     </row>
-    <row r="22" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>311</v>
       </c>
@@ -4217,7 +4226,7 @@
         <v>case_type4</v>
       </c>
     </row>
-    <row r="23" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>312</v>
       </c>
@@ -4236,7 +4245,7 @@
         <v>case_type3</v>
       </c>
     </row>
-    <row r="24" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>313</v>
       </c>
@@ -4255,7 +4264,7 @@
         <v>case_type5</v>
       </c>
     </row>
-    <row r="25" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>314</v>
       </c>
@@ -4274,7 +4283,7 @@
         <v>case_type5</v>
       </c>
     </row>
-    <row r="26" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>315</v>
       </c>
@@ -4308,21 +4317,21 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{255ABC7C-6CF8-4305-B66D-D3F56E6B0FAE}">
   <dimension ref="A1:J56"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="49.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="49.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4354,7 +4363,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>814</v>
       </c>
@@ -4385,7 +4394,7 @@
         <v>dim1_1_1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>813</v>
       </c>
@@ -4416,7 +4425,7 @@
         <v>dim1_1_2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>812</v>
       </c>
@@ -4447,7 +4456,7 @@
         <v>dim1_1_3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>811</v>
       </c>
@@ -4478,7 +4487,7 @@
         <v>dim1_2_1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>810</v>
       </c>
@@ -4509,7 +4518,7 @@
         <v>dim1_2_2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>809</v>
       </c>
@@ -4540,7 +4549,7 @@
         <v>dim1_2_3</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>808</v>
       </c>
@@ -4571,7 +4580,7 @@
         <v>dim1_3_1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>807</v>
       </c>
@@ -4602,7 +4611,7 @@
         <v>dim1_3_2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>806</v>
       </c>
@@ -4633,7 +4642,7 @@
         <v>dim1_3_3</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>805</v>
       </c>
@@ -4664,7 +4673,7 @@
         <v>dim1_4_1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>804</v>
       </c>
@@ -4695,7 +4704,7 @@
         <v>dim1_4_2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>803</v>
       </c>
@@ -4726,7 +4735,7 @@
         <v>dim2_1_1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>802</v>
       </c>
@@ -4757,7 +4766,7 @@
         <v>dim2_1_2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>801</v>
       </c>
@@ -4788,7 +4797,7 @@
         <v>dim2_1_3</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>800</v>
       </c>
@@ -4819,7 +4828,7 @@
         <v>dim2_2_1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>799</v>
       </c>
@@ -4850,7 +4859,7 @@
         <v>dim2_2_2</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>798</v>
       </c>
@@ -4881,7 +4890,7 @@
         <v>dim2_2_3</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>797</v>
       </c>
@@ -4912,7 +4921,7 @@
         <v>dim2_3_1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>796</v>
       </c>
@@ -4943,7 +4952,7 @@
         <v>dim2_3_2</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>795</v>
       </c>
@@ -4974,7 +4983,7 @@
         <v>dim2_3_3</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>794</v>
       </c>
@@ -5005,7 +5014,7 @@
         <v>dim2_4_1</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>793</v>
       </c>
@@ -5036,7 +5045,7 @@
         <v>dim2_4_2</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>792</v>
       </c>
@@ -5067,7 +5076,7 @@
         <v>dim3_1_1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>791</v>
       </c>
@@ -5098,7 +5107,7 @@
         <v>dim3_1_2</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>790</v>
       </c>
@@ -5129,7 +5138,7 @@
         <v>dim3_1_3</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>789</v>
       </c>
@@ -5160,7 +5169,7 @@
         <v>dim3_2_1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>788</v>
       </c>
@@ -5191,7 +5200,7 @@
         <v>dim3_2_2</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>787</v>
       </c>
@@ -5222,7 +5231,7 @@
         <v>dim3_2_3</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>786</v>
       </c>
@@ -5253,7 +5262,7 @@
         <v>dim3_3_1</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>785</v>
       </c>
@@ -5284,7 +5293,7 @@
         <v>dim3_3_2</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>784</v>
       </c>
@@ -5315,7 +5324,7 @@
         <v>dim3_3_3</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>783</v>
       </c>
@@ -5346,7 +5355,7 @@
         <v>dim3_4_1</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>782</v>
       </c>
@@ -5377,7 +5386,7 @@
         <v>dim3_4_2</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>781</v>
       </c>
@@ -5408,7 +5417,7 @@
         <v>dim4_1_1</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>780</v>
       </c>
@@ -5439,7 +5448,7 @@
         <v>dim4_1_2</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>779</v>
       </c>
@@ -5470,7 +5479,7 @@
         <v>dim4_1_3</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>778</v>
       </c>
@@ -5501,7 +5510,7 @@
         <v>dim4_2_1</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>777</v>
       </c>
@@ -5532,7 +5541,7 @@
         <v>dim4_2_2</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>776</v>
       </c>
@@ -5563,7 +5572,7 @@
         <v>dim4_2_3</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>775</v>
       </c>
@@ -5594,7 +5603,7 @@
         <v>dim4_3_1</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>774</v>
       </c>
@@ -5625,7 +5634,7 @@
         <v>dim4_3_2</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>773</v>
       </c>
@@ -5656,7 +5665,7 @@
         <v>dim4_3_3</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>772</v>
       </c>
@@ -5687,7 +5696,7 @@
         <v>dim4_4_1</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>771</v>
       </c>
@@ -5718,7 +5727,7 @@
         <v>dim4_4_2</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>770</v>
       </c>
@@ -5749,7 +5758,7 @@
         <v>dim5_1_1</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>769</v>
       </c>
@@ -5780,7 +5789,7 @@
         <v>dim5_1_2</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>768</v>
       </c>
@@ -5811,7 +5820,7 @@
         <v>dim5_1_3</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>767</v>
       </c>
@@ -5842,7 +5851,7 @@
         <v>dim5_2_1</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>766</v>
       </c>
@@ -5873,7 +5882,7 @@
         <v>dim5_2_2</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>765</v>
       </c>
@@ -5904,7 +5913,7 @@
         <v>dim5_2_3</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>764</v>
       </c>
@@ -5935,7 +5944,7 @@
         <v>dim5_3_1</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>763</v>
       </c>
@@ -5966,7 +5975,7 @@
         <v>dim5_3_2</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>762</v>
       </c>
@@ -5997,7 +6006,7 @@
         <v>dim5_3_3</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>761</v>
       </c>
@@ -6028,7 +6037,7 @@
         <v>dim5_4_1</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>760</v>
       </c>
@@ -6068,31 +6077,30 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:U56"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="29.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="38.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="29.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="38.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="4.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="13" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="7" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="31.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6157,7 +6165,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>138</v>
       </c>
@@ -6193,7 +6201,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>141</v>
       </c>
@@ -6229,7 +6237,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>144</v>
       </c>
@@ -6265,7 +6273,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>147</v>
       </c>
@@ -6301,7 +6309,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>150</v>
       </c>
@@ -6337,7 +6345,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>153</v>
       </c>
@@ -6373,7 +6381,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>156</v>
       </c>
@@ -6409,7 +6417,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>159</v>
       </c>
@@ -6445,7 +6453,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>162</v>
       </c>
@@ -6481,7 +6489,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>663</v>
       </c>
@@ -6517,7 +6525,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>662</v>
       </c>
@@ -6553,7 +6561,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>164</v>
       </c>
@@ -6589,7 +6597,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>167</v>
       </c>
@@ -6625,7 +6633,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>170</v>
       </c>
@@ -6661,7 +6669,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>173</v>
       </c>
@@ -6697,7 +6705,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>176</v>
       </c>
@@ -6733,7 +6741,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>179</v>
       </c>
@@ -6769,7 +6777,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>182</v>
       </c>
@@ -6805,7 +6813,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>185</v>
       </c>
@@ -6841,7 +6849,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>188</v>
       </c>
@@ -6877,7 +6885,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>671</v>
       </c>
@@ -6913,7 +6921,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>670</v>
       </c>
@@ -6949,7 +6957,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>190</v>
       </c>
@@ -6985,7 +6993,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>193</v>
       </c>
@@ -7021,7 +7029,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>196</v>
       </c>
@@ -7057,7 +7065,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>199</v>
       </c>
@@ -7093,7 +7101,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>202</v>
       </c>
@@ -7129,7 +7137,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>205</v>
       </c>
@@ -7165,7 +7173,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>208</v>
       </c>
@@ -7201,7 +7209,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>211</v>
       </c>
@@ -7237,7 +7245,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>214</v>
       </c>
@@ -7273,7 +7281,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>669</v>
       </c>
@@ -7309,7 +7317,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>668</v>
       </c>
@@ -7345,7 +7353,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>216</v>
       </c>
@@ -7381,7 +7389,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>219</v>
       </c>
@@ -7417,7 +7425,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>222</v>
       </c>
@@ -7453,7 +7461,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>225</v>
       </c>
@@ -7489,7 +7497,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>228</v>
       </c>
@@ -7525,7 +7533,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>231</v>
       </c>
@@ -7561,7 +7569,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>234</v>
       </c>
@@ -7597,7 +7605,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>237</v>
       </c>
@@ -7633,7 +7641,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>240</v>
       </c>
@@ -7669,7 +7677,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>667</v>
       </c>
@@ -7705,7 +7713,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>666</v>
       </c>
@@ -7741,7 +7749,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>242</v>
       </c>
@@ -7777,7 +7785,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>245</v>
       </c>
@@ -7813,7 +7821,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>248</v>
       </c>
@@ -7849,7 +7857,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>251</v>
       </c>
@@ -7885,7 +7893,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>254</v>
       </c>
@@ -7921,7 +7929,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>257</v>
       </c>
@@ -7957,7 +7965,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>260</v>
       </c>
@@ -7993,7 +8001,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>263</v>
       </c>
@@ -8029,7 +8037,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>266</v>
       </c>
@@ -8065,7 +8073,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>665</v>
       </c>
@@ -8101,7 +8109,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>664</v>
       </c>
@@ -8145,58 +8153,58 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E0C7C33-6768-4AAE-A57E-F80585DED472}">
   <dimension ref="A1:AU75"/>
-  <sheetFormatPr defaultColWidth="5.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="5.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.44140625" customWidth="1"/>
-    <col min="3" max="3" width="36.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.42578125" customWidth="1"/>
+    <col min="3" max="3" width="36.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.6640625" style="19" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="35.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="29.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="37.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="62.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="41.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="37.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="62.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="41.7109375" style="6" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="45" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="30.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="56.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="30.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="56.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="35" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="38.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="36.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="23.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="28.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="34.44140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="38.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="38.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="36.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="23.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="28.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="34.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="38.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="12" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="34.6640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="35.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="66.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="66.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="59.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="35.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="66.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="66.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="59.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="60" style="6" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="35.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="66.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="66.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="59.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="35.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="66.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="66.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="59.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="60" style="6" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="35.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="66.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="66.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="59.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="35.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="66.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="66.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="59.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="47" max="47" width="60" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>471</v>
       </c>
@@ -8339,7 +8347,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -8494,7 +8502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -8649,7 +8657,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -8804,7 +8812,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -8959,7 +8967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -9114,7 +9122,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -9269,7 +9277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -9424,7 +9432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -9579,7 +9587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -9734,7 +9742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -9889,7 +9897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -10044,7 +10052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -10199,7 +10207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -10354,7 +10362,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -10509,7 +10517,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -10664,7 +10672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -10819,7 +10827,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -10974,7 +10982,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -11129,7 +11137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -11284,7 +11292,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -11439,7 +11447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -11594,7 +11602,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -11749,7 +11757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -11904,7 +11912,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -12059,7 +12067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -12214,7 +12222,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -12369,7 +12377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -12524,7 +12532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -12679,7 +12687,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -12834,7 +12842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -12989,7 +12997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -13144,7 +13152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -13299,7 +13307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -13466,7 +13474,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -13624,7 +13632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -13782,7 +13790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -13940,7 +13948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -14098,7 +14106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -14256,7 +14264,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -14414,7 +14422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -14572,7 +14580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -14730,7 +14738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -14888,7 +14896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -15043,7 +15051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -15198,7 +15206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -15356,7 +15364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -15514,7 +15522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -15672,7 +15680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -15830,7 +15838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -15988,7 +15996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -16146,7 +16154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -16304,7 +16312,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -16462,7 +16470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -16629,7 +16637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -16796,7 +16804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -16963,7 +16971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -17124,7 +17132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -17285,7 +17293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -17446,7 +17454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -17604,7 +17612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -17762,7 +17770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -17920,7 +17928,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -18078,7 +18086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -18239,7 +18247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -18400,7 +18408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -18561,7 +18569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -18722,7 +18730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -18883,7 +18891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -19044,7 +19052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -19205,7 +19213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -19366,7 +19374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -19524,7 +19532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -19682,7 +19690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -19840,7 +19848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -20013,13 +20021,13 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:C56"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="21.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -20030,7 +20038,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>62</v>
       </c>
@@ -20041,7 +20049,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>140</v>
       </c>
@@ -20052,7 +20060,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>143</v>
       </c>
@@ -20063,7 +20071,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>146</v>
       </c>
@@ -20074,7 +20082,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>149</v>
       </c>
@@ -20085,7 +20093,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>152</v>
       </c>
@@ -20096,7 +20104,7 @@
         <v>854</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>155</v>
       </c>
@@ -20107,7 +20115,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>158</v>
       </c>
@@ -20118,7 +20126,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>161</v>
       </c>
@@ -20129,7 +20137,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>680</v>
       </c>
@@ -20140,7 +20148,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>681</v>
       </c>
@@ -20151,7 +20159,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>64</v>
       </c>
@@ -20162,7 +20170,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>166</v>
       </c>
@@ -20173,7 +20181,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>169</v>
       </c>
@@ -20184,7 +20192,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>172</v>
       </c>
@@ -20195,7 +20203,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>175</v>
       </c>
@@ -20206,7 +20214,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>178</v>
       </c>
@@ -20217,7 +20225,7 @@
         <v>865</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>181</v>
       </c>
@@ -20228,7 +20236,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>184</v>
       </c>
@@ -20239,7 +20247,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>187</v>
       </c>
@@ -20250,7 +20258,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>678</v>
       </c>
@@ -20261,7 +20269,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>679</v>
       </c>
@@ -20272,7 +20280,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>66</v>
       </c>
@@ -20283,7 +20291,7 @@
         <v>871</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>192</v>
       </c>
@@ -20294,7 +20302,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>195</v>
       </c>
@@ -20305,7 +20313,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>198</v>
       </c>
@@ -20316,7 +20324,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>201</v>
       </c>
@@ -20327,7 +20335,7 @@
         <v>875</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>204</v>
       </c>
@@ -20338,7 +20346,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>207</v>
       </c>
@@ -20349,7 +20357,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>210</v>
       </c>
@@ -20360,7 +20368,7 @@
         <v>878</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>213</v>
       </c>
@@ -20371,7 +20379,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>677</v>
       </c>
@@ -20382,7 +20390,7 @@
         <v>880</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>676</v>
       </c>
@@ -20393,7 +20401,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>68</v>
       </c>
@@ -20404,7 +20412,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>218</v>
       </c>
@@ -20415,7 +20423,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>221</v>
       </c>
@@ -20426,7 +20434,7 @@
         <v>884</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>224</v>
       </c>
@@ -20437,7 +20445,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>227</v>
       </c>
@@ -20448,7 +20456,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>230</v>
       </c>
@@ -20459,7 +20467,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>233</v>
       </c>
@@ -20470,7 +20478,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>236</v>
       </c>
@@ -20481,7 +20489,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>239</v>
       </c>
@@ -20492,7 +20500,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>675</v>
       </c>
@@ -20503,7 +20511,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>674</v>
       </c>
@@ -20514,7 +20522,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>70</v>
       </c>
@@ -20525,7 +20533,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>244</v>
       </c>
@@ -20536,7 +20544,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>247</v>
       </c>
@@ -20547,7 +20555,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>250</v>
       </c>
@@ -20558,7 +20566,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>253</v>
       </c>
@@ -20569,7 +20577,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>256</v>
       </c>
@@ -20580,7 +20588,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>259</v>
       </c>
@@ -20591,7 +20599,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>262</v>
       </c>
@@ -20602,7 +20610,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>265</v>
       </c>
@@ -20613,7 +20621,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>673</v>
       </c>
@@ -20624,7 +20632,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>672</v>
       </c>
@@ -20644,18 +20652,18 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H56"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.6640625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" style="6"/>
+    <col min="5" max="5" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.7109375" style="6" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -20681,7 +20689,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>137</v>
       </c>
@@ -20704,7 +20712,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0195d18c-1caa-1722-0366-f73bd3f09ee8</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>139</v>
       </c>
@@ -20727,7 +20735,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0195d18c-1cab-86f3-5faf-507bfa221cf6</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>142</v>
       </c>
@@ -20750,7 +20758,7 @@
         <v>0195d18c-1cc2-37d1-f6c3-0e7c8d6b1f07|0195d18c-1cab-b4e5-a81b-6acdcc710af2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>145</v>
       </c>
@@ -20773,7 +20781,7 @@
         <v>0195d18c-1cc2-7cf5-8b5c-03f41714d8b8|0195d18c-1cab-3208-7ccc-820a8c522208</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>148</v>
       </c>
@@ -20796,7 +20804,7 @@
         <v>0195d18c-1cc2-50aa-7113-6b261eaeec7a|0195d18c-1cab-767e-81b1-986e918827fb</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>151</v>
       </c>
@@ -20819,7 +20827,7 @@
         <v>0195d18c-1cc3-0cbc-2362-c1cfe3fdec5a|0195d18c-1cab-22f7-dda1-cc74cee303ca</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>154</v>
       </c>
@@ -20842,7 +20850,7 @@
         <v>0195d18c-1cc3-e9c0-5858-8bf9d9d8c36f|0195d18c-1cac-4ed2-2296-a46fa423ce99</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>157</v>
       </c>
@@ -20865,7 +20873,7 @@
         <v>0195d18c-1cc4-9f18-3767-29d288f47190|0195d18c-1cac-9221-a9c7-72e70e09dea9</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>160</v>
       </c>
@@ -20888,7 +20896,7 @@
         <v>0195d18c-1cc5-2ea3-8102-7b410f3146c8|0195d18c-1cac-4d0a-db2e-5a54065df180</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>682</v>
       </c>
@@ -20911,7 +20919,7 @@
         <v>019a8753-bed9-afc6-e887-8b50ddfd6962|019a8753-bed9-180c-d818-10c8aed7f4c5</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>683</v>
       </c>
@@ -20934,7 +20942,7 @@
         <v>019a8753-bed9-869e-506b-15ae88b8c755|019a8753-bed9-8a7b-7c82-adf57928fa72</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>163</v>
       </c>
@@ -20957,7 +20965,7 @@
         <v>0195d18c-1cc6-a324-3f72-222014292515|0195d18c-1cad-37c6-0826-9671f313fb2b</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>165</v>
       </c>
@@ -20980,7 +20988,7 @@
         <v>0195d18c-1cc7-243f-f4e7-3dbdfe691c71|0195d18c-1cad-5b48-8a72-25050cbf379e</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>168</v>
       </c>
@@ -21003,7 +21011,7 @@
         <v>0195d18c-1cc7-60b4-b4e6-8ff7fabb2b09|0195d18c-1cad-e18e-a87d-8af6760d00e1</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>171</v>
       </c>
@@ -21026,7 +21034,7 @@
         <v>0195d18c-1cc8-bcf2-c56f-04928f2e3635|0195d18c-1cad-9467-449f-6341c820b944</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>174</v>
       </c>
@@ -21049,7 +21057,7 @@
         <v>0195d18c-1cc8-18f5-27a5-fd3874e6b78b|0195d18c-1cae-fcea-56fe-4577ada0491d</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>177</v>
       </c>
@@ -21072,7 +21080,7 @@
         <v>0195d18c-1cc8-5a76-0a72-16117b0a5a5e|0195d18c-1cae-cdba-00d9-e8405172259e</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>180</v>
       </c>
@@ -21095,7 +21103,7 @@
         <v>0195d18c-1cc9-7181-fd5b-078012e228f2|0195d18c-1cae-faa7-ac0d-22cce7d230ec</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>183</v>
       </c>
@@ -21118,7 +21126,7 @@
         <v>0195d18c-1cc9-c61f-4e7e-a00189d3cc75|0195d18c-1cae-45ab-ca21-9cee527b9482</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>186</v>
       </c>
@@ -21141,7 +21149,7 @@
         <v>0195d18c-1cca-878e-2110-0116e848541b|0195d18c-1caf-d364-c3b5-e73ba434270e</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>684</v>
       </c>
@@ -21164,7 +21172,7 @@
         <v>019a8753-bed9-8f84-5827-8c0fedea4c3d|019a8753-bed9-10ef-cde6-dd672b6f1342</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>685</v>
       </c>
@@ -21187,7 +21195,7 @@
         <v>019a8753-bed9-2ec3-f155-116a4b0fe44d|019a8753-bed9-423c-9007-26ece8e894c8</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>189</v>
       </c>
@@ -21210,7 +21218,7 @@
         <v>0195d18c-1cca-26c0-66df-979380a43b16|0195d18c-1caf-b3af-f64e-bd18810c4521</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>191</v>
       </c>
@@ -21233,7 +21241,7 @@
         <v>0195d18c-1ccb-f06f-162f-a5dc745a5198|0195d18c-1caf-84ca-1737-a8f8788cd464</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>194</v>
       </c>
@@ -21256,7 +21264,7 @@
         <v>0195d18c-1ccb-b068-d845-d61fb54721f1|0195d18c-1cb0-7655-a8bb-f656b1b8b72c</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>197</v>
       </c>
@@ -21279,7 +21287,7 @@
         <v>0195d18c-1ccc-f754-4a4f-89cdc532a3be|0195d18c-1cb0-4c24-e2e8-b92cfc74f7cc</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>200</v>
       </c>
@@ -21302,7 +21310,7 @@
         <v>0195d18c-1ccc-3f10-cc4e-636793b1e9dd|0195d18c-1cb0-8d34-e3f0-ab091b80ab8f</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>203</v>
       </c>
@@ -21325,7 +21333,7 @@
         <v>0195d18c-1ccd-3f53-ad72-f2d3c667b246|0195d18c-1cb0-db51-ed28-2a4481c5f1ac</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>206</v>
       </c>
@@ -21348,7 +21356,7 @@
         <v>0195d18c-1ccd-d664-179c-a1a90c3c886c|0195d18c-1cb1-b5d5-ee26-96c6a9678489</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>209</v>
       </c>
@@ -21371,7 +21379,7 @@
         <v>0195d18c-1ccd-12ae-b807-5b71d1b4e1f1|0195d18c-1cb1-f7bb-aa5b-6f2c6f5d3696</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>212</v>
       </c>
@@ -21394,7 +21402,7 @@
         <v>0195d18c-1cce-3516-017e-cf05c78d4433|0195d18c-1cb1-2097-fae7-ffcb7e109be5</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>686</v>
       </c>
@@ -21417,7 +21425,7 @@
         <v>019a8753-bed9-c7d8-6072-9a0d42887e0f|019a8753-bed9-0ab7-4323-aa6aedd4c1cc</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>687</v>
       </c>
@@ -21440,7 +21448,7 @@
         <v>019a8753-bed9-9918-33cd-c862ad905516|019a8753-bed9-af63-b674-d9ae3c5f0a08</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>215</v>
       </c>
@@ -21463,7 +21471,7 @@
         <v>0195d18c-1cce-585d-e95b-79f3fbfdd12b|0195d18c-1cb2-95e6-139d-1dbe7ffdd3d0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>217</v>
       </c>
@@ -21486,7 +21494,7 @@
         <v>0195d18c-1ccf-c9fa-4e69-800cfa6c5e86|0195d18c-1cb2-995c-625d-dfa62a674ff8</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>220</v>
       </c>
@@ -21509,7 +21517,7 @@
         <v>0195d18c-1ccf-d319-afba-0f13f0d06256|0195d18c-1cb2-7a1f-c2f8-ce2096e4cbbc</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>223</v>
       </c>
@@ -21532,7 +21540,7 @@
         <v>0195d18c-1cd0-951a-878d-5fe5fcd0015a|0195d18c-1cb3-b49c-ddc2-f5174414bfdc</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>226</v>
       </c>
@@ -21555,7 +21563,7 @@
         <v>0195d18c-1cd0-0128-08ed-42804fabb534|0195d18c-1cb3-9495-0b74-a14fa0378944</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>229</v>
       </c>
@@ -21578,7 +21586,7 @@
         <v>0195d18c-1cd1-9702-2218-87932d7bfde7|0195d18c-1cb3-7165-f2c8-1549624bce57</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>232</v>
       </c>
@@ -21601,7 +21609,7 @@
         <v>0195d18c-1cd1-a4b4-2764-66bf69a9f28c|0195d18c-1cb4-62ef-acc3-d4754efbcff5</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>235</v>
       </c>
@@ -21624,7 +21632,7 @@
         <v>0195d18c-1cd2-3359-f0c5-d09dfe10cbd9|0195d18c-1cb4-4080-ce72-0ae401b350e2</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>238</v>
       </c>
@@ -21647,7 +21655,7 @@
         <v>0195d18c-1cd2-c028-2759-dfa197e2e6c0|0195d18c-1cb4-7eca-c0f5-e64333747c9b</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>689</v>
       </c>
@@ -21670,7 +21678,7 @@
         <v>019a8753-bed9-eba4-fbce-8c553ccd262a|019a8753-bed9-9436-d94c-4e4ee8856951</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>688</v>
       </c>
@@ -21693,7 +21701,7 @@
         <v>019a8753-bed9-47cd-cf12-b0da18fd2588|019a8753-bed9-9857-f307-13b9f5a150d1</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>241</v>
       </c>
@@ -21716,7 +21724,7 @@
         <v>0195d18c-1cd3-02c7-4a0d-80f544cc425a|0195d18c-1cb5-c3e7-b945-7d438ce70962</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>243</v>
       </c>
@@ -21739,7 +21747,7 @@
         <v>0195d18c-1cd3-acd1-2f6c-f9db7a3cd290|0195d18c-1cb5-8fdb-b13a-19f20c06817d</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>246</v>
       </c>
@@ -21762,7 +21770,7 @@
         <v>0195d18c-1cd4-44f9-ea4c-4ab401e03f8f|0195d18c-1cb5-5dbb-4903-872ca139254e</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>249</v>
       </c>
@@ -21785,7 +21793,7 @@
         <v>0195d18c-1cd4-a35d-3e85-41eb9f24a911|0195d18c-1cb6-9ffa-e835-0b70cc4b0ae9</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>252</v>
       </c>
@@ -21808,7 +21816,7 @@
         <v>0195d18c-1cd5-e8f4-76f8-56e13a8aec12|0195d18c-1cb6-a2b9-4827-77425c5ab615</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>255</v>
       </c>
@@ -21831,7 +21839,7 @@
         <v>0195d18c-1cd6-da43-ec75-25feee641928|0195d18c-1cb6-04b0-5474-a6411b693a97</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>258</v>
       </c>
@@ -21854,7 +21862,7 @@
         <v>0195d18c-1cd6-2f81-aefd-93fce854296f|0195d18c-1cb7-05e5-fd6b-6914a124e649</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>261</v>
       </c>
@@ -21877,7 +21885,7 @@
         <v>0195d18c-1cd7-22bb-71ce-9110669bbfef|0195d18c-1cb7-44c6-2f56-594e12327604</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>264</v>
       </c>
@@ -21900,7 +21908,7 @@
         <v>0195d18c-1cd7-b95b-ced6-589a63e3e6eb|0195d18c-1cb7-e7f7-a41d-bacd0f861a06</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>691</v>
       </c>
@@ -21923,7 +21931,7 @@
         <v>019a8753-bed9-8d4b-cfe4-957f28881a67|019a8753-bed9-e6df-c1d5-00f9f7cf16f3</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>690</v>
       </c>
@@ -21954,17 +21962,17 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -21984,7 +21992,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -22006,7 +22014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -22028,7 +22036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>48</v>
       </c>
@@ -22050,7 +22058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -22072,7 +22080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -22102,32 +22110,32 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6F0F389-1562-4A7F-BB5E-AAA96B2F3DDB}">
   <dimension ref="A1:V11"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="35.6640625" customWidth="1"/>
-    <col min="13" max="13" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="35.7109375" customWidth="1"/>
+    <col min="13" max="13" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="36" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.44140625" customWidth="1"/>
+    <col min="19" max="19" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -22195,7 +22203,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>60</v>
       </c>
@@ -22271,7 +22279,7 @@
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653|0195d18c-1ca2-a23d-1f64-00271f63199c</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -22347,7 +22355,7 @@
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3|0195d18c-1ca2-2a29-96a5-37c6bf87f586</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>72</v>
       </c>
@@ -22423,7 +22431,7 @@
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037|0195d18c-1ca2-3a4f-1878-fbe3282c9c76</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>73</v>
       </c>
@@ -22499,7 +22507,7 @@
         <v>0195d18c-1c92-d419-4c71-a570f428499b|0195d18c-1ca2-e55a-608d-a42fc6f948e1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>74</v>
       </c>
@@ -22575,7 +22583,7 @@
         <v>0195d18c-1c93-02a2-6920-7e4dbfb73ce0|0195d18c-1ca2-b728-a2a1-d2a4cf7b8eb8</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>75</v>
       </c>
@@ -22648,7 +22656,7 @@
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653|0195d18c-1ca3-f309-f6f1-e4807afe3802</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>76</v>
       </c>
@@ -22721,7 +22729,7 @@
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3|0195d18c-1ca3-db40-a2a8-6dc905d6c1e9</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -22794,7 +22802,7 @@
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037|0195d18c-1ca3-da0a-44bb-877b3a1eb73e</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>78</v>
       </c>
@@ -22867,7 +22875,7 @@
         <v>0195d18c-1c92-d419-4c71-a570f428499b|0195d18c-1ca3-4d34-d0e9-8f024ad8651a</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>79</v>
       </c>
@@ -22949,14 +22957,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -22967,7 +22975,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -22979,7 +22987,7 @@
         <v>dc1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -22991,7 +22999,7 @@
         <v>dc2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -23003,7 +23011,7 @@
         <v>dc3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -23015,7 +23023,7 @@
         <v>dc4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -23027,7 +23035,7 @@
         <v>dc5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -23039,7 +23047,7 @@
         <v>dc6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -23051,7 +23059,7 @@
         <v>dc7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -23063,7 +23071,7 @@
         <v>dc8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -23075,7 +23083,7 @@
         <v>dc9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -23087,7 +23095,7 @@
         <v>dc10</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -23108,32 +23116,32 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{413B6EDF-4214-4325-A1BD-732A42D052EA}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:W11"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="35.6640625" customWidth="1"/>
-    <col min="12" max="12" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="25.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="42.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="35.7109375" customWidth="1"/>
+    <col min="12" max="12" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="42.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="36" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -23204,7 +23212,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>60</v>
       </c>
@@ -23285,7 +23293,7 @@
         <v>0195d18c-1c98-7e0b-0c91-8cafbdb2c852|0195d18c-1ca2-a23d-1f64-00271f63199c</v>
       </c>
     </row>
-    <row r="3" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -23366,7 +23374,7 @@
         <v>0195d18c-1c9a-1178-0519-9124131763a6|0195d18c-1ca2-2a29-96a5-37c6bf87f586</v>
       </c>
     </row>
-    <row r="4" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>72</v>
       </c>
@@ -23447,7 +23455,7 @@
         <v>0195d18c-1c9c-0d8f-435a-5ca8b45939b8|0195d18c-1ca2-3a4f-1878-fbe3282c9c76</v>
       </c>
     </row>
-    <row r="5" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>73</v>
       </c>
@@ -23528,7 +23536,7 @@
         <v>0195d18c-1c9e-1c4a-1311-4f22f0d59f61|0195d18c-1ca2-e55a-608d-a42fc6f948e1</v>
       </c>
     </row>
-    <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>74</v>
       </c>
@@ -23609,7 +23617,7 @@
         <v>0195d18c-1ca0-e0db-7a87-6237ad6380c8|0195d18c-1ca2-b728-a2a1-d2a4cf7b8eb8</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>75</v>
       </c>
@@ -23690,7 +23698,7 @@
         <v>0195d18c-1c98-7e0b-0c91-8cafbdb2c852|0195d18c-1ca3-f309-f6f1-e4807afe3802</v>
       </c>
     </row>
-    <row r="8" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>76</v>
       </c>
@@ -23771,7 +23779,7 @@
         <v>0195d18c-1c9a-1178-0519-9124131763a6|0195d18c-1ca3-db40-a2a8-6dc905d6c1e9</v>
       </c>
     </row>
-    <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -23852,7 +23860,7 @@
         <v>0195d18c-1c9c-0d8f-435a-5ca8b45939b8|0195d18c-1ca3-da0a-44bb-877b3a1eb73e</v>
       </c>
     </row>
-    <row r="10" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>78</v>
       </c>
@@ -23933,7 +23941,7 @@
         <v>0195d18c-1c9e-1c4a-1311-4f22f0d59f61|0195d18c-1ca3-4d34-d0e9-8f024ad8651a</v>
       </c>
     </row>
-    <row r="11" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>79</v>
       </c>
@@ -24029,26 +24037,26 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46B1A0CE-352C-4E69-8986-540397C3CD9D}">
   <dimension ref="A1:P2"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="35.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="27.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="36" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="35.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -24098,7 +24106,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>453</v>
       </c>
@@ -24166,25 +24174,25 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21E03A8B-A0A1-46B6-957F-B8B3E001E975}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="27.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="36" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -24228,7 +24236,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>453</v>
       </c>
@@ -24288,22 +24296,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:M29"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.33203125" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.28515625" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="36" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="14.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -24344,7 +24352,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>586</v>
       </c>
@@ -24392,7 +24400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>337</v>
       </c>
@@ -24440,7 +24448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>339</v>
       </c>
@@ -24488,7 +24496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -24536,7 +24544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>47</v>
       </c>
@@ -24584,7 +24592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>50</v>
       </c>
@@ -24632,7 +24640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>53</v>
       </c>
@@ -24680,7 +24688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>56</v>
       </c>
@@ -24728,7 +24736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -24776,7 +24784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -24824,7 +24832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -24872,7 +24880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -24920,7 +24928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -24968,7 +24976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -25016,7 +25024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -25064,7 +25072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -25112,7 +25120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -25160,7 +25168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -25208,7 +25216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -25256,7 +25264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -25304,7 +25312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -25352,7 +25360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -25400,7 +25408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>31</v>
       </c>
@@ -25448,7 +25456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -25496,7 +25504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>34</v>
       </c>
@@ -25544,7 +25552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -25592,7 +25600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -25640,7 +25648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -25700,21 +25708,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:K28"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="27" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" style="6" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="36" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -25749,7 +25757,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>385</v>
       </c>
@@ -25787,7 +25795,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>387</v>
       </c>
@@ -25825,7 +25833,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>389</v>
       </c>
@@ -25863,7 +25871,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>391</v>
       </c>
@@ -25901,7 +25909,7 @@
         <v>org2</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>393</v>
       </c>
@@ -25939,7 +25947,7 @@
         <v>org3</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>395</v>
       </c>
@@ -25977,7 +25985,7 @@
         <v>org4</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>397</v>
       </c>
@@ -26015,7 +26023,7 @@
         <v>org5</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>399</v>
       </c>
@@ -26053,7 +26061,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>401</v>
       </c>
@@ -26091,7 +26099,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>403</v>
       </c>
@@ -26129,7 +26137,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>405</v>
       </c>
@@ -26167,7 +26175,7 @@
         <v>org1</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>407</v>
       </c>
@@ -26205,7 +26213,7 @@
         <v>org2</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>409</v>
       </c>
@@ -26243,7 +26251,7 @@
         <v>org2</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>411</v>
       </c>
@@ -26281,7 +26289,7 @@
         <v>org2</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>413</v>
       </c>
@@ -26319,7 +26327,7 @@
         <v>org2</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>415</v>
       </c>
@@ -26357,7 +26365,7 @@
         <v>org3</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>417</v>
       </c>
@@ -26395,7 +26403,7 @@
         <v>org3</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>419</v>
       </c>
@@ -26433,7 +26441,7 @@
         <v>org3</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>421</v>
       </c>
@@ -26471,7 +26479,7 @@
         <v>org3</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>423</v>
       </c>
@@ -26509,7 +26517,7 @@
         <v>org4</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>425</v>
       </c>
@@ -26547,7 +26555,7 @@
         <v>org4</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>427</v>
       </c>
@@ -26585,7 +26593,7 @@
         <v>org4</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>429</v>
       </c>
@@ -26623,7 +26631,7 @@
         <v>org4</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>431</v>
       </c>
@@ -26661,7 +26669,7 @@
         <v>org5</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>433</v>
       </c>
@@ -26699,7 +26707,7 @@
         <v>org5</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>435</v>
       </c>
@@ -26737,7 +26745,7 @@
         <v>org5</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>437</v>
       </c>
@@ -26787,18 +26795,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -26824,7 +26832,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>326</v>
       </c>
@@ -26852,7 +26860,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>327</v>
       </c>
@@ -26880,7 +26888,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>328</v>
       </c>
@@ -26908,7 +26916,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>655</v>
       </c>
@@ -26943,28 +26951,28 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:P12"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:S12"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.6640625" style="13" customWidth="1"/>
-    <col min="16" max="16" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="26.28515625" style="13" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -27013,8 +27021,17 @@
       <c r="P1" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q1" t="s">
+        <v>908</v>
+      </c>
+      <c r="R1" t="s">
+        <v>909</v>
+      </c>
+      <c r="S1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>281</v>
       </c>
@@ -27041,7 +27058,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>283</v>
       </c>
@@ -27068,7 +27085,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>284</v>
       </c>
@@ -27095,7 +27112,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>285</v>
       </c>
@@ -27122,7 +27139,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>286</v>
       </c>
@@ -27149,7 +27166,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>287</v>
       </c>
@@ -27176,7 +27193,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>288</v>
       </c>
@@ -27203,7 +27220,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>289</v>
       </c>
@@ -27230,7 +27247,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>290</v>
       </c>
@@ -27257,7 +27274,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>654</v>
       </c>
@@ -27284,7 +27301,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>653</v>
       </c>
@@ -27319,12 +27336,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BFE9DBA-4D09-4E45-A394-72AC78245E1D}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -27335,7 +27352,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>119</v>
       </c>
@@ -27343,7 +27360,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>123</v>
       </c>
@@ -27351,7 +27368,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>127</v>
       </c>
@@ -27359,7 +27376,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>131</v>
       </c>
@@ -27367,7 +27384,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>135</v>
       </c>
@@ -27384,14 +27401,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFBF5204-3F7C-438F-A194-7543BC84CF2A}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -27402,7 +27419,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>120</v>
       </c>
@@ -27413,7 +27430,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>124</v>
       </c>
@@ -27424,7 +27441,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>128</v>
       </c>
@@ -27435,7 +27452,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>132</v>
       </c>
@@ -27446,7 +27463,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>136</v>
       </c>
@@ -27466,19 +27483,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.6640625" style="13" customWidth="1"/>
+    <col min="4" max="4" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.7109375" style="13" customWidth="1"/>
     <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="35.33203125" style="13" customWidth="1"/>
+    <col min="7" max="7" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.28515625" style="13" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -27507,7 +27524,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>117</v>
       </c>
@@ -27529,7 +27546,7 @@
         <v>etiological_agent1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>121</v>
       </c>
@@ -27551,7 +27568,7 @@
         <v>etiological_agent2</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>125</v>
       </c>
@@ -27573,7 +27590,7 @@
         <v>etiological_agent3</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>129</v>
       </c>
@@ -27595,7 +27612,7 @@
         <v>etiological_agent4</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>133</v>
       </c>

</xml_diff>